<commit_message>
Swap Sheet status/Export with the permitted-printers field (0.9.19)
User request: Sheet status and Export move to the side panel; the
permitted-printers list moves the other way onto the main block,
reformatted for people rather than code - "N printers (comma,
separated, list)" with correct singular/plural.

LOC_Printers itself is untouched functionally - still the exact
semicolon-delimited string the Select printers... picker writes and
modCatalog's compatibility checks read, just relocated to the side
panel under its own label. The friendly display is a separate,
read-only LET formula (modInit.EnsurePrintersDisplay) deriving from
it, never written to directly.

modExport.EXPORT_CELL moves from $B$8 to $AM$6 - a one-line change,
since RefreshExportStatus already writes its own label via an
Offset(0, -1) rather than a second hardcoded address. The live job
count moves up to A8/B8, the row Export vacated.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c54d1abecbe6fecc/Development/OfficeApps/PrintJob/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="6_{24FC9915-6BA6-43A0-B0CA-D3ADEEE53F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F69C9187-3FD8-472A-9B34-944521AD99AC}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="6_{24FC9915-6BA6-43A0-B0CA-D3ADEEE53F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C302A1D-FF0C-4FFC-8E72-FDFF9E18DB88}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,10 +36,10 @@
     <definedName name="LOC_Dept" localSheetId="9">'Main Print Room'!$B$2</definedName>
     <definedName name="LOC_Name" localSheetId="10">Annexe!$B$1</definedName>
     <definedName name="LOC_Name" localSheetId="9">'Main Print Room'!$B$1</definedName>
-    <definedName name="LOC_Printers" localSheetId="10">Annexe!$AM$5</definedName>
-    <definedName name="LOC_Printers" localSheetId="9">'Main Print Room'!$AM$5</definedName>
-    <definedName name="LOC_Status" localSheetId="10">Annexe!$B$7</definedName>
-    <definedName name="LOC_Status" localSheetId="9">'Main Print Room'!$B$7</definedName>
+    <definedName name="LOC_Printers" localSheetId="10">Annexe!$AM$7</definedName>
+    <definedName name="LOC_Printers" localSheetId="9">'Main Print Room'!$AM$7</definedName>
+    <definedName name="LOC_Status" localSheetId="10">Annexe!$AM$5</definedName>
+    <definedName name="LOC_Status" localSheetId="9">'Main Print Room'!$AM$5</definedName>
     <definedName name="lstConsumables">tblConsumables[Consumable type]</definedName>
     <definedName name="lstFamilies">tblPaperFamilies[Family]</definedName>
     <definedName name="lstPaperTypes">tblPaperTypes[Paper type]</definedName>
@@ -540,9 +540,6 @@
     <t>Default: disregard consumable cost</t>
   </si>
   <si>
-    <t>Printers at this location</t>
-  </si>
-  <si>
     <t>Epson SureColor P9500;HP DesignJet Z9+;Xerox Versant 180</t>
   </si>
   <si>
@@ -742,6 +739,9 @@
   </si>
   <si>
     <t>Printers are chosen with the Select printers... button (side panel below); only printers listed here can be used for jobs on this sheet.</t>
+  </si>
+  <si>
+    <t>Permitted printers (raw list)</t>
   </si>
 </sst>
 </file>
@@ -3091,13 +3091,13 @@
         <v>148</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AL1" s="19" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AZ1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:52" x14ac:dyDescent="0.35">
@@ -3108,7 +3108,7 @@
         <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AL2" s="19" t="s">
         <v>149</v>
@@ -3142,149 +3142,154 @@
       <c r="A5" s="21"/>
       <c r="B5" s="7"/>
       <c r="AL5" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="AM5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A6" s="21"/>
       <c r="B6" s="5"/>
-      <c r="AL6" s="20" t="s">
+      <c r="AL6" s="20"/>
+    </row>
+    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A7" s="21"/>
+      <c r="B7" s="5"/>
+      <c r="AL7" s="19" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>157</v>
+      <c r="AM7" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="8" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="AL8" s="20" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="I10" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="K10" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="M10" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:52" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="H12" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="I12" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="J12" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="K12" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="L12" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="L12" s="4" t="s">
+      <c r="M12" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="N12" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="O12" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="O12" s="4" t="s">
+      <c r="P12" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="P12" s="4" t="s">
+      <c r="Q12" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="Q12" s="4" t="s">
+      <c r="R12" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="R12" s="4" t="s">
+      <c r="S12" s="4" t="s">
         <v>185</v>
-      </c>
-      <c r="S12" s="4" t="s">
-        <v>186</v>
       </c>
       <c r="T12" s="4" t="s">
         <v>6</v>
       </c>
       <c r="U12" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="V12" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="V12" s="4" t="s">
+      <c r="W12" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="W12" s="4" t="s">
+      <c r="X12" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="X12" s="4" t="s">
+      <c r="Y12" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="Y12" s="4" t="s">
+      <c r="Z12" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="Z12" s="4" t="s">
+      <c r="AA12" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="AA12" s="4" t="s">
+      <c r="AB12" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="AB12" s="4" t="s">
+      <c r="AC12" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="AC12" s="4" t="s">
+      <c r="AD12" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="AD12" s="4" t="s">
+      <c r="AE12" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="AE12" s="4" t="s">
+      <c r="AF12" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="AF12" s="4" t="s">
+      <c r="AG12" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="AG12" s="4" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:52" x14ac:dyDescent="0.35">
@@ -3293,16 +3298,16 @@
         <v>OK</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C13" s="12">
         <v>46280.425000000003</v>
       </c>
       <c r="D13" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="E13" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>83</v>
@@ -3352,7 +3357,7 @@
         <v>44.68</v>
       </c>
       <c r="T13" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="U13" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3389,7 +3394,7 @@
         <v>46282.375</v>
       </c>
       <c r="AF13" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AG13" s="17" t="s">
         <v>35</v>
@@ -3401,16 +3406,16 @@
         <v>OK</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C14" s="12">
         <v>46280.611111111109</v>
       </c>
       <c r="D14" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="E14" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="F14" s="13" t="s">
         <v>85</v>
@@ -3460,7 +3465,7 @@
         <v>136.26</v>
       </c>
       <c r="T14" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="U14" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3495,7 +3500,7 @@
         <v>46282.375</v>
       </c>
       <c r="AF14" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AG14" s="17" t="s">
         <v>35</v>
@@ -3507,16 +3512,16 @@
         <v>OK</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C15" s="12">
         <v>46281.461805555547</v>
       </c>
       <c r="D15" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="E15" s="13" t="s">
         <v>208</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>209</v>
       </c>
       <c r="F15" s="13" t="s">
         <v>85</v>
@@ -3568,7 +3573,7 @@
         <v>125.52</v>
       </c>
       <c r="T15" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="U15" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3603,7 +3608,7 @@
         <v>46282.375</v>
       </c>
       <c r="AF15" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AG15" s="17" t="s">
         <v>35</v>
@@ -3615,16 +3620,16 @@
         <v>OK</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C16" s="12">
         <v>46281.638888888891</v>
       </c>
       <c r="D16" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="E16" s="13" t="s">
         <v>208</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>209</v>
       </c>
       <c r="F16" s="13" t="s">
         <v>83</v>
@@ -3674,7 +3679,7 @@
         <v>8.69</v>
       </c>
       <c r="T16" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="U16" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3709,7 +3714,7 @@
         <v>46282.375</v>
       </c>
       <c r="AF16" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AG16" s="17" t="s">
         <v>35</v>
@@ -3721,7 +3726,7 @@
         <v>Student name or number required; Print width exceeds stock width</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C17" s="12">
         <v>46282.395833333343</v>
@@ -3778,7 +3783,7 @@
         <v>146.04</v>
       </c>
       <c r="T17" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="U17" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3813,7 +3818,7 @@
         <v>46282.375</v>
       </c>
       <c r="AF17" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AG17" s="17" t="s">
         <v>35</v>
@@ -3893,16 +3898,16 @@
         <v>147</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AL1" s="19" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AZ1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:52" x14ac:dyDescent="0.35">
@@ -3913,13 +3918,13 @@
         <v>88</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AL2" s="19" t="s">
         <v>149</v>
       </c>
       <c r="AM2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:52" x14ac:dyDescent="0.35">
@@ -3947,149 +3952,154 @@
       <c r="A5" s="21"/>
       <c r="B5" s="7"/>
       <c r="AL5" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="AM5" t="s">
-        <v>217</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A6" s="21"/>
       <c r="B6" s="5"/>
-      <c r="AL6" s="20" t="s">
+      <c r="AL6" s="20"/>
+    </row>
+    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A7" s="21"/>
+      <c r="B7" s="5"/>
+      <c r="AL7" s="19" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>157</v>
+      <c r="AM7" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="8" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="AL8" s="20" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="I10" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="K10" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="M10" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:52" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="H12" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="I12" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="J12" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="K12" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="L12" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="L12" s="4" t="s">
+      <c r="M12" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="N12" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="O12" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="O12" s="4" t="s">
+      <c r="P12" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="P12" s="4" t="s">
+      <c r="Q12" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="Q12" s="4" t="s">
+      <c r="R12" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="R12" s="4" t="s">
+      <c r="S12" s="4" t="s">
         <v>185</v>
-      </c>
-      <c r="S12" s="4" t="s">
-        <v>186</v>
       </c>
       <c r="T12" s="4" t="s">
         <v>6</v>
       </c>
       <c r="U12" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="V12" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="V12" s="4" t="s">
+      <c r="W12" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="W12" s="4" t="s">
+      <c r="X12" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="X12" s="4" t="s">
+      <c r="Y12" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="Y12" s="4" t="s">
+      <c r="Z12" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="Z12" s="4" t="s">
+      <c r="AA12" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="AA12" s="4" t="s">
+      <c r="AB12" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="AB12" s="4" t="s">
+      <c r="AC12" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="AC12" s="4" t="s">
+      <c r="AD12" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="AD12" s="4" t="s">
+      <c r="AE12" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="AE12" s="4" t="s">
+      <c r="AF12" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="AF12" s="4" t="s">
+      <c r="AG12" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="AG12" s="4" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:52" x14ac:dyDescent="0.35">
@@ -4098,16 +4108,16 @@
         <v>OK</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C13" s="12">
         <v>46281.40625</v>
       </c>
       <c r="D13" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="E13" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>202</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>87</v>
@@ -4157,7 +4167,7 @@
         <v>17.87</v>
       </c>
       <c r="T13" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="U13" s="17" t="str">
         <f>IF(tblJobs_ANNEX[[#This Row],[Job ID]]="","",IF(tblJobs_ANNEX[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_ANNEX[[#This Row],[Student Name]]="",tblJobs_ANNEX[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_ANNEX[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_ANNEX[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_ANNEX[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_ANNEX[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet",tblJobs_ANNEX[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_ANNEX[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_ANNEX[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet",tblJobs_ANNEX[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_ANNEX[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_ANNEX[[#This Row],[Print Width mm]]&gt;tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -4194,7 +4204,7 @@
         <v>46282.375</v>
       </c>
       <c r="AF13" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AG13" s="17" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
Reorder PrintCosts.xlsx job-table columns to match built .xlsm layout
Moves Status and Job ID from columns 1-2 to just after Chargeable Cost
in both tblJobs_MAIN and tblJobs_ANNEX, matching where
modInit.ReorderJobColumns settles them in the built workbook, so
editing the source .xlsx directly no longer requires mentally
replaying that VBA step to know where a column ends up. Paid and the
Quantity->Qty rename stay VBA-only, unchanged.

Also fixes two column-index-keyed properties that don't travel with a
Range.Cut/Insert reorder (data validation ranges smeared across the
whole table width, and column widths left following the wrong
content) - the same class of bug modInit.bas already documents for
the .xlsm case, reproduced by hand since the .xlsx has no VBA to
self-heal it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c54d1abecbe6fecc/Development/OfficeApps/PrintJob/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="6_{24FC9915-6BA6-43A0-B0CA-D3ADEEE53F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C302A1D-FF0C-4FFC-8E72-FDFF9E18DB88}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="6_{24FC9915-6BA6-43A0-B0CA-D3ADEEE53F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21341A50-9C56-4BFB-83BA-FFF4C95B0D5C}"/>
   <bookViews>
-    <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -991,138 +991,92 @@
   <dxfs count="82">
     <dxf>
       <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="167" formatCode="#,##0.000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1138,81 +1092,12 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="167" formatCode="#,##0.000"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1228,9 +1113,12 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1246,10 +1134,22 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="#,##0.###"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1265,10 +1165,25 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="#,##0.###"/>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1284,20 +1199,11 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1313,9 +1219,11 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1331,9 +1239,11 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1349,9 +1259,12 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1367,9 +1280,12 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1385,10 +1301,96 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="167" formatCode="#,##0.000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1404,162 +1406,12 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1575,81 +1427,12 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="167" formatCode="#,##0.000"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1665,9 +1448,22 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="#,##0.###"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1683,10 +1479,25 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1702,10 +1513,11 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="#,##0.###"/>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1721,20 +1533,11 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1750,9 +1553,11 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1768,9 +1573,12 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1786,9 +1594,12 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
@@ -1804,6 +1615,139 @@
         <vertical/>
         <horizontal/>
       </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border>
@@ -1824,7 +1768,159 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <border>
         <left style="medium">
           <color rgb="FFBFBFBF"/>
@@ -1963,7 +2059,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
       <border>
         <left style="medium">
           <color rgb="FFBFBFBF"/>
@@ -1982,26 +2078,6 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="3" formatCode="#,##0"/>
       <border>
         <left style="medium">
@@ -2021,9 +2097,23 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDEEAF6"/>
+        </patternFill>
+      </fill>
       <border>
-        <left style="medium">
+        <left style="thin">
           <color rgb="FFBFBFBF"/>
         </left>
         <right style="thin">
@@ -2041,6 +2131,12 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <color rgb="FF595959"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF808080"/>
       </font>
       <fill>
@@ -2050,13 +2146,19 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFDEEAF6"/>
-        </patternFill>
-      </fill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
       <border>
-        <left style="thin">
+        <left style="medium">
           <color rgb="FFBFBFBF"/>
         </left>
         <right style="thin">
@@ -2071,12 +2173,6 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -2109,10 +2205,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A5:D15" totalsRowShown="0">
   <autoFilter ref="A5:D15" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key" dataDxfId="81"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Setting" dataDxfId="80"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Value" dataDxfId="79"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Notes" dataDxfId="78"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key" dataDxfId="78"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Setting" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Value" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Notes" dataDxfId="75"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2136,57 +2232,57 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_MAIN" displayName="tblJobs_MAIN" ref="A12:AG17" totalsRowShown="0">
   <autoFilter ref="A12:AG17" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="33">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Date/Time" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Student No" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="Technician" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="28"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="27">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Quantity" dataDxfId="26"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Print Width mm" dataDxfId="25"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Disregard Paper" dataDxfId="24"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Disregard Consumable" dataDxfId="23"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Area m2" dataDxfId="22">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="21">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="20">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="19">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Disregarded" dataDxfId="18">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" name="Chargeable Cost" dataDxfId="17">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Status" dataDxfId="65">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Job ID" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Date/Time" dataDxfId="63"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="62"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Student No" dataDxfId="61"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="Technician" dataDxfId="60"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="59"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="57">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Quantity" dataDxfId="56"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Print Width mm" dataDxfId="55"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Disregard Paper" dataDxfId="54"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Disregard Consumable" dataDxfId="53"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Area m2" dataDxfId="52">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="51">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="50">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="49">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Disregarded" dataDxfId="48">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" name="Chargeable Cost" dataDxfId="47">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="46"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="45">
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="63"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="62">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="44"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="43"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="42"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0A00-000019000000}" name="S_Family" dataDxfId="41"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="40"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="39"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="38"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="37"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="36"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="35"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="34"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="33"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="61"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="60"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="59"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0A00-000019000000}" name="S_Family" dataDxfId="58"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="57"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="56"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="55"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="54"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="53"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="52"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="51"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2196,57 +2292,57 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="tblJobs_ANNEX" displayName="tblJobs_ANNEX" ref="A12:AG13" totalsRowShown="0">
   <autoFilter ref="A12:AG13" xr:uid="{00000000-0009-0000-0100-00000C000000}"/>
   <tableColumns count="33">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="Status" dataDxfId="32">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="Date/Time" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="Student Name" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="Student No" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="Technician" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="Printer" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="Paper Stock" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="Unit" dataDxfId="10">
+      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="","",IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="Quantity" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0B00-00000B000000}" name="Print Width mm" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0B00-00000C000000}" name="Disregard Paper" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0B00-00000D000000}" name="Disregard Consumable" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0B00-00000E000000}" name="Area m2" dataDxfId="5">
+      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","",IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet",(tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_ANNEX[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_ANNEX[[#This Row],[Quantity]],(IF(tblJobs_ANNEX[[#This Row],[Print Width mm]]="",tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]],tblJobs_ANNEX[[#This Row],[Print Width mm]])/1000)*tblJobs_ANNEX[[#This Row],[Quantity]]))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0B00-00000F000000}" name="Paper Cost" dataDxfId="4">
+      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","",ROUND(tblJobs_ANNEX[[#This Row],[Quantity]]*tblJobs_ANNEX[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0B00-000010000000}" name="Consumable Cost" dataDxfId="3">
+      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Area m2]]="","",ROUND(tblJobs_ANNEX[[#This Row],[Area m2]]*tblJobs_ANNEX[[#This Row],[S_ConsRate]],SET_ROUND_DP))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0B00-000011000000}" name="Gross Cost" dataDxfId="2">
+      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Paper Cost]]="","",tblJobs_ANNEX[[#This Row],[Paper Cost]]+tblJobs_ANNEX[[#This Row],[Consumable Cost]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0B00-000012000000}" name="Disregarded" dataDxfId="1">
+      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Gross Cost]]="","",tblJobs_ANNEX[[#This Row],[Gross Cost]]-tblJobs_ANNEX[[#This Row],[Chargeable Cost]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0B00-000013000000}" name="Chargeable Cost" dataDxfId="0">
+      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Paper Cost]]="","",IF(tblJobs_ANNEX[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_ANNEX[[#This Row],[Paper Cost]])+IF(tblJobs_ANNEX[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_ANNEX[[#This Row],[Consumable Cost]]))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="Status" dataDxfId="49">
       <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Job ID]]="","",IF(tblJobs_ANNEX[[#This Row],[H_Issues]]="","OK",MID(tblJobs_ANNEX[[#This Row],[H_Issues]],3,255)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="Job ID" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="Date/Time" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="Student Name" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="Student No" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="Technician" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="Printer" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="Paper Stock" dataDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="Unit" dataDxfId="24">
-      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="","",IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="Quantity" dataDxfId="23"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0B00-00000B000000}" name="Print Width mm" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0B00-00000C000000}" name="Disregard Paper" dataDxfId="21"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0B00-00000D000000}" name="Disregard Consumable" dataDxfId="20"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0B00-00000E000000}" name="Area m2" dataDxfId="19">
-      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","",IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet",(tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_ANNEX[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_ANNEX[[#This Row],[Quantity]],(IF(tblJobs_ANNEX[[#This Row],[Print Width mm]]="",tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]],tblJobs_ANNEX[[#This Row],[Print Width mm]])/1000)*tblJobs_ANNEX[[#This Row],[Quantity]]))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0B00-00000F000000}" name="Paper Cost" dataDxfId="18">
-      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","",ROUND(tblJobs_ANNEX[[#This Row],[Quantity]]*tblJobs_ANNEX[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0B00-000010000000}" name="Consumable Cost" dataDxfId="17">
-      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Area m2]]="","",ROUND(tblJobs_ANNEX[[#This Row],[Area m2]]*tblJobs_ANNEX[[#This Row],[S_ConsRate]],SET_ROUND_DP))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0B00-000011000000}" name="Gross Cost" dataDxfId="16">
-      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Paper Cost]]="","",tblJobs_ANNEX[[#This Row],[Paper Cost]]+tblJobs_ANNEX[[#This Row],[Consumable Cost]])</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0B00-000012000000}" name="Disregarded" dataDxfId="15">
-      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Gross Cost]]="","",tblJobs_ANNEX[[#This Row],[Gross Cost]]-tblJobs_ANNEX[[#This Row],[Chargeable Cost]])</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0B00-000013000000}" name="Chargeable Cost" dataDxfId="14">
-      <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Paper Cost]]="","",IF(tblJobs_ANNEX[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_ANNEX[[#This Row],[Paper Cost]])+IF(tblJobs_ANNEX[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_ANNEX[[#This Row],[Consumable Cost]]))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0B00-000014000000}" name="Notes" dataDxfId="13"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0B00-000015000000}" name="H_Issues" dataDxfId="12">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="Job ID" dataDxfId="48"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0B00-000014000000}" name="Notes" dataDxfId="47"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0B00-000015000000}" name="H_Issues" dataDxfId="46">
       <calculatedColumnFormula>IF(tblJobs_ANNEX[[#This Row],[Job ID]]="","",IF(tblJobs_ANNEX[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_ANNEX[[#This Row],[Student Name]]="",tblJobs_ANNEX[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_ANNEX[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_ANNEX[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_ANNEX[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_ANNEX[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet",tblJobs_ANNEX[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_ANNEX[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_ANNEX[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet",tblJobs_ANNEX[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_ANNEX[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_ANNEX[[#This Row],[Print Width mm]]&gt;tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0B00-000016000000}" name="S_PrinterID" dataDxfId="11"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0B00-000017000000}" name="S_StockID" dataDxfId="10"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0B00-000018000000}" name="S_TechID" dataDxfId="9"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0B00-000019000000}" name="S_Family" dataDxfId="8"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0B00-00001A000000}" name="S_Measure" dataDxfId="7"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0B00-00001B000000}" name="S_UnitCost" dataDxfId="6"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0B00-00001C000000}" name="S_StockWidth_mm" dataDxfId="5"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0B00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="4"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0B00-00001E000000}" name="S_ConsRate" dataDxfId="3"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0B00-00001F000000}" name="S_StampedAt" dataDxfId="2"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0B00-000020000000}" name="S_StampedBy" dataDxfId="1"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0B00-000021000000}" name="S_SchemaVer" dataDxfId="0"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0B00-000016000000}" name="S_PrinterID" dataDxfId="45"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0B00-000017000000}" name="S_StockID" dataDxfId="44"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0B00-000018000000}" name="S_TechID" dataDxfId="43"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0B00-000019000000}" name="S_Family" dataDxfId="42"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0B00-00001A000000}" name="S_Measure" dataDxfId="41"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0B00-00001B000000}" name="S_UnitCost" dataDxfId="40"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0B00-00001C000000}" name="S_StockWidth_mm" dataDxfId="39"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0B00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="38"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0B00-00001E000000}" name="S_ConsRate" dataDxfId="37"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0B00-00001F000000}" name="S_StampedAt" dataDxfId="36"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0B00-000020000000}" name="S_StampedBy" dataDxfId="35"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0B00-000021000000}" name="S_SchemaVer" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2280,8 +2376,8 @@
   <autoFilter ref="M5:O11" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Size name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Width mm" dataDxfId="77"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Height mm" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Width mm" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Height mm" dataDxfId="73"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2302,7 +2398,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblTechnicians" displayName="tblTechnicians" ref="A5:D8" totalsRowShown="0">
   <autoFilter ref="A5:D8" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="75"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="72"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Department"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Active"/>
@@ -2315,11 +2411,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblPrinters" displayName="tblPrinters" ref="A5:F9" totalsRowShown="0">
   <autoFilter ref="A5:F9" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="74"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="81"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Model"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Consumable type"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="73"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Supported families" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Supported families" dataDxfId="79"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Active"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3050,24 +3146,835 @@
   <dimension ref="A1:AZ17"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.7265625" customWidth="1"/>
-    <col min="2" max="2" width="16.7265625" customWidth="1"/>
-    <col min="3" max="3" width="17.7265625" customWidth="1"/>
-    <col min="4" max="4" width="22.7265625" customWidth="1"/>
-    <col min="5" max="5" width="13.7265625" customWidth="1"/>
-    <col min="6" max="6" width="18.7265625" customWidth="1"/>
-    <col min="7" max="7" width="24.7265625" customWidth="1"/>
-    <col min="8" max="8" width="30.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.7265625" customWidth="1"/>
-    <col min="10" max="10" width="10.7265625" customWidth="1"/>
-    <col min="11" max="11" width="13.7265625" customWidth="1"/>
-    <col min="12" max="12" width="15.7265625" customWidth="1"/>
-    <col min="13" max="13" width="19.7265625" customWidth="1"/>
-    <col min="14" max="14" width="11.7265625" customWidth="1"/>
-    <col min="15" max="15" width="12.7265625" customWidth="1"/>
-    <col min="16" max="16" width="15.7265625" customWidth="1"/>
-    <col min="17" max="18" width="12.7265625" customWidth="1"/>
-    <col min="19" max="19" width="15.7265625" customWidth="1"/>
+    <col min="1" max="1" width="17.7265625" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" customWidth="1"/>
+    <col min="4" max="4" width="18.7265625" customWidth="1"/>
+    <col min="5" max="5" width="24.7265625" customWidth="1"/>
+    <col min="6" max="6" width="30.7265625" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" customWidth="1"/>
+    <col min="8" max="8" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="13.7265625" customWidth="1"/>
+    <col min="10" max="10" width="15.7265625" customWidth="1"/>
+    <col min="11" max="11" width="19.7265625" customWidth="1"/>
+    <col min="12" max="12" width="11.7265625" customWidth="1"/>
+    <col min="13" max="13" width="12.7265625" customWidth="1"/>
+    <col min="14" max="14" width="15.7265625" customWidth="1"/>
+    <col min="15" max="16" width="12.7265625" customWidth="1"/>
+    <col min="17" max="17" width="15.7265625" customWidth="1"/>
+    <col min="18" max="18" width="30.7265625" customWidth="1"/>
+    <col min="19" max="19" width="16.7265625" customWidth="1"/>
+    <col min="20" max="20" width="34.7265625" customWidth="1"/>
+    <col min="21" max="21" width="40.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="24" width="11.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="25" max="25" width="13.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="26" max="26" width="10.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="27" width="12.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="28" width="13.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="29" max="29" width="14.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="30" max="30" width="12.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="31" max="31" width="16.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="32" max="32" width="14.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="33" width="11.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="34" max="34" width="8.7265625" collapsed="1"/>
+    <col min="52" max="52" width="0" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="AL1" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="AL2" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A3" s="21"/>
+      <c r="B3" s="5"/>
+      <c r="D3" s="2"/>
+      <c r="AL3" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A4" s="21"/>
+      <c r="B4" s="7"/>
+      <c r="AL4" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A5" s="21"/>
+      <c r="B5" s="7"/>
+      <c r="AL5" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A6" s="21"/>
+      <c r="B6" s="5"/>
+      <c r="AL6" s="20"/>
+    </row>
+    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A7" s="21"/>
+      <c r="B7" s="5"/>
+      <c r="AL7" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="8" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="AL8" s="20" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="10" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12" spans="1:52" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="R12" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="S12" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="T12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U12" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="V12" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="W12" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="X12" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="Y12" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="Z12" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="AA12" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="AB12" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="AC12" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="AD12" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="AE12" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="AF12" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="AG12" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="13" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A13" s="12">
+        <v>46280.425000000003</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="G13" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+        <v>sheets</v>
+      </c>
+      <c r="H13" s="14">
+        <v>100</v>
+      </c>
+      <c r="I13" s="8"/>
+      <c r="J13" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="K13" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="L13" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
+        <v>14.400000000000002</v>
+      </c>
+      <c r="M13" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>31</v>
+      </c>
+      <c r="N13" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <v>13.68</v>
+      </c>
+      <c r="O13" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <v>44.68</v>
+      </c>
+      <c r="P13" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <v>0</v>
+      </c>
+      <c r="Q13" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <v>44.68</v>
+      </c>
+      <c r="R13" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+        <v>OK</v>
+      </c>
+      <c r="S13" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="T13" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="U13" s="17" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
+        <v/>
+      </c>
+      <c r="V13" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="W13" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="X13" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y13" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z13" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA13" s="18">
+        <v>0.31</v>
+      </c>
+      <c r="AB13" s="17">
+        <v>320</v>
+      </c>
+      <c r="AC13" s="17">
+        <v>450</v>
+      </c>
+      <c r="AD13" s="18">
+        <v>0.95</v>
+      </c>
+      <c r="AE13" s="17">
+        <v>46282.375</v>
+      </c>
+      <c r="AF13" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="AG13" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A14" s="12">
+        <v>46280.611111111109</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="G14" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+        <v>metres</v>
+      </c>
+      <c r="H14" s="14">
+        <v>12</v>
+      </c>
+      <c r="I14" s="8"/>
+      <c r="J14" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="K14" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="L14" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
+        <v>10.968</v>
+      </c>
+      <c r="M14" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>105</v>
+      </c>
+      <c r="N14" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <v>31.26</v>
+      </c>
+      <c r="O14" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <v>136.26</v>
+      </c>
+      <c r="P14" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <v>0</v>
+      </c>
+      <c r="Q14" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <v>136.26</v>
+      </c>
+      <c r="R14" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+        <v>OK</v>
+      </c>
+      <c r="S14" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="T14" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="U14" s="17" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
+        <v/>
+      </c>
+      <c r="V14" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="W14" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="X14" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y14" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z14" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA14" s="18">
+        <v>8.75</v>
+      </c>
+      <c r="AB14" s="17">
+        <v>914</v>
+      </c>
+      <c r="AC14" s="17"/>
+      <c r="AD14" s="18">
+        <v>2.85</v>
+      </c>
+      <c r="AE14" s="17">
+        <v>46282.375</v>
+      </c>
+      <c r="AF14" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="AG14" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A15" s="12">
+        <v>46281.461805555547</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="G15" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+        <v>metres</v>
+      </c>
+      <c r="H15" s="14">
+        <v>12</v>
+      </c>
+      <c r="I15" s="8">
+        <v>600</v>
+      </c>
+      <c r="J15" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="K15" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="L15" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
+        <v>7.1999999999999993</v>
+      </c>
+      <c r="M15" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>105</v>
+      </c>
+      <c r="N15" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <v>20.52</v>
+      </c>
+      <c r="O15" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <v>125.52</v>
+      </c>
+      <c r="P15" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <v>125.52</v>
+      </c>
+      <c r="R15" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+        <v>OK</v>
+      </c>
+      <c r="S15" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="T15" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="U15" s="17" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
+        <v/>
+      </c>
+      <c r="V15" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="W15" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="X15" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y15" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z15" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA15" s="18">
+        <v>8.75</v>
+      </c>
+      <c r="AB15" s="17">
+        <v>914</v>
+      </c>
+      <c r="AC15" s="17"/>
+      <c r="AD15" s="18">
+        <v>2.85</v>
+      </c>
+      <c r="AE15" s="17">
+        <v>46282.375</v>
+      </c>
+      <c r="AF15" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="AG15" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A16" s="12">
+        <v>46281.638888888891</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="G16" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+        <v>metres</v>
+      </c>
+      <c r="H16" s="14">
+        <v>5</v>
+      </c>
+      <c r="I16" s="8"/>
+      <c r="J16" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="K16" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="L16" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
+        <v>3.05</v>
+      </c>
+      <c r="M16" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>15.5</v>
+      </c>
+      <c r="N16" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <v>8.69</v>
+      </c>
+      <c r="O16" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <v>24.189999999999998</v>
+      </c>
+      <c r="P16" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <v>15.499999999999998</v>
+      </c>
+      <c r="Q16" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <v>8.69</v>
+      </c>
+      <c r="R16" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+        <v>OK</v>
+      </c>
+      <c r="S16" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="T16" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="U16" s="17" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
+        <v/>
+      </c>
+      <c r="V16" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="W16" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="X16" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y16" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="Z16" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA16" s="18">
+        <v>3.1</v>
+      </c>
+      <c r="AB16" s="17">
+        <v>610</v>
+      </c>
+      <c r="AC16" s="17"/>
+      <c r="AD16" s="18">
+        <v>2.85</v>
+      </c>
+      <c r="AE16" s="17">
+        <v>46282.375</v>
+      </c>
+      <c r="AF16" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="AG16" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="A17" s="12">
+        <v>46282.395833333343</v>
+      </c>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="G17" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+        <v>metres</v>
+      </c>
+      <c r="H17" s="14">
+        <v>12</v>
+      </c>
+      <c r="I17" s="8">
+        <v>1200</v>
+      </c>
+      <c r="J17" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="K17" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="L17" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
+        <v>14.399999999999999</v>
+      </c>
+      <c r="M17" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>105</v>
+      </c>
+      <c r="N17" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <v>41.04</v>
+      </c>
+      <c r="O17" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <v>146.04</v>
+      </c>
+      <c r="P17" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <v>0</v>
+      </c>
+      <c r="Q17" s="16">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <v>146.04</v>
+      </c>
+      <c r="R17" s="10" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+        <v>Student name or number required; Print width exceeds stock width</v>
+      </c>
+      <c r="S17" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="T17" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="U17" s="17" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
+        <v>; Student name or number required; Print width exceeds stock width</v>
+      </c>
+      <c r="V17" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="W17" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="X17" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y17" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z17" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA17" s="18">
+        <v>8.75</v>
+      </c>
+      <c r="AB17" s="17">
+        <v>914</v>
+      </c>
+      <c r="AC17" s="17"/>
+      <c r="AD17" s="18">
+        <v>2.85</v>
+      </c>
+      <c r="AE17" s="17">
+        <v>46282.375</v>
+      </c>
+      <c r="AF17" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="AG17" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="7">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Technician" error="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." promptTitle="Technician" prompt="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." sqref="D13:D2000" xr:uid="{00000000-0002-0000-0900-000000000000}">
+      <formula1>lstTechnicians</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Only printers available at this print room may be selected." promptTitle="Printer" prompt="Only printers available at this print room may be selected." sqref="E13:E2000" xr:uid="{00000000-0002-0000-0900-000001000000}">
+      <formula1>lstPrinters</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." promptTitle="Paper stock" prompt="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." sqref="F13:F2000" xr:uid="{00000000-0002-0000-0900-000002000000}">
+      <formula1>lstStocks</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J13:K2000" xr:uid="{00000000-0002-0000-0900-000003000000}">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle="Quantity" error="Sheets for sheet stock, metres for roll stock. Must be greater than zero." promptTitle="Quantity" prompt="Sheets for sheet stock, metres for roll stock. Must be greater than zero." sqref="H13:H2000" xr:uid="{00000000-0002-0000-0900-000005000000}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Print width" error="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." promptTitle="Print width" prompt="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." sqref="I13:I2000" xr:uid="{00000000-0002-0000-0900-000006000000}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date and time" error="Date and time the print was produced. Use the Now button to stamp the current date and time." promptTitle="Date and time" prompt="Date and time the print was produced. Use the Now button to stamp the current date and time." sqref="A13:A2000" xr:uid="{00000000-0002-0000-0900-000007000000}">
+      <formula1>36526</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A1:AZ13"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.7265625" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" customWidth="1"/>
+    <col min="4" max="4" width="18.7265625" customWidth="1"/>
+    <col min="5" max="5" width="24.7265625" customWidth="1"/>
+    <col min="6" max="6" width="30.7265625" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" customWidth="1"/>
+    <col min="8" max="8" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="13.7265625" customWidth="1"/>
+    <col min="10" max="10" width="15.7265625" customWidth="1"/>
+    <col min="11" max="11" width="19.7265625" customWidth="1"/>
+    <col min="12" max="12" width="11.7265625" customWidth="1"/>
+    <col min="13" max="13" width="12.7265625" customWidth="1"/>
+    <col min="14" max="14" width="15.7265625" customWidth="1"/>
+    <col min="15" max="16" width="12.7265625" customWidth="1"/>
+    <col min="17" max="17" width="15.7265625" customWidth="1"/>
+    <col min="18" max="18" width="30.7265625" customWidth="1"/>
+    <col min="19" max="19" width="16.7265625" customWidth="1"/>
     <col min="20" max="20" width="34.7265625" customWidth="1"/>
     <col min="21" max="21" width="40.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="22" max="24" width="11.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
@@ -3088,7 +3995,7 @@
         <v>147</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>148</v>
+        <v>214</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>158</v>
@@ -3105,7 +4012,7 @@
         <v>19</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>159</v>
@@ -3114,7 +4021,7 @@
         <v>149</v>
       </c>
       <c r="AM2" t="s">
-        <v>150</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:52" x14ac:dyDescent="0.35">
@@ -3135,7 +4042,7 @@
         <v>153</v>
       </c>
       <c r="AM4" t="s">
-        <v>152</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:52" x14ac:dyDescent="0.35">
@@ -3160,7 +4067,7 @@
         <v>221</v>
       </c>
       <c r="AM7" t="s">
-        <v>154</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:52" x14ac:dyDescent="0.35">
@@ -3193,61 +4100,61 @@
     </row>
     <row r="12" spans="1:52" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="R12" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="S12" s="4" t="s">
         <v>168</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="M12" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="N12" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="O12" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="P12" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Q12" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="R12" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="S12" s="4" t="s">
-        <v>185</v>
       </c>
       <c r="T12" s="4" t="s">
         <v>6</v>
@@ -3293,878 +4200,68 @@
       </c>
     </row>
     <row r="13" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A13" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
-        <v>OK</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="C13" s="12">
-        <v>46280.425000000003</v>
+      <c r="A13" s="12">
+        <v>46281.40625</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>201</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>200</v>
+        <v>87</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>201</v>
+        <v>101</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="H13" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="I13" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+      <c r="G13" s="10" t="str">
+        <f>IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="","",IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
         <v>sheets</v>
       </c>
-      <c r="J13" s="14">
-        <v>100</v>
-      </c>
-      <c r="K13" s="8"/>
-      <c r="L13" s="13" t="s">
+      <c r="H13" s="14">
+        <v>40</v>
+      </c>
+      <c r="I13" s="8"/>
+      <c r="J13" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="M13" s="13" t="s">
+      <c r="K13" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="N13" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
-        <v>14.400000000000002</v>
+      <c r="L13" s="15">
+        <f>IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","",IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet",(tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_ANNEX[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_ANNEX[[#This Row],[Quantity]],(IF(tblJobs_ANNEX[[#This Row],[Print Width mm]]="",tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]],tblJobs_ANNEX[[#This Row],[Print Width mm]])/1000)*tblJobs_ANNEX[[#This Row],[Quantity]]))</f>
+        <v>5.7600000000000007</v>
+      </c>
+      <c r="M13" s="16">
+        <f>IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","",ROUND(tblJobs_ANNEX[[#This Row],[Quantity]]*tblJobs_ANNEX[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>12.4</v>
+      </c>
+      <c r="N13" s="16">
+        <f>IF(tblJobs_ANNEX[[#This Row],[Area m2]]="","",ROUND(tblJobs_ANNEX[[#This Row],[Area m2]]*tblJobs_ANNEX[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <v>5.47</v>
       </c>
       <c r="O13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>31</v>
+        <f>IF(tblJobs_ANNEX[[#This Row],[Paper Cost]]="","",tblJobs_ANNEX[[#This Row],[Paper Cost]]+tblJobs_ANNEX[[#This Row],[Consumable Cost]])</f>
+        <v>17.87</v>
       </c>
       <c r="P13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>13.68</v>
+        <f>IF(tblJobs_ANNEX[[#This Row],[Gross Cost]]="","",tblJobs_ANNEX[[#This Row],[Gross Cost]]-tblJobs_ANNEX[[#This Row],[Chargeable Cost]])</f>
+        <v>0</v>
       </c>
       <c r="Q13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>44.68</v>
-      </c>
-      <c r="R13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>0</v>
-      </c>
-      <c r="S13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>44.68</v>
-      </c>
-      <c r="T13" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="U13" s="17" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
-        <v/>
-      </c>
-      <c r="V13" s="17" t="s">
-        <v>100</v>
-      </c>
-      <c r="W13" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="X13" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="Y13" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z13" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="AA13" s="18">
-        <v>0.31</v>
-      </c>
-      <c r="AB13" s="17">
-        <v>320</v>
-      </c>
-      <c r="AC13" s="17">
-        <v>450</v>
-      </c>
-      <c r="AD13" s="18">
-        <v>0.95</v>
-      </c>
-      <c r="AE13" s="17">
-        <v>46282.375</v>
-      </c>
-      <c r="AF13" s="17" t="s">
-        <v>203</v>
-      </c>
-      <c r="AG13" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A14" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
-        <v>OK</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="C14" s="12">
-        <v>46280.611111111109</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="G14" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="H14" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="I14" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>metres</v>
-      </c>
-      <c r="J14" s="14">
-        <v>12</v>
-      </c>
-      <c r="K14" s="8"/>
-      <c r="L14" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="M14" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="N14" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
-        <v>10.968</v>
-      </c>
-      <c r="O14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>105</v>
-      </c>
-      <c r="P14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>31.26</v>
-      </c>
-      <c r="Q14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>136.26</v>
-      </c>
-      <c r="R14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>0</v>
-      </c>
-      <c r="S14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>136.26</v>
-      </c>
-      <c r="T14" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="U14" s="17" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
-        <v/>
-      </c>
-      <c r="V14" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="W14" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="X14" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="Y14" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z14" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="AA14" s="18">
-        <v>8.75</v>
-      </c>
-      <c r="AB14" s="17">
-        <v>914</v>
-      </c>
-      <c r="AC14" s="17"/>
-      <c r="AD14" s="18">
-        <v>2.85</v>
-      </c>
-      <c r="AE14" s="17">
-        <v>46282.375</v>
-      </c>
-      <c r="AF14" s="17" t="s">
-        <v>203</v>
-      </c>
-      <c r="AG14" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
-        <v>OK</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="C15" s="12">
-        <v>46281.461805555547</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>207</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>208</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="G15" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="H15" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="I15" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>metres</v>
-      </c>
-      <c r="J15" s="14">
-        <v>12</v>
-      </c>
-      <c r="K15" s="8">
-        <v>600</v>
-      </c>
-      <c r="L15" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="M15" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="N15" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
-        <v>7.1999999999999993</v>
-      </c>
-      <c r="O15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>105</v>
-      </c>
-      <c r="P15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>20.52</v>
-      </c>
-      <c r="Q15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>125.52</v>
-      </c>
-      <c r="R15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>0</v>
-      </c>
-      <c r="S15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>125.52</v>
-      </c>
-      <c r="T15" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="U15" s="17" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
-        <v/>
-      </c>
-      <c r="V15" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="W15" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="X15" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="Y15" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z15" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="AA15" s="18">
-        <v>8.75</v>
-      </c>
-      <c r="AB15" s="17">
-        <v>914</v>
-      </c>
-      <c r="AC15" s="17"/>
-      <c r="AD15" s="18">
-        <v>2.85</v>
-      </c>
-      <c r="AE15" s="17">
-        <v>46282.375</v>
-      </c>
-      <c r="AF15" s="17" t="s">
-        <v>203</v>
-      </c>
-      <c r="AG15" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A16" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
-        <v>OK</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="C16" s="12">
-        <v>46281.638888888891</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>207</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>208</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="H16" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="I16" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>metres</v>
-      </c>
-      <c r="J16" s="14">
-        <v>5</v>
-      </c>
-      <c r="K16" s="8"/>
-      <c r="L16" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="M16" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="N16" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
-        <v>3.05</v>
-      </c>
-      <c r="O16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>15.5</v>
-      </c>
-      <c r="P16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>8.69</v>
-      </c>
-      <c r="Q16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>24.189999999999998</v>
-      </c>
-      <c r="R16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>15.499999999999998</v>
-      </c>
-      <c r="S16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>8.69</v>
-      </c>
-      <c r="T16" s="13" t="s">
-        <v>211</v>
-      </c>
-      <c r="U16" s="17" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
-        <v/>
-      </c>
-      <c r="V16" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="W16" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="X16" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="Y16" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="Z16" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="AA16" s="18">
-        <v>3.1</v>
-      </c>
-      <c r="AB16" s="17">
-        <v>610</v>
-      </c>
-      <c r="AC16" s="17"/>
-      <c r="AD16" s="18">
-        <v>2.85</v>
-      </c>
-      <c r="AE16" s="17">
-        <v>46282.375</v>
-      </c>
-      <c r="AF16" s="17" t="s">
-        <v>203</v>
-      </c>
-      <c r="AG16" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
-        <v>Student name or number required; Print width exceeds stock width</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="C17" s="12">
-        <v>46282.395833333343</v>
-      </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="I17" s="10" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>metres</v>
-      </c>
-      <c r="J17" s="14">
-        <v>12</v>
-      </c>
-      <c r="K17" s="8">
-        <v>1200</v>
-      </c>
-      <c r="L17" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="M17" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="N17" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
-        <v>14.399999999999999</v>
-      </c>
-      <c r="O17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>105</v>
-      </c>
-      <c r="P17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>41.04</v>
-      </c>
-      <c r="Q17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>146.04</v>
-      </c>
-      <c r="R17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>0</v>
-      </c>
-      <c r="S17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>146.04</v>
-      </c>
-      <c r="T17" s="13" t="s">
-        <v>213</v>
-      </c>
-      <c r="U17" s="17" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
-        <v>; Student name or number required; Print width exceeds stock width</v>
-      </c>
-      <c r="V17" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="W17" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="X17" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="Y17" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z17" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="AA17" s="18">
-        <v>8.75</v>
-      </c>
-      <c r="AB17" s="17">
-        <v>914</v>
-      </c>
-      <c r="AC17" s="17"/>
-      <c r="AD17" s="18">
-        <v>2.85</v>
-      </c>
-      <c r="AE17" s="17">
-        <v>46282.375</v>
-      </c>
-      <c r="AF17" s="17" t="s">
-        <v>203</v>
-      </c>
-      <c r="AG17" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Technician" error="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." promptTitle="Technician" prompt="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." sqref="F13:F2000" xr:uid="{00000000-0002-0000-0900-000000000000}">
-      <formula1>lstTechnicians</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Only printers available at this print room may be selected." promptTitle="Printer" prompt="Only printers available at this print room may be selected." sqref="G13:G2000" xr:uid="{00000000-0002-0000-0900-000001000000}">
-      <formula1>lstPrinters</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." promptTitle="Paper stock" prompt="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." sqref="H13:H2000" xr:uid="{00000000-0002-0000-0900-000002000000}">
-      <formula1>lstStocks</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L13:M2000" xr:uid="{00000000-0002-0000-0900-000003000000}">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle="Quantity" error="Sheets for sheet stock, metres for roll stock. Must be greater than zero." promptTitle="Quantity" prompt="Sheets for sheet stock, metres for roll stock. Must be greater than zero." sqref="J13:J2000" xr:uid="{00000000-0002-0000-0900-000005000000}">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Print width" error="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." promptTitle="Print width" prompt="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." sqref="K13:K2000" xr:uid="{00000000-0002-0000-0900-000006000000}">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date and time" error="Date and time the print was produced. Use the Now button to stamp the current date and time." promptTitle="Date and time" prompt="Date and time the print was produced. Use the Now button to stamp the current date and time." sqref="C13:C2000" xr:uid="{00000000-0002-0000-0900-000007000000}">
-      <formula1>36526</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:AZ13"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="30.7265625" customWidth="1"/>
-    <col min="2" max="2" width="16.7265625" customWidth="1"/>
-    <col min="3" max="3" width="17.7265625" customWidth="1"/>
-    <col min="4" max="4" width="22.7265625" customWidth="1"/>
-    <col min="5" max="5" width="13.7265625" customWidth="1"/>
-    <col min="6" max="6" width="18.7265625" customWidth="1"/>
-    <col min="7" max="7" width="24.7265625" customWidth="1"/>
-    <col min="8" max="8" width="30.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.7265625" customWidth="1"/>
-    <col min="10" max="10" width="10.7265625" customWidth="1"/>
-    <col min="11" max="11" width="13.7265625" customWidth="1"/>
-    <col min="12" max="12" width="15.7265625" customWidth="1"/>
-    <col min="13" max="13" width="19.7265625" customWidth="1"/>
-    <col min="14" max="14" width="11.7265625" customWidth="1"/>
-    <col min="15" max="15" width="12.7265625" customWidth="1"/>
-    <col min="16" max="16" width="15.7265625" customWidth="1"/>
-    <col min="17" max="18" width="12.7265625" customWidth="1"/>
-    <col min="19" max="19" width="15.7265625" customWidth="1"/>
-    <col min="20" max="20" width="34.7265625" customWidth="1"/>
-    <col min="21" max="21" width="40.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="22" max="24" width="11.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="25" max="25" width="13.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="26" max="26" width="10.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="27" max="27" width="12.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="28" max="28" width="13.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="29" max="29" width="14.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="30" max="30" width="12.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="31" max="31" width="16.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="32" max="32" width="14.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="33" width="11.7265625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="52" max="52" width="0" hidden="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="AL1" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="AL2" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A3" s="21"/>
-      <c r="B3" s="5"/>
-      <c r="D3" s="2"/>
-      <c r="AL3" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A4" s="21"/>
-      <c r="B4" s="7"/>
-      <c r="AL4" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A5" s="21"/>
-      <c r="B5" s="7"/>
-      <c r="AL5" s="19" t="s">
-        <v>155</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A6" s="21"/>
-      <c r="B6" s="5"/>
-      <c r="AL6" s="20"/>
-    </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A7" s="21"/>
-      <c r="B7" s="5"/>
-      <c r="AL7" s="19" t="s">
-        <v>221</v>
-      </c>
-      <c r="AM7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="AL8" s="20" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="10" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="12" spans="1:52" ht="29" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="M12" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="N12" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="O12" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="P12" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Q12" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="R12" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="S12" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="T12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="U12" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="V12" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="W12" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="X12" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="Y12" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="Z12" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="AA12" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="AB12" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="AC12" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="AD12" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="AE12" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="AF12" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="AG12" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="13" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A13" s="10" t="str">
+        <f>IF(tblJobs_ANNEX[[#This Row],[Paper Cost]]="","",IF(tblJobs_ANNEX[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_ANNEX[[#This Row],[Paper Cost]])+IF(tblJobs_ANNEX[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_ANNEX[[#This Row],[Consumable Cost]]))</f>
+        <v>17.87</v>
+      </c>
+      <c r="R13" s="10" t="str">
         <f>IF(tblJobs_ANNEX[[#This Row],[Job ID]]="","",IF(tblJobs_ANNEX[[#This Row],[H_Issues]]="","OK",MID(tblJobs_ANNEX[[#This Row],[H_Issues]],3,255)))</f>
         <v>OK</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="S13" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="C13" s="12">
-        <v>46281.40625</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="H13" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="I13" s="10" t="str">
-        <f>IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="","",IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>sheets</v>
-      </c>
-      <c r="J13" s="14">
-        <v>40</v>
-      </c>
-      <c r="K13" s="8"/>
-      <c r="L13" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="M13" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="N13" s="15">
-        <f>IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","",IF(tblJobs_ANNEX[[#This Row],[S_Measure]]="Sheet",(tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_ANNEX[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_ANNEX[[#This Row],[Quantity]],(IF(tblJobs_ANNEX[[#This Row],[Print Width mm]]="",tblJobs_ANNEX[[#This Row],[S_StockWidth_mm]],tblJobs_ANNEX[[#This Row],[Print Width mm]])/1000)*tblJobs_ANNEX[[#This Row],[Quantity]]))</f>
-        <v>5.7600000000000007</v>
-      </c>
-      <c r="O13" s="16">
-        <f>IF(tblJobs_ANNEX[[#This Row],[Quantity]]="","",ROUND(tblJobs_ANNEX[[#This Row],[Quantity]]*tblJobs_ANNEX[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>12.4</v>
-      </c>
-      <c r="P13" s="16">
-        <f>IF(tblJobs_ANNEX[[#This Row],[Area m2]]="","",ROUND(tblJobs_ANNEX[[#This Row],[Area m2]]*tblJobs_ANNEX[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>5.47</v>
-      </c>
-      <c r="Q13" s="16">
-        <f>IF(tblJobs_ANNEX[[#This Row],[Paper Cost]]="","",tblJobs_ANNEX[[#This Row],[Paper Cost]]+tblJobs_ANNEX[[#This Row],[Consumable Cost]])</f>
-        <v>17.87</v>
-      </c>
-      <c r="R13" s="16">
-        <f>IF(tblJobs_ANNEX[[#This Row],[Gross Cost]]="","",tblJobs_ANNEX[[#This Row],[Gross Cost]]-tblJobs_ANNEX[[#This Row],[Chargeable Cost]])</f>
-        <v>0</v>
-      </c>
-      <c r="S13" s="16">
-        <f>IF(tblJobs_ANNEX[[#This Row],[Paper Cost]]="","",IF(tblJobs_ANNEX[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_ANNEX[[#This Row],[Paper Cost]])+IF(tblJobs_ANNEX[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_ANNEX[[#This Row],[Consumable Cost]]))</f>
-        <v>17.87</v>
       </c>
       <c r="T13" s="13" t="s">
         <v>218</v>
@@ -4212,25 +4309,25 @@
     </row>
   </sheetData>
   <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Technician" error="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." promptTitle="Technician" prompt="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." sqref="F13:F2000" xr:uid="{00000000-0002-0000-0A00-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Technician" error="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." promptTitle="Technician" prompt="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." sqref="D13:D2000" xr:uid="{00000000-0002-0000-0A00-000000000000}">
       <formula1>lstTechnicians</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Only printers available at this print room may be selected." promptTitle="Printer" prompt="Only printers available at this print room may be selected." sqref="G13:G2000" xr:uid="{00000000-0002-0000-0A00-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Only printers available at this print room may be selected." promptTitle="Printer" prompt="Only printers available at this print room may be selected." sqref="E13:E2000" xr:uid="{00000000-0002-0000-0A00-000001000000}">
       <formula1>lstPrinters</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." promptTitle="Paper stock" prompt="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." sqref="H13:H2000" xr:uid="{00000000-0002-0000-0A00-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." promptTitle="Paper stock" prompt="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." sqref="F13:F2000" xr:uid="{00000000-0002-0000-0A00-000002000000}">
       <formula1>lstStocks</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L13:M2000" xr:uid="{00000000-0002-0000-0A00-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J13:K2000" xr:uid="{00000000-0002-0000-0A00-000003000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle="Quantity" error="Sheets for sheet stock, metres for roll stock. Must be greater than zero." promptTitle="Quantity" prompt="Sheets for sheet stock, metres for roll stock. Must be greater than zero." sqref="J13:J2000" xr:uid="{00000000-0002-0000-0A00-000005000000}">
+    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle="Quantity" error="Sheets for sheet stock, metres for roll stock. Must be greater than zero." promptTitle="Quantity" prompt="Sheets for sheet stock, metres for roll stock. Must be greater than zero." sqref="H13:H2000" xr:uid="{00000000-0002-0000-0A00-000005000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Print width" error="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." promptTitle="Print width" prompt="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." sqref="K13:K2000" xr:uid="{00000000-0002-0000-0A00-000006000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Print width" error="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." promptTitle="Print width" prompt="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." sqref="I13:I2000" xr:uid="{00000000-0002-0000-0A00-000006000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date and time" error="Date and time the print was produced. Use the Now button to stamp the current date and time." promptTitle="Date and time" prompt="Date and time the print was produced. Use the Now button to stamp the current date and time." sqref="C13:C2000" xr:uid="{00000000-0002-0000-0A00-000007000000}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date and time" error="Date and time the print was produced. Use the Now button to stamp the current date and time." promptTitle="Date and time" prompt="Date and time the print was produced. Use the Now button to stamp the current date and time." sqref="A13:A2000" xr:uid="{00000000-0002-0000-0A00-000007000000}">
       <formula1>36526</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix Qty cell style on sample rows 7-12 (UNI-MAIN-00006 onward)
Rows 18-24 of Main Print Room's Qty column shipped with the grey
calculated-column style (fontId7/fillId3) instead of the plain white
input style every other column's row uses - a mistake from rewriting
this sheet's sample data, not a formula or value problem. Repeat Job
(and any other row later appended after one of these) inherited it via
Excel's normal copy-the-row-above formatting behaviour, which is what
made it look like Repeat Job or a centimetres entry was doing the
shading - neither actually touches cell formatting.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -3431,7 +3431,7 @@
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
         <v>sheets</v>
       </c>
-      <c r="H18" s="23">
+      <c r="H18" s="14">
         <v>15</v>
       </c>
       <c r="I18" s="8"/>
@@ -3539,7 +3539,7 @@
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
         <v>metres</v>
       </c>
-      <c r="H19" s="23">
+      <c r="H19" s="14">
         <v>8</v>
       </c>
       <c r="I19" s="8"/>
@@ -3643,7 +3643,7 @@
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
         <v>metres</v>
       </c>
-      <c r="H20" s="23">
+      <c r="H20" s="14">
         <v>3</v>
       </c>
       <c r="I20" s="8"/>
@@ -3747,7 +3747,7 @@
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
         <v>sheets</v>
       </c>
-      <c r="H21" s="23">
+      <c r="H21" s="14">
         <v>30</v>
       </c>
       <c r="I21" s="8"/>
@@ -3855,7 +3855,7 @@
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
         <v>metres</v>
       </c>
-      <c r="H22" s="23">
+      <c r="H22" s="14">
         <v>20</v>
       </c>
       <c r="I22" s="8"/>
@@ -3961,7 +3961,7 @@
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
         <v>sheets</v>
       </c>
-      <c r="H23" s="23">
+      <c r="H23" s="14">
         <v>40</v>
       </c>
       <c r="I23" s="8"/>
@@ -4065,7 +4065,7 @@
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
         <v>metres</v>
       </c>
-      <c r="H24" s="23">
+      <c r="H24" s="14">
         <v>12</v>
       </c>
       <c r="I24" s="8">

</xml_diff>

<commit_message>
Remove HP Latex 335 from Main Print Room's permitted printers
It had drifted back onto LOC_Printers, breaking test-dropdowns.ps1's
Long Roll auto-fill scenario, which needs exactly one permitted
printer (Epson) supporting Long Roll.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\PrintCostsFix-c708740d6a5d43ea83fedea3cc905c21\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFB4C955-97CB-4C4E-87BC-31FAB63B1A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5602741-F2E2-48B5-BFEE-59EFA7E02F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -751,13 +751,13 @@
     <t>UNI-MAIN-00011</t>
   </si>
   <si>
-    <t>Epson SureColor P9500;HP DesignJet Z9+;Xerox Versant 180;HP Latex 335</t>
-  </si>
-  <si>
     <t>UNI-MAIN-00012</t>
   </si>
   <si>
     <t>Open day posters</t>
+  </si>
+  <si>
+    <t>Epson SureColor P9500;HP DesignJet Z9+;Xerox Versant 180</t>
   </si>
 </sst>
 </file>
@@ -1019,6 +1019,231 @@
   <dxfs count="49">
     <dxf>
       <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <border>
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border>
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border>
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <border>
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border>
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border>
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDEEAF6"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF595959"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF808080"/>
       </font>
       <fill>
@@ -1492,231 +1717,6 @@
       </border>
       <protection locked="0" hidden="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <border>
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border>
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border>
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
-      <border>
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border>
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border>
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDEEAF6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1734,10 +1734,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A5:D15" totalsRowShown="0">
   <autoFilter ref="A5:D15" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Setting" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Value" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Notes" dataDxfId="45"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Setting" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Value" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Notes" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1761,57 +1761,57 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_MAIN" displayName="tblJobs_MAIN" ref="A12:AG24" totalsRowShown="0">
   <autoFilter ref="A12:AG24" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="33">
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Date/Time" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Student No" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="Technician" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="27"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="26">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Date/Time" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Student No" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="Technician" dataDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="42">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Quantity" dataDxfId="25"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Print Width mm" dataDxfId="24"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Disregard Paper" dataDxfId="23"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Disregard Consumable" dataDxfId="22"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Area m2" dataDxfId="21">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Quantity" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Print Width mm" dataDxfId="40"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Disregard Paper" dataDxfId="39"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Disregard Consumable" dataDxfId="38"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Area m2" dataDxfId="37">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="20">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="36">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="19">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="35">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="18">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="34">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Disregarded" dataDxfId="17">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Disregarded" dataDxfId="33">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" name="Chargeable Cost" dataDxfId="16">
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" name="Chargeable Cost" dataDxfId="32">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Status" dataDxfId="15">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Status" dataDxfId="31">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Job ID" dataDxfId="14"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="13"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="12">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Job ID" dataDxfId="30"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="29"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="28">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="11"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="10"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="9"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0A00-000019000000}" name="S_Family" dataDxfId="8"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="7"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="6"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="5"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="4"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="3"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="2"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="1"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="0"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="27"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="26"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="25"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0A00-000019000000}" name="S_Family" dataDxfId="24"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="23"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="22"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="21"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="20"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="19"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="18"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="17"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1845,8 +1845,8 @@
   <autoFilter ref="M5:O11" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Size name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Width mm" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Height mm" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Width mm" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Height mm" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1867,7 +1867,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblTechnicians" displayName="tblTechnicians" ref="A5:D8" totalsRowShown="0">
   <autoFilter ref="A5:D8" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Department"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Active"/>
@@ -1880,11 +1880,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblPrinters" displayName="tblPrinters" ref="A5:F9" totalsRowShown="0">
   <autoFilter ref="A5:F9" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Model"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Consumable type"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Supported families" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Supported families" dataDxfId="6"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Active"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1895,19 +1895,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A5:L14" totalsRowShown="0">
   <autoFilter ref="A5:L14" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Description"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Paper type"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Family"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Measure" dataDxfId="37">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Measure" dataDxfId="4">
       <calculatedColumnFormula>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Size mode"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Standard size"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Width mm" dataDxfId="36"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Height mm" dataDxfId="35"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Cost" dataDxfId="34"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Cost unit" dataDxfId="33">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Width mm" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Height mm" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Cost" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Cost unit" dataDxfId="0">
       <calculatedColumnFormula>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Active"/>
@@ -2726,7 +2726,7 @@
         <v>212</v>
       </c>
       <c r="AM7" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:52" x14ac:dyDescent="0.35">
@@ -3989,7 +3989,7 @@
         <v>226</v>
       </c>
       <c r="T23" s="13" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="U23" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -4092,7 +4092,7 @@
         <v>Student name or number required; Print width exceeds stock width</v>
       </c>
       <c r="S24" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="T24" s="13" t="s">
         <v>225</v>

</xml_diff>

<commit_message>
Rename shipped location sheet to Example Print Room
Its literal name read as a real production room; renaming it (tab and
LOC_Name) makes clear it is the template duplicated when adding a new
print room, especially now that an automated add-room command is
about to treat it as exactly that. Updates every test script and doc
reference alongside it.
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\PrintCostsFix-c708740d6a5d43ea83fedea3cc905c21\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5602741-F2E2-48B5-BFEE-59EFA7E02F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FA38F3-9CFE-400B-90FC-58AFAF48BE81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,16 +22,16 @@
     <sheet name="_Export" sheetId="7" state="veryHidden" r:id="rId7"/>
     <sheet name="_Audit" sheetId="8" state="veryHidden" r:id="rId8"/>
     <sheet name="_Picker" sheetId="9" state="veryHidden" r:id="rId9"/>
-    <sheet name="Main Print Room" sheetId="10" r:id="rId10"/>
+    <sheet name="Example Print Room" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="LOC_Code" localSheetId="9">'Main Print Room'!$AM$2</definedName>
-    <definedName name="LOC_DefDisCons" localSheetId="9">'Main Print Room'!$AM$4</definedName>
-    <definedName name="LOC_DefDisPaper" localSheetId="9">'Main Print Room'!$AM$3</definedName>
-    <definedName name="LOC_Dept" localSheetId="9">'Main Print Room'!$B$2</definedName>
-    <definedName name="LOC_Name" localSheetId="9">'Main Print Room'!$B$1</definedName>
-    <definedName name="LOC_Printers" localSheetId="9">'Main Print Room'!$AM$7</definedName>
-    <definedName name="LOC_Status" localSheetId="9">'Main Print Room'!$AM$5</definedName>
+    <definedName name="LOC_Code" localSheetId="9">'Example Print Room'!$AM$2</definedName>
+    <definedName name="LOC_DefDisCons" localSheetId="9">'Example Print Room'!$AM$4</definedName>
+    <definedName name="LOC_DefDisPaper" localSheetId="9">'Example Print Room'!$AM$3</definedName>
+    <definedName name="LOC_Dept" localSheetId="9">'Example Print Room'!$B$2</definedName>
+    <definedName name="LOC_Name" localSheetId="9">'Example Print Room'!$B$1</definedName>
+    <definedName name="LOC_Printers" localSheetId="9">'Example Print Room'!$AM$7</definedName>
+    <definedName name="LOC_Status" localSheetId="9">'Example Print Room'!$AM$5</definedName>
     <definedName name="lstConsumables">tblConsumables[Consumable type]</definedName>
     <definedName name="lstFamilies">tblPaperFamilies[Family]</definedName>
     <definedName name="lstPaperTypes">tblPaperTypes[Paper type]</definedName>
@@ -50,7 +50,7 @@
     <definedName name="SET_SITE_ID">Settings!$C$6</definedName>
     <definedName name="SET_SITE_NAME">Settings!$C$7</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="manual" calcOnSave="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -514,9 +514,6 @@
     <t>Print room</t>
   </si>
   <si>
-    <t>Main Print Room</t>
-  </si>
-  <si>
     <t>Location code</t>
   </si>
   <si>
@@ -758,6 +755,9 @@
   </si>
   <si>
     <t>Epson SureColor P9500;HP DesignJet Z9+;Xerox Versant 180</t>
+  </si>
+  <si>
+    <t>Example Print Room</t>
   </si>
 </sst>
 </file>
@@ -2654,16 +2654,16 @@
         <v>147</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>148</v>
+        <v>229</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AL1" s="19" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AZ1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:52" x14ac:dyDescent="0.35">
@@ -2674,13 +2674,13 @@
         <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AL2" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="AM2" t="s">
         <v>149</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:52" x14ac:dyDescent="0.35">
@@ -2688,30 +2688,30 @@
       <c r="B3" s="5"/>
       <c r="D3" s="2"/>
       <c r="AL3" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="AM3" t="s">
         <v>151</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A4" s="21"/>
       <c r="B4" s="7"/>
       <c r="AL4" s="19" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AM4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A5" s="21"/>
       <c r="B5" s="7"/>
       <c r="AL5" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="AM5" t="s">
         <v>154</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.35">
@@ -2723,139 +2723,139 @@
       <c r="A7" s="21"/>
       <c r="B7" s="5"/>
       <c r="AL7" s="19" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AM7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8" spans="1:52" x14ac:dyDescent="0.35">
       <c r="AL8" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="I10" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="K10" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="M10" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="12" spans="1:52" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="H12" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="I12" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="J12" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="K12" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="L12" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="L12" s="4" t="s">
+      <c r="M12" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="N12" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="O12" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="O12" s="4" t="s">
+      <c r="P12" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="P12" s="4" t="s">
+      <c r="Q12" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="Q12" s="4" t="s">
-        <v>184</v>
-      </c>
       <c r="R12" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="S12" s="4" t="s">
         <v>166</v>
-      </c>
-      <c r="S12" s="4" t="s">
-        <v>167</v>
       </c>
       <c r="T12" s="4" t="s">
         <v>6</v>
       </c>
       <c r="U12" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="V12" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="V12" s="4" t="s">
+      <c r="W12" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="W12" s="4" t="s">
+      <c r="X12" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="X12" s="4" t="s">
+      <c r="Y12" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="Y12" s="4" t="s">
+      <c r="Z12" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="Z12" s="4" t="s">
+      <c r="AA12" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="AA12" s="4" t="s">
+      <c r="AB12" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="AB12" s="4" t="s">
+      <c r="AC12" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="AC12" s="4" t="s">
+      <c r="AD12" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="AD12" s="4" t="s">
+      <c r="AE12" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="AE12" s="4" t="s">
+      <c r="AF12" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="AF12" s="4" t="s">
+      <c r="AG12" s="4" t="s">
         <v>196</v>
-      </c>
-      <c r="AG12" s="4" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="13" spans="1:52" x14ac:dyDescent="0.35">
@@ -2863,7 +2863,7 @@
         <v>46280.425000000003</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C13" s="13">
         <v>2201884</v>
@@ -2886,10 +2886,10 @@
       </c>
       <c r="I13" s="8"/>
       <c r="J13" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L13" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -2920,10 +2920,10 @@
         <v>OK</v>
       </c>
       <c r="S13" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="T13" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="U13" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -2960,7 +2960,7 @@
         <v>46280.425000000003</v>
       </c>
       <c r="AF13" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG13" s="17">
         <v>1</v>
@@ -2971,7 +2971,7 @@
         <v>46280.611111111109</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C14" s="13">
         <v>2201884</v>
@@ -2994,10 +2994,10 @@
       </c>
       <c r="I14" s="8"/>
       <c r="J14" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L14" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -3028,10 +3028,10 @@
         <v>OK</v>
       </c>
       <c r="S14" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="T14" s="13" t="s">
         <v>202</v>
-      </c>
-      <c r="T14" s="13" t="s">
-        <v>203</v>
       </c>
       <c r="U14" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3066,7 +3066,7 @@
         <v>46280.611111111109</v>
       </c>
       <c r="AF14" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG14" s="17">
         <v>1</v>
@@ -3077,7 +3077,7 @@
         <v>46281.461805555555</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C15" s="13">
         <v>2203110</v>
@@ -3102,10 +3102,10 @@
         <v>600</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L15" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -3136,10 +3136,10 @@
         <v>OK</v>
       </c>
       <c r="S15" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="T15" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="U15" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3174,7 +3174,7 @@
         <v>46281.461805555555</v>
       </c>
       <c r="AF15" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG15" s="17">
         <v>1</v>
@@ -3185,7 +3185,7 @@
         <v>46281.638888888891</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C16" s="13">
         <v>2203110</v>
@@ -3211,7 +3211,7 @@
         <v>44</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L16" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -3242,10 +3242,10 @@
         <v>OK</v>
       </c>
       <c r="S16" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="T16" s="13" t="s">
         <v>207</v>
-      </c>
-      <c r="T16" s="13" t="s">
-        <v>208</v>
       </c>
       <c r="U16" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3280,7 +3280,7 @@
         <v>46281.638888888891</v>
       </c>
       <c r="AF16" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG16" s="17">
         <v>1</v>
@@ -3291,7 +3291,7 @@
         <v>46282.381944444445</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C17" s="13">
         <v>2204521</v>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="I17" s="8"/>
       <c r="J17" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K17" s="13" t="s">
         <v>44</v>
@@ -3348,10 +3348,10 @@
         <v>OK</v>
       </c>
       <c r="S17" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="T17" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="U17" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3388,7 +3388,7 @@
         <v>46282.381944444445</v>
       </c>
       <c r="AF17" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG17" s="17">
         <v>1</v>
@@ -3399,7 +3399,7 @@
         <v>46282.559027777781</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C18" s="13">
         <v>2204521</v>
@@ -3422,10 +3422,10 @@
       </c>
       <c r="I18" s="8"/>
       <c r="J18" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L18" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -3456,10 +3456,10 @@
         <v>OK</v>
       </c>
       <c r="S18" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="T18" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="U18" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3496,7 +3496,7 @@
         <v>46282.559027777781</v>
       </c>
       <c r="AF18" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG18" s="17">
         <v>1</v>
@@ -3507,7 +3507,7 @@
         <v>46282.666666666664</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C19" s="13">
         <v>2204521</v>
@@ -3530,10 +3530,10 @@
       </c>
       <c r="I19" s="8"/>
       <c r="J19" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L19" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -3564,10 +3564,10 @@
         <v>OK</v>
       </c>
       <c r="S19" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="T19" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="U19" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3602,7 +3602,7 @@
         <v>46282.666666666664</v>
       </c>
       <c r="AF19" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG19" s="17">
         <v>1</v>
@@ -3634,10 +3634,10 @@
       </c>
       <c r="I20" s="8"/>
       <c r="J20" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L20" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -3668,10 +3668,10 @@
         <v>OK</v>
       </c>
       <c r="S20" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="T20" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="U20" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3706,7 +3706,7 @@
         <v>46283.427083333336</v>
       </c>
       <c r="AF20" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG20" s="17">
         <v>1</v>
@@ -3738,10 +3738,10 @@
       </c>
       <c r="I21" s="8"/>
       <c r="J21" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L21" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -3772,10 +3772,10 @@
         <v>OK</v>
       </c>
       <c r="S21" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="T21" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="U21" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3812,7 +3812,7 @@
         <v>46283.486111111109</v>
       </c>
       <c r="AF21" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG21" s="17">
         <v>1</v>
@@ -3823,7 +3823,7 @@
         <v>46283.638888888891</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C22" s="13">
         <v>2204521</v>
@@ -3846,10 +3846,10 @@
       </c>
       <c r="I22" s="8"/>
       <c r="J22" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K22" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L22" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -3880,10 +3880,10 @@
         <v>OK</v>
       </c>
       <c r="S22" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="T22" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="U22" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -3918,7 +3918,7 @@
         <v>46283.638888888891</v>
       </c>
       <c r="AF22" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG22" s="17">
         <v>1</v>
@@ -3929,7 +3929,7 @@
         <v>46284.34375</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C23" s="13">
         <v>2203110</v>
@@ -3952,10 +3952,10 @@
       </c>
       <c r="I23" s="8"/>
       <c r="J23" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L23" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -3986,10 +3986,10 @@
         <v>OK</v>
       </c>
       <c r="S23" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="T23" s="13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="U23" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -4026,7 +4026,7 @@
         <v>46284.34375</v>
       </c>
       <c r="AF23" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG23" s="17">
         <v>1</v>
@@ -4058,10 +4058,10 @@
         <v>1200</v>
       </c>
       <c r="J24" s="23" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K24" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L24" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
@@ -4092,10 +4092,10 @@
         <v>Student name or number required; Print width exceeds stock width</v>
       </c>
       <c r="S24" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="T24" s="13" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="U24" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
@@ -4130,7 +4130,7 @@
         <v>46284.395833333336</v>
       </c>
       <c r="AF24" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG24" s="17">
         <v>1</v>

</xml_diff>

<commit_message>
Drop unused SET_FOOTER and SET_FY_START settings
Both were defined names with no code consumer since inception. Asked
whether to wire each up or drop them; user chose to drop both, so the
tblSettings rows and defined names are removed rather than left as
dead weight.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FA38F3-9CFE-400B-90FC-58AFAF48BE81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7036EBF1-67B3-4238-8892-9A211C6737BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,16 +41,14 @@
     <definedName name="lstTechnicians">tblTechnicians[Name]</definedName>
     <definedName name="SET_CURRENCY">Settings!$C$10</definedName>
     <definedName name="SET_DEPT">Settings!$C$9</definedName>
-    <definedName name="SET_FOOTER">Settings!$C$12</definedName>
-    <definedName name="SET_FY_START">Settings!$C$13</definedName>
-    <definedName name="SET_LASTREF">Settings!$C$15</definedName>
+    <definedName name="SET_LASTREF">Settings!$C$13</definedName>
     <definedName name="SET_ORG">Settings!$C$8</definedName>
     <definedName name="SET_ROUND_DP">Settings!$C$11</definedName>
-    <definedName name="SET_SCHEMA">Settings!$C$14</definedName>
+    <definedName name="SET_SCHEMA">Settings!$C$12</definedName>
     <definedName name="SET_SITE_ID">Settings!$C$6</definedName>
     <definedName name="SET_SITE_NAME">Settings!$C$7</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcMode="manual" calcOnSave="0"/>
+  <calcPr calcId="191029" calcMode="manual" calcCompleted="0" calcOnSave="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -68,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="225">
   <si>
     <t>Settings</t>
   </si>
@@ -152,21 +150,6 @@
   </si>
   <si>
     <t>WARNING: changing this recalculates the cost of existing records.</t>
-  </si>
-  <si>
-    <t>FOOTER</t>
-  </si>
-  <si>
-    <t>Report footer</t>
-  </si>
-  <si>
-    <t>FY_START</t>
-  </si>
-  <si>
-    <t>Financial year start</t>
-  </si>
-  <si>
-    <t>1 August</t>
   </si>
   <si>
     <t>SCHEMA</t>
@@ -1731,8 +1714,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A5:D15" totalsRowShown="0">
-  <autoFilter ref="A5:D15" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A5:D13" totalsRowShown="0">
+  <autoFilter ref="A5:D13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Setting" dataDxfId="14"/>
@@ -2220,7 +2203,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
@@ -2249,12 +2232,12 @@
         <v>1</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="T3" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.35">
@@ -2262,16 +2245,16 @@
         <v>2</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.35">
@@ -2288,34 +2271,34 @@
         <v>6</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.35">
@@ -2332,22 +2315,22 @@
         <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I6" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="J6" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="K6" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="M6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="N6" s="8">
         <v>841</v>
@@ -2356,10 +2339,10 @@
         <v>1189</v>
       </c>
       <c r="Q6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="R6" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.35">
@@ -2374,22 +2357,22 @@
       </c>
       <c r="D7" s="5"/>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="J7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="K7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="M7" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="N7" s="8">
         <v>594</v>
@@ -2398,10 +2381,10 @@
         <v>841</v>
       </c>
       <c r="Q7" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="R7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.35">
@@ -2418,22 +2401,22 @@
         <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="J8" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="K8" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="M8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="N8" s="8">
         <v>420</v>
@@ -2442,10 +2425,10 @@
         <v>594</v>
       </c>
       <c r="Q8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="R8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.35">
@@ -2460,13 +2443,13 @@
       </c>
       <c r="D9" s="5"/>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="M9" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="N9" s="8">
         <v>297</v>
@@ -2475,10 +2458,10 @@
         <v>420</v>
       </c>
       <c r="Q9" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="R9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.35">
@@ -2495,13 +2478,13 @@
         <v>24</v>
       </c>
       <c r="F10" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="G10" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="M10" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="N10" s="8">
         <v>210</v>
@@ -2524,13 +2507,13 @@
         <v>27</v>
       </c>
       <c r="F11" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G11" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="M11" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="N11" s="8">
         <v>320</v>
@@ -2546,48 +2529,27 @@
       <c r="B12" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="5"/>
+      <c r="C12" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="5"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A14" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C13" s="7"/>
+      <c r="D13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A15" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="5" t="s">
-        <v>39</v>
-      </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Measurement basis" error="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." promptTitle="Measurement basis" prompt="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." sqref="J6:J2000" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Sheet,Roll"</formula1>
@@ -2651,19 +2613,19 @@
   <sheetData>
     <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="AL1" s="19" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="AZ1" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:52" x14ac:dyDescent="0.35">
@@ -2674,13 +2636,13 @@
         <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="AL2" s="19" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="AM2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:52" x14ac:dyDescent="0.35">
@@ -2688,30 +2650,30 @@
       <c r="B3" s="5"/>
       <c r="D3" s="2"/>
       <c r="AL3" s="19" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="AM3" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A4" s="21"/>
       <c r="B4" s="7"/>
       <c r="AL4" s="19" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="AM4" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A5" s="21"/>
       <c r="B5" s="7"/>
       <c r="AL5" s="19" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="AM5" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.35">
@@ -2723,139 +2685,139 @@
       <c r="A7" s="21"/>
       <c r="B7" s="5"/>
       <c r="AL7" s="19" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="AM7" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:52" x14ac:dyDescent="0.35">
       <c r="AL8" s="20" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="K10" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="M10" s="2" t="s">
         <v>159</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:52" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="H12" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="I12" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="J12" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="K12" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="L12" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="M12" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="N12" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="O12" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="P12" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="L12" s="4" t="s">
+      <c r="Q12" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="M12" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="N12" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="O12" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="P12" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="Q12" s="4" t="s">
-        <v>183</v>
-      </c>
       <c r="R12" s="4" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="T12" s="4" t="s">
         <v>6</v>
       </c>
       <c r="U12" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="V12" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="W12" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="X12" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y12" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="Z12" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="V12" s="4" t="s">
+      <c r="AA12" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="W12" s="4" t="s">
+      <c r="AB12" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="X12" s="4" t="s">
+      <c r="AC12" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="Y12" s="4" t="s">
+      <c r="AD12" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="Z12" s="4" t="s">
+      <c r="AE12" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="AA12" s="4" t="s">
+      <c r="AF12" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="AB12" s="4" t="s">
+      <c r="AG12" s="4" t="s">
         <v>191</v>
-      </c>
-      <c r="AC12" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="AD12" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="AE12" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="AF12" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="AG12" s="4" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="13" spans="1:52" x14ac:dyDescent="0.35">
@@ -2863,19 +2825,19 @@
         <v>46280.425000000003</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C13" s="13">
         <v>2201884</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="G13" s="10" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -2886,33 +2848,33 @@
       </c>
       <c r="I13" s="8"/>
       <c r="J13" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L13" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>14.400000000000002</v>
       </c>
       <c r="M13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>31</v>
       </c>
       <c r="N13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>13.68</v>
       </c>
       <c r="O13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>44.68</v>
       </c>
       <c r="P13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q13" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>44.68</v>
       </c>
       <c r="R13" s="10" t="str">
@@ -2920,29 +2882,29 @@
         <v>OK</v>
       </c>
       <c r="S13" s="5" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="T13" s="13" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="U13" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V13" s="17" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="W13" s="17" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="X13" s="17" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="Y13" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="Z13" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="AA13" s="18">
         <v>0.31</v>
@@ -2960,7 +2922,7 @@
         <v>46280.425000000003</v>
       </c>
       <c r="AF13" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG13" s="17">
         <v>1</v>
@@ -2971,19 +2933,19 @@
         <v>46280.611111111109</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C14" s="13">
         <v>2201884</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="G14" s="10" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -2994,33 +2956,33 @@
       </c>
       <c r="I14" s="8"/>
       <c r="J14" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L14" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>10.968</v>
       </c>
       <c r="M14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>105</v>
       </c>
       <c r="N14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>31.26</v>
       </c>
       <c r="O14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>136.26</v>
       </c>
       <c r="P14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q14" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>136.26</v>
       </c>
       <c r="R14" s="10" t="str">
@@ -3028,29 +2990,29 @@
         <v>OK</v>
       </c>
       <c r="S14" s="5" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="T14" s="13" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="U14" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V14" s="17" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="W14" s="17" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="X14" s="17" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="Y14" s="17" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="Z14" s="17" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AA14" s="18">
         <v>8.75</v>
@@ -3066,7 +3028,7 @@
         <v>46280.611111111109</v>
       </c>
       <c r="AF14" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG14" s="17">
         <v>1</v>
@@ -3077,19 +3039,19 @@
         <v>46281.461805555555</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C15" s="13">
         <v>2203110</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="G15" s="10" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -3102,33 +3064,33 @@
         <v>600</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L15" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>7.1999999999999993</v>
       </c>
       <c r="M15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>105</v>
       </c>
       <c r="N15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>20.52</v>
       </c>
       <c r="O15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>125.52</v>
       </c>
       <c r="P15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q15" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>125.52</v>
       </c>
       <c r="R15" s="10" t="str">
@@ -3136,29 +3098,29 @@
         <v>OK</v>
       </c>
       <c r="S15" s="5" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="T15" s="13" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="U15" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V15" s="17" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="W15" s="17" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="X15" s="17" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="Y15" s="17" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="Z15" s="17" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AA15" s="18">
         <v>8.75</v>
@@ -3174,7 +3136,7 @@
         <v>46281.461805555555</v>
       </c>
       <c r="AF15" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG15" s="17">
         <v>1</v>
@@ -3185,19 +3147,19 @@
         <v>46281.638888888891</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C16" s="13">
         <v>2203110</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="G16" s="10" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -3208,33 +3170,33 @@
       </c>
       <c r="I16" s="8"/>
       <c r="J16" s="13" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L16" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>3.05</v>
       </c>
       <c r="M16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>15.5</v>
       </c>
       <c r="N16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>8.69</v>
       </c>
       <c r="O16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>24.189999999999998</v>
       </c>
       <c r="P16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>15.499999999999998</v>
       </c>
       <c r="Q16" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>8.69</v>
       </c>
       <c r="R16" s="10" t="str">
@@ -3242,29 +3204,29 @@
         <v>OK</v>
       </c>
       <c r="S16" s="5" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="T16" s="13" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="U16" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V16" s="17" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="W16" s="17" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="X16" s="17" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="Y16" s="17" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="Z16" s="17" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AA16" s="18">
         <v>3.1</v>
@@ -3280,7 +3242,7 @@
         <v>46281.638888888891</v>
       </c>
       <c r="AF16" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG16" s="17">
         <v>1</v>
@@ -3291,19 +3253,19 @@
         <v>46282.381944444445</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C17" s="13">
         <v>2204521</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="G17" s="10" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -3314,33 +3276,33 @@
       </c>
       <c r="I17" s="8"/>
       <c r="J17" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="L17" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>3.1184999999999996</v>
       </c>
       <c r="M17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>2.25</v>
       </c>
       <c r="N17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>2.96</v>
       </c>
       <c r="O17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>5.21</v>
       </c>
       <c r="P17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>2.96</v>
       </c>
       <c r="Q17" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>2.25</v>
       </c>
       <c r="R17" s="10" t="str">
@@ -3348,29 +3310,29 @@
         <v>OK</v>
       </c>
       <c r="S17" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="T17" s="13" t="s">
         <v>208</v>
-      </c>
-      <c r="T17" s="13" t="s">
-        <v>213</v>
       </c>
       <c r="U17" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V17" s="17" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="W17" s="17" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="X17" s="17" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="Y17" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="Z17" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="AA17" s="18">
         <v>0.09</v>
@@ -3388,7 +3350,7 @@
         <v>46282.381944444445</v>
       </c>
       <c r="AF17" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG17" s="17">
         <v>1</v>
@@ -3399,19 +3361,19 @@
         <v>46282.559027777781</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C18" s="13">
         <v>2204521</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="G18" s="22" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -3422,33 +3384,33 @@
       </c>
       <c r="I18" s="8"/>
       <c r="J18" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L18" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>2.16</v>
       </c>
       <c r="M18" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>2.7</v>
       </c>
       <c r="N18" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>2.0499999999999998</v>
       </c>
       <c r="O18" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>4.75</v>
       </c>
       <c r="P18" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q18" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>4.75</v>
       </c>
       <c r="R18" s="10" t="str">
@@ -3456,29 +3418,29 @@
         <v>OK</v>
       </c>
       <c r="S18" s="5" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="T18" s="13" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="U18" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V18" s="17" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="W18" s="17" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="X18" s="17" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="Y18" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="Z18" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="AA18" s="18">
         <v>0.18</v>
@@ -3496,7 +3458,7 @@
         <v>46282.559027777781</v>
       </c>
       <c r="AF18" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG18" s="17">
         <v>1</v>
@@ -3507,19 +3469,19 @@
         <v>46282.666666666664</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C19" s="13">
         <v>2204521</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G19" s="22" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -3530,33 +3492,33 @@
       </c>
       <c r="I19" s="8"/>
       <c r="J19" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L19" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>10.96</v>
       </c>
       <c r="M19" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>91.2</v>
       </c>
       <c r="N19" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>19.18</v>
       </c>
       <c r="O19" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>110.38</v>
       </c>
       <c r="P19" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q19" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>110.38</v>
       </c>
       <c r="R19" s="10" t="str">
@@ -3564,29 +3526,29 @@
         <v>OK</v>
       </c>
       <c r="S19" s="5" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="T19" s="13" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="U19" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V19" s="17" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="W19" s="17" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="X19" s="17" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="Y19" s="17" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="Z19" s="17" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AA19" s="18">
         <v>11.4</v>
@@ -3602,7 +3564,7 @@
         <v>46282.666666666664</v>
       </c>
       <c r="AF19" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG19" s="17">
         <v>1</v>
@@ -3617,13 +3579,13 @@
         <v>2205077</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="G20" s="22" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -3634,33 +3596,33 @@
       </c>
       <c r="I20" s="8"/>
       <c r="J20" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L20" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>1.83</v>
       </c>
       <c r="M20" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>9.3000000000000007</v>
       </c>
       <c r="N20" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>4.3899999999999997</v>
       </c>
       <c r="O20" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>13.690000000000001</v>
       </c>
       <c r="P20" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q20" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>13.690000000000001</v>
       </c>
       <c r="R20" s="10" t="str">
@@ -3668,29 +3630,29 @@
         <v>OK</v>
       </c>
       <c r="S20" s="5" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="T20" s="13" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="U20" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V20" s="17" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="W20" s="17" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="X20" s="17" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="Y20" s="17" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="Z20" s="17" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AA20" s="18">
         <v>3.1</v>
@@ -3706,7 +3668,7 @@
         <v>46283.427083333336</v>
       </c>
       <c r="AF20" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG20" s="17">
         <v>1</v>
@@ -3717,17 +3679,17 @@
         <v>46283.486111111109</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="13" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="G21" s="22" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -3738,33 +3700,33 @@
       </c>
       <c r="I21" s="8"/>
       <c r="J21" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L21" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>7.4843999999999991</v>
       </c>
       <c r="M21" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>7.2</v>
       </c>
       <c r="N21" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>7.11</v>
       </c>
       <c r="O21" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>14.31</v>
       </c>
       <c r="P21" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q21" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>14.31</v>
       </c>
       <c r="R21" s="10" t="str">
@@ -3772,29 +3734,29 @@
         <v>OK</v>
       </c>
       <c r="S21" s="5" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="T21" s="13" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="U21" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V21" s="17" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="W21" s="17" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="X21" s="17" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="Y21" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="Z21" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="AA21" s="18">
         <v>0.24</v>
@@ -3812,7 +3774,7 @@
         <v>46283.486111111109</v>
       </c>
       <c r="AF21" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG21" s="17">
         <v>1</v>
@@ -3823,19 +3785,19 @@
         <v>46283.638888888891</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C22" s="13">
         <v>2204521</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="G22" s="22" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -3846,33 +3808,33 @@
       </c>
       <c r="I22" s="8"/>
       <c r="J22" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K22" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L22" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>21.34</v>
       </c>
       <c r="M22" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>112</v>
       </c>
       <c r="N22" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>60.82</v>
       </c>
       <c r="O22" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>172.82</v>
       </c>
       <c r="P22" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q22" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>172.82</v>
       </c>
       <c r="R22" s="10" t="str">
@@ -3880,29 +3842,29 @@
         <v>OK</v>
       </c>
       <c r="S22" s="5" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="T22" s="13" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="U22" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V22" s="17" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="W22" s="17" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="X22" s="17" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="Y22" s="17" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="Z22" s="17" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AA22" s="18">
         <v>5.6</v>
@@ -3918,7 +3880,7 @@
         <v>46283.638888888891</v>
       </c>
       <c r="AF22" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG22" s="17">
         <v>1</v>
@@ -3929,19 +3891,19 @@
         <v>46284.34375</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C23" s="13">
         <v>2203110</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="G23" s="22" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -3952,33 +3914,33 @@
       </c>
       <c r="I23" s="8"/>
       <c r="J23" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L23" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>19.982159999999997</v>
       </c>
       <c r="M23" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>16.8</v>
       </c>
       <c r="N23" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>18.98</v>
       </c>
       <c r="O23" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>35.78</v>
       </c>
       <c r="P23" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q23" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>35.78</v>
       </c>
       <c r="R23" s="10" t="str">
@@ -3986,29 +3948,29 @@
         <v>OK</v>
       </c>
       <c r="S23" s="5" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="T23" s="13" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="U23" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v/>
       </c>
       <c r="V23" s="17" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="W23" s="17" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="X23" s="17" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="Y23" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="Z23" s="17" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="AA23" s="18">
         <v>0.42</v>
@@ -4026,7 +3988,7 @@
         <v>46284.34375</v>
       </c>
       <c r="AF23" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG23" s="17">
         <v>1</v>
@@ -4039,13 +4001,13 @@
       <c r="B24" s="12"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="G24" s="22" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
@@ -4058,33 +4020,33 @@
         <v>1200</v>
       </c>
       <c r="J24" s="23" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K24" s="13" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L24" s="24">
         <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Quantity]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Quantity]]))</f>
         <v>14.399999999999999</v>
       </c>
       <c r="M24" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Quantity]]="","",ROUND(tblJobs_MAIN[[#This Row],[Quantity]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>105</v>
       </c>
       <c r="N24" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>41.04</v>
       </c>
       <c r="O24" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>146.04</v>
       </c>
       <c r="P24" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="Q24" s="16">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <f ca="1">IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
         <v>146.04</v>
       </c>
       <c r="R24" s="10" t="str">
@@ -4092,29 +4054,29 @@
         <v>Student name or number required; Print width exceeds stock width</v>
       </c>
       <c r="S24" s="5" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="T24" s="13" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="U24" s="17" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Quantity]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Quantity]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Quantity]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Quantity]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width",""))</f>
         <v>; Student name or number required; Print width exceeds stock width</v>
       </c>
       <c r="V24" s="17" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="W24" s="17" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="X24" s="17" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="Y24" s="17" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="Z24" s="17" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AA24" s="18">
         <v>8.75</v>
@@ -4130,7 +4092,7 @@
         <v>46284.395833333336</v>
       </c>
       <c r="AF24" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="AG24" s="17">
         <v>1</v>
@@ -4180,68 +4142,68 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B6" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B8" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -4272,117 +4234,117 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="H4" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D6" s="9">
         <v>2.85</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F6" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D7" s="9">
         <v>2.4</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D8" s="9">
         <v>0.95</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C9" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D9" s="9">
         <v>1.75</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -4422,79 +4384,79 @@
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="N4" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>113</v>
-      </c>
       <c r="L5" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B6" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E6" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
         <v>Sheet</v>
       </c>
       <c r="F6" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G6" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H6" s="8">
         <v>594</v>
@@ -4506,35 +4468,35 @@
         <v>0.42</v>
       </c>
       <c r="K6" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
       <c r="L6" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E7" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
         <v>Sheet</v>
       </c>
       <c r="F7" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="H7" s="8">
         <v>420</v>
@@ -4546,35 +4508,35 @@
         <v>0.24</v>
       </c>
       <c r="K7" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
       <c r="L7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B8" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E8" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
         <v>Sheet</v>
       </c>
       <c r="F8" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G8" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="H8" s="8">
         <v>320</v>
@@ -4586,35 +4548,35 @@
         <v>0.31</v>
       </c>
       <c r="K8" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
       <c r="L8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B9" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E9" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
         <v>Sheet</v>
       </c>
       <c r="F9" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G9" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="H9" s="8">
         <v>297</v>
@@ -4626,32 +4588,32 @@
         <v>0.09</v>
       </c>
       <c r="K9" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
       <c r="L9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B10" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E10" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
         <v>Roll</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H10" s="8">
         <v>610</v>
@@ -4661,32 +4623,32 @@
         <v>3.1</v>
       </c>
       <c r="K10" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per metre</v>
       </c>
       <c r="L10" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B11" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E11" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
         <v>Roll</v>
       </c>
       <c r="F11" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H11" s="8">
         <v>914</v>
@@ -4696,32 +4658,32 @@
         <v>8.75</v>
       </c>
       <c r="K11" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per metre</v>
       </c>
       <c r="L11" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E12" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
         <v>Roll</v>
       </c>
       <c r="F12" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H12" s="8">
         <v>1370</v>
@@ -4731,32 +4693,32 @@
         <v>11.4</v>
       </c>
       <c r="K12" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per metre</v>
       </c>
       <c r="L12" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B13" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C13" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E13" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
         <v>Roll</v>
       </c>
       <c r="F13" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H13" s="8">
         <v>1067</v>
@@ -4766,32 +4728,32 @@
         <v>5.6</v>
       </c>
       <c r="K13" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per metre</v>
       </c>
       <c r="L13" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B14" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E14" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
         <v>Sheet</v>
       </c>
       <c r="F14" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="H14" s="8">
         <v>320</v>
@@ -4803,11 +4765,11 @@
         <v>0.18</v>
       </c>
       <c r="K14" s="10" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
+        <f ca="1">IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
       <c r="L14" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -4851,28 +4813,28 @@
   <sheetData>
     <row r="1" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -4908,19 +4870,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -4942,7 +4904,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove paper family; Measure is the single Sheet/Roll input
Papers' Family and calculated Measure columns always matched once the width-band families merged. Measure is now a Sheet/Roll dropdown; tblPaperFamilies, S_Family and Summary's Family column are removed. Schema 1.3, app 0.10.3. No migration (no workbooks in the wild).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01EtP3nAP3Yy7UKVWYkX8JFg
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -38,7 +38,6 @@
     <definedName name="LOC_RollUnit" localSheetId="0">'Example Print Room'!$B$6</definedName>
     <definedName name="LOC_Status" localSheetId="0">'Example Print Room'!$AM$5</definedName>
     <definedName name="lstConsumables">tblConsumables[Consumable type]</definedName>
-    <definedName name="lstFamilies">tblPaperFamilies[Family]</definedName>
     <definedName name="lstPaperTypes">tblPaperTypes[Paper type]</definedName>
     <definedName name="lstPrinters">tblPrinters[Model]</definedName>
     <definedName name="lstStandardSizes">tblStandardSizes[Size name]</definedName>
@@ -2205,9 +2204,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_MAIN" displayName="tblJobs_MAIN" ref="A13:AI25" totalsRowShown="0">
-  <autoFilter ref="A13:AI25" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
-  <tableColumns count="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_MAIN" displayName="tblJobs_MAIN" ref="A13:AH25" totalsRowShown="0">
+  <autoFilter ref="A13:AH25" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
+  <tableColumns count="34">
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Date/Time" dataDxfId="82"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="81"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Student No" dataDxfId="80"/>
@@ -2252,7 +2251,6 @@
     <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="59"/>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="58"/>
     <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="57"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0A00-000019000000}" name="S_Family" dataDxfId="56"/>
     <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="55"/>
     <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="54"/>
     <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="53"/>
@@ -2330,16 +2328,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:M17" totalsRowShown="0" dataDxfId="34">
-  <autoFilter ref="A6:M17" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:L17" totalsRowShown="0" dataDxfId="34">
+  <autoFilter ref="A6:L17" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="33"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Description" dataDxfId="32"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Paper type" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Family" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Measure" dataDxfId="29">
-      <calculatedColumnFormula>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</calculatedColumnFormula>
-    </tableColumn>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Measure" dataDxfId="30"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Size mode" dataDxfId="28"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Std. size" dataDxfId="27"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Width mm" dataDxfId="26"/>
@@ -2379,21 +2374,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tblPaperFamilies" displayName="tblPaperFamilies" ref="I5:K7" totalsRowShown="0" dataDxfId="13">
-  <autoFilter ref="I5:K7" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Family" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Measurement basis" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Notes" dataDxfId="10"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="tblStandardSizes" displayName="tblStandardSizes" ref="M5:O11" totalsRowShown="0" dataDxfId="9">
-  <autoFilter ref="M5:O11" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="tblStandardSizes" displayName="tblStandardSizes" ref="I5:K11" totalsRowShown="0" dataDxfId="9">
+  <autoFilter ref="I5:K11" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Size name" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Width mm" dataDxfId="7"/>
@@ -2404,8 +2387,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="tblConsumables" displayName="tblConsumables" ref="Q5:R9" totalsRowShown="0" dataDxfId="5">
-  <autoFilter ref="Q5:R9" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="tblConsumables" displayName="tblConsumables" ref="M5:N9" totalsRowShown="0" dataDxfId="5">
+  <autoFilter ref="M5:N9" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Consumable type" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Active" dataDxfId="3"/>
@@ -2727,20 +2710,19 @@
     <col min="23" max="24" width="11.7265625" hidden="1" customWidth="1"/>
     <col min="25" max="25" width="13.7265625" hidden="1" customWidth="1"/>
     <col min="26" max="26" width="10.7265625" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="12.7265625" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="13.7265625" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="14.7265625" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="12.7265625" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="16.7265625" hidden="1" customWidth="1"/>
-    <col min="32" max="32" width="14.7265625" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="11.7265625" hidden="1" customWidth="1"/>
-    <col min="34" max="34" width="0" hidden="1" customWidth="1" collapsed="1"/>
-    <col min="35" max="35" width="8.7265625" customWidth="1"/>
+    <col min="27" max="27" width="13.7265625" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="14.7265625" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="12.7265625" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="16.7265625" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="14.7265625" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="11.7265625" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="0" hidden="1" customWidth="1" collapsed="1"/>
+    <col min="34" max="34" width="8.7265625" customWidth="1"/>
     <col min="36" max="36" width="29.90625" customWidth="1"/>
     <col min="52" max="52" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>136</v>
       </c>
@@ -2757,7 +2739,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="2" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>19</v>
       </c>
@@ -2774,7 +2756,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="3" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>249</v>
       </c>
@@ -2787,7 +2769,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="4" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>250</v>
       </c>
@@ -2799,7 +2781,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="5" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>251</v>
       </c>
@@ -2811,7 +2793,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="6" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>252</v>
       </c>
@@ -2825,7 +2807,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="7" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>254</v>
       </c>
@@ -2840,7 +2822,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="8" x14ac:dyDescent="0.35">
       <c r="A8" s="30" t="s">
         <v>255</v>
       </c>
@@ -2852,7 +2834,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="11" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="11" x14ac:dyDescent="0.35">
       <c r="A11" s="32"/>
       <c r="C11" s="32"/>
       <c r="E11" s="32"/>
@@ -2861,7 +2843,7 @@
       <c r="K11" s="32"/>
       <c r="M11" s="2"/>
     </row>
-    <row r="13" spans="1:52" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>149</v>
       </c>
@@ -2941,34 +2923,31 @@
         <v>168</v>
       </c>
       <c r="AA13" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AB13" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AC13" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AD13" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="AE13" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AF13" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AG13" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AH13" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="AI13" s="4" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="14" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="14" x14ac:dyDescent="0.35">
       <c r="A14" s="11">
         <v>46280.425000000003</v>
       </c>
@@ -3053,32 +3032,29 @@
       <c r="AA14" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="AB14" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="AC14" s="17">
+      <c r="AB14" s="17">
         <v>0.31</v>
       </c>
+      <c r="AC14" s="16">
+        <v>320</v>
+      </c>
       <c r="AD14" s="16">
-        <v>320</v>
-      </c>
-      <c r="AE14" s="16">
         <v>450</v>
       </c>
-      <c r="AF14" s="17">
+      <c r="AE14" s="17">
         <v>0.95</v>
       </c>
-      <c r="AG14" s="16">
+      <c r="AF14" s="16">
         <v>46280.425000000003</v>
       </c>
-      <c r="AH14" s="16" t="s">
+      <c r="AG14" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI14" s="16">
+      <c r="AH14" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="15" x14ac:dyDescent="0.35">
       <c r="A15" s="11">
         <v>46280.611111111109</v>
       </c>
@@ -3161,32 +3137,29 @@
         <v>77</v>
       </c>
       <c r="AA15" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB15" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="AC15" s="17">
+      <c r="AB15" s="17">
         <v>8.75</v>
       </c>
-      <c r="AD15" s="16">
+      <c r="AC15" s="16">
         <v>914</v>
       </c>
-      <c r="AE15" s="16"/>
-      <c r="AF15" s="17">
+      <c r="AD15" s="16"/>
+      <c r="AE15" s="17">
         <v>2.85</v>
       </c>
-      <c r="AG15" s="16">
+      <c r="AF15" s="16">
         <v>46280.611111111109</v>
       </c>
-      <c r="AH15" s="16" t="s">
+      <c r="AG15" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI15" s="16">
+      <c r="AH15" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="16" x14ac:dyDescent="0.35">
       <c r="A16" s="11">
         <v>46281.461805555555</v>
       </c>
@@ -3271,32 +3244,29 @@
         <v>77</v>
       </c>
       <c r="AA16" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB16" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="AC16" s="17">
+      <c r="AB16" s="17">
         <v>8.75</v>
       </c>
-      <c r="AD16" s="16">
+      <c r="AC16" s="16">
         <v>914</v>
       </c>
-      <c r="AE16" s="16"/>
-      <c r="AF16" s="17">
+      <c r="AD16" s="16"/>
+      <c r="AE16" s="17">
         <v>2.85</v>
       </c>
-      <c r="AG16" s="16">
+      <c r="AF16" s="16">
         <v>46281.461805555555</v>
       </c>
-      <c r="AH16" s="16" t="s">
+      <c r="AG16" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI16" s="16">
+      <c r="AH16" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="17" x14ac:dyDescent="0.35">
       <c r="A17" s="11">
         <v>46281.638888888891</v>
       </c>
@@ -3379,32 +3349,29 @@
         <v>75</v>
       </c>
       <c r="AA17" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="AB17" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="AC17" s="17">
+      <c r="AB17" s="17">
         <v>3.1</v>
       </c>
-      <c r="AD17" s="16">
+      <c r="AC17" s="16">
         <v>610</v>
       </c>
-      <c r="AE17" s="16"/>
-      <c r="AF17" s="17">
+      <c r="AD17" s="16"/>
+      <c r="AE17" s="17">
         <v>2.85</v>
       </c>
-      <c r="AG17" s="16">
+      <c r="AF17" s="16">
         <v>46281.638888888891</v>
       </c>
-      <c r="AH17" s="16" t="s">
+      <c r="AG17" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI17" s="16">
+      <c r="AH17" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="18" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
         <v>46282.381944444445</v>
       </c>
@@ -3489,32 +3456,29 @@
       <c r="AA18" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="AB18" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="AC18" s="17">
+      <c r="AB18" s="17">
         <v>0.09</v>
       </c>
+      <c r="AC18" s="16">
+        <v>297</v>
+      </c>
       <c r="AD18" s="16">
-        <v>297</v>
-      </c>
-      <c r="AE18" s="16">
         <v>420</v>
       </c>
-      <c r="AF18" s="17">
+      <c r="AE18" s="17">
         <v>0.95</v>
       </c>
-      <c r="AG18" s="16">
+      <c r="AF18" s="16">
         <v>46282.381944444445</v>
       </c>
-      <c r="AH18" s="16" t="s">
+      <c r="AG18" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI18" s="16">
+      <c r="AH18" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="19" x14ac:dyDescent="0.35">
       <c r="A19" s="11">
         <v>46282.559027777781</v>
       </c>
@@ -3599,32 +3563,29 @@
       <c r="AA19" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="AB19" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="AC19" s="17">
+      <c r="AB19" s="17">
         <v>0.18</v>
       </c>
+      <c r="AC19" s="16">
+        <v>320</v>
+      </c>
       <c r="AD19" s="16">
-        <v>320</v>
-      </c>
-      <c r="AE19" s="16">
         <v>450</v>
       </c>
-      <c r="AF19" s="17">
+      <c r="AE19" s="17">
         <v>0.95</v>
       </c>
-      <c r="AG19" s="16">
+      <c r="AF19" s="16">
         <v>46282.559027777781</v>
       </c>
-      <c r="AH19" s="16" t="s">
+      <c r="AG19" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI19" s="16">
+      <c r="AH19" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="20" x14ac:dyDescent="0.35">
       <c r="A20" s="11">
         <v>46282.666666666664</v>
       </c>
@@ -3707,32 +3668,29 @@
         <v>77</v>
       </c>
       <c r="AA20" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB20" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="AC20" s="17">
+      <c r="AB20" s="17">
         <v>11.4</v>
       </c>
-      <c r="AD20" s="16">
+      <c r="AC20" s="16">
         <v>1370</v>
       </c>
-      <c r="AE20" s="16"/>
-      <c r="AF20" s="17">
+      <c r="AD20" s="16"/>
+      <c r="AE20" s="17">
         <v>1.75</v>
       </c>
-      <c r="AG20" s="16">
+      <c r="AF20" s="16">
         <v>46282.666666666664</v>
       </c>
-      <c r="AH20" s="16" t="s">
+      <c r="AG20" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI20" s="16">
+      <c r="AH20" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="21" x14ac:dyDescent="0.35">
       <c r="A21" s="11">
         <v>46283.427083333336</v>
       </c>
@@ -3813,32 +3771,29 @@
         <v>75</v>
       </c>
       <c r="AA21" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="AB21" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="AC21" s="17">
+      <c r="AB21" s="17">
         <v>3.1</v>
       </c>
-      <c r="AD21" s="16">
+      <c r="AC21" s="16">
         <v>610</v>
       </c>
-      <c r="AE21" s="16"/>
-      <c r="AF21" s="17">
+      <c r="AD21" s="16"/>
+      <c r="AE21" s="17">
         <v>2.4</v>
       </c>
-      <c r="AG21" s="16">
+      <c r="AF21" s="16">
         <v>46283.427083333336</v>
       </c>
-      <c r="AH21" s="16" t="s">
+      <c r="AG21" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI21" s="16">
+      <c r="AH21" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="22" x14ac:dyDescent="0.35">
       <c r="A22" s="11">
         <v>46283.486111111109</v>
       </c>
@@ -3921,32 +3876,29 @@
       <c r="AA22" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="AB22" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="AC22" s="17">
+      <c r="AB22" s="17">
         <v>0.24</v>
       </c>
+      <c r="AC22" s="16">
+        <v>420</v>
+      </c>
       <c r="AD22" s="16">
-        <v>420</v>
-      </c>
-      <c r="AE22" s="16">
         <v>594</v>
       </c>
-      <c r="AF22" s="17">
+      <c r="AE22" s="17">
         <v>0.95</v>
       </c>
-      <c r="AG22" s="16">
+      <c r="AF22" s="16">
         <v>46283.486111111109</v>
       </c>
-      <c r="AH22" s="16" t="s">
+      <c r="AG22" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI22" s="16">
+      <c r="AH22" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="23" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
         <v>46283.638888888891</v>
       </c>
@@ -4029,32 +3981,29 @@
         <v>77</v>
       </c>
       <c r="AA23" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB23" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="AC23" s="17">
+      <c r="AB23" s="17">
         <v>5.6</v>
       </c>
-      <c r="AD23" s="16">
+      <c r="AC23" s="16">
         <v>1067</v>
       </c>
-      <c r="AE23" s="16"/>
-      <c r="AF23" s="17">
+      <c r="AD23" s="16"/>
+      <c r="AE23" s="17">
         <v>2.85</v>
       </c>
-      <c r="AG23" s="16">
+      <c r="AF23" s="16">
         <v>46283.638888888891</v>
       </c>
-      <c r="AH23" s="16" t="s">
+      <c r="AG23" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI23" s="16">
+      <c r="AH23" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="24" x14ac:dyDescent="0.35">
       <c r="A24" s="11">
         <v>46284.34375</v>
       </c>
@@ -4139,32 +4088,29 @@
       <c r="AA24" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="AB24" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="AC24" s="17">
+      <c r="AB24" s="17">
         <v>0.42</v>
       </c>
+      <c r="AC24" s="16">
+        <v>594</v>
+      </c>
       <c r="AD24" s="16">
-        <v>594</v>
-      </c>
-      <c r="AE24" s="16">
         <v>841</v>
       </c>
-      <c r="AF24" s="17">
+      <c r="AE24" s="17">
         <v>0.95</v>
       </c>
-      <c r="AG24" s="16">
+      <c r="AF24" s="16">
         <v>46284.34375</v>
       </c>
-      <c r="AH24" s="16" t="s">
+      <c r="AG24" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI24" s="16">
+      <c r="AH24" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="25" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
         <v>46284.395833333336</v>
       </c>
@@ -4245,28 +4191,25 @@
         <v>75</v>
       </c>
       <c r="AA25" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB25" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="AC25" s="17">
+      <c r="AB25" s="17">
         <v>8.75</v>
       </c>
-      <c r="AD25" s="16">
+      <c r="AC25" s="16">
         <v>914</v>
       </c>
-      <c r="AE25" s="16"/>
-      <c r="AF25" s="17">
+      <c r="AD25" s="16"/>
+      <c r="AE25" s="17">
         <v>2.85</v>
       </c>
-      <c r="AG25" s="16">
+      <c r="AF25" s="16">
         <v>46284.395833333336</v>
       </c>
-      <c r="AH25" s="16" t="s">
+      <c r="AG25" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="AI25" s="16">
+      <c r="AH25" s="16">
         <v>1</v>
       </c>
     </row>
@@ -4718,39 +4661,37 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.7265625" customWidth="1"/>
     <col min="2" max="2" width="34.7265625" customWidth="1"/>
-    <col min="3" max="4" width="14.7265625" customWidth="1"/>
-    <col min="5" max="5" width="10.7265625" customWidth="1"/>
-    <col min="6" max="6" width="14.7265625" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" customWidth="1"/>
-    <col min="8" max="10" width="10.7265625" customWidth="1"/>
-    <col min="11" max="11" width="14.7265625" customWidth="1"/>
-    <col min="12" max="12" width="9.7265625" customWidth="1"/>
+    <col min="3" max="5" width="14.7265625" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" customWidth="1"/>
+    <col min="7" max="9" width="10.7265625" customWidth="1"/>
+    <col min="10" max="10" width="14.7265625" customWidth="1"/>
+    <col min="11" max="11" width="9.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="N4" s="2" t="s">
+    <row r="4" x14ac:dyDescent="0.35">
+      <c r="M4" s="2" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="N5" s="2"/>
-    </row>
-    <row r="6" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" x14ac:dyDescent="0.35">
+      <c r="M5" s="2"/>
+    </row>
+    <row r="6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>97</v>
       </c>
@@ -4761,37 +4702,34 @@
         <v>35</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>45</v>
+        <v>99</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>100</v>
+        <v>237</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>237</v>
+        <v>55</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="L6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="M6" s="22" t="s">
+      <c r="L6" s="22" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" x14ac:dyDescent="0.35">
       <c r="A7" s="33" t="s">
         <v>103</v>
       </c>
@@ -4804,37 +4742,33 @@
       <c r="D7" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Sheet</v>
+      <c r="E7" s="27" t="s">
+        <v>105</v>
       </c>
       <c r="F7" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="G7" s="27" t="s">
         <v>58</v>
       </c>
+      <c r="G7" s="8">
+        <v>594</v>
+      </c>
       <c r="H7" s="8">
-        <v>594</v>
-      </c>
-      <c r="I7" s="8">
         <v>841</v>
       </c>
-      <c r="J7" s="10">
+      <c r="I7" s="10">
         <v>0.42</v>
       </c>
-      <c r="K7" s="20" t="str">
+      <c r="J7" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
-      <c r="L7" s="27" t="s">
+      <c r="K7" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M7" s="28" t="s">
+      <c r="L7" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" x14ac:dyDescent="0.35">
       <c r="A8" s="33" t="s">
         <v>106</v>
       </c>
@@ -4847,37 +4781,33 @@
       <c r="D8" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Sheet</v>
+      <c r="E8" s="27" t="s">
+        <v>105</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="G8" s="27" t="s">
         <v>59</v>
       </c>
+      <c r="G8" s="8">
+        <v>420</v>
+      </c>
       <c r="H8" s="8">
-        <v>420</v>
-      </c>
-      <c r="I8" s="8">
         <v>594</v>
       </c>
-      <c r="J8" s="10">
+      <c r="I8" s="10">
         <v>0.24</v>
       </c>
-      <c r="K8" s="20" t="str">
+      <c r="J8" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
-      <c r="L8" s="27" t="s">
+      <c r="K8" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M8" s="28" t="s">
+      <c r="L8" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" x14ac:dyDescent="0.35">
       <c r="A9" s="33" t="s">
         <v>108</v>
       </c>
@@ -4890,37 +4820,33 @@
       <c r="D9" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Sheet</v>
+      <c r="E9" s="27" t="s">
+        <v>105</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="G9" s="27" t="s">
         <v>62</v>
       </c>
+      <c r="G9" s="8">
+        <v>320</v>
+      </c>
       <c r="H9" s="8">
-        <v>320</v>
-      </c>
-      <c r="I9" s="8">
         <v>450</v>
       </c>
-      <c r="J9" s="10">
+      <c r="I9" s="10">
         <v>0.31</v>
       </c>
-      <c r="K9" s="20" t="str">
+      <c r="J9" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
-      <c r="L9" s="27" t="s">
+      <c r="K9" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M9" s="28" t="s">
+      <c r="L9" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" x14ac:dyDescent="0.35">
       <c r="A10" s="33" t="s">
         <v>110</v>
       </c>
@@ -4933,37 +4859,33 @@
       <c r="D10" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Sheet</v>
+      <c r="E10" s="27" t="s">
+        <v>105</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="G10" s="27" t="s">
         <v>60</v>
       </c>
+      <c r="G10" s="8">
+        <v>297</v>
+      </c>
       <c r="H10" s="8">
-        <v>297</v>
-      </c>
-      <c r="I10" s="8">
         <v>420</v>
       </c>
-      <c r="J10" s="10">
+      <c r="I10" s="10">
         <v>0.09</v>
       </c>
-      <c r="K10" s="20" t="str">
+      <c r="J10" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
-      <c r="L10" s="27" t="s">
+      <c r="K10" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M10" s="28" t="s">
+      <c r="L10" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" x14ac:dyDescent="0.35">
       <c r="A11" s="33" t="s">
         <v>112</v>
       </c>
@@ -4976,33 +4898,29 @@
       <c r="D11" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="E11" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Roll</v>
-      </c>
-      <c r="F11" s="27" t="s">
+      <c r="E11" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="27"/>
-      <c r="H11" s="8">
+      <c r="F11" s="27"/>
+      <c r="G11" s="8">
         <v>610</v>
       </c>
-      <c r="I11" s="8"/>
-      <c r="J11" s="10">
+      <c r="H11" s="8"/>
+      <c r="I11" s="10">
         <v>3.1</v>
       </c>
-      <c r="K11" s="20" t="str">
+      <c r="J11" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per metre</v>
       </c>
-      <c r="L11" s="27" t="s">
+      <c r="K11" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M11" s="28" t="s">
+      <c r="L11" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" x14ac:dyDescent="0.35">
       <c r="A12" s="33" t="s">
         <v>114</v>
       </c>
@@ -5015,33 +4933,29 @@
       <c r="D12" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Roll</v>
-      </c>
-      <c r="F12" s="27" t="s">
+      <c r="E12" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="27"/>
-      <c r="H12" s="8">
+      <c r="F12" s="27"/>
+      <c r="G12" s="8">
         <v>914</v>
       </c>
-      <c r="I12" s="8"/>
-      <c r="J12" s="10">
+      <c r="H12" s="8"/>
+      <c r="I12" s="10">
         <v>8.75</v>
       </c>
-      <c r="K12" s="20" t="str">
+      <c r="J12" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per metre</v>
       </c>
-      <c r="L12" s="27" t="s">
+      <c r="K12" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M12" s="28" t="s">
+      <c r="L12" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" x14ac:dyDescent="0.35">
       <c r="A13" s="33" t="s">
         <v>116</v>
       </c>
@@ -5054,33 +4968,29 @@
       <c r="D13" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="E13" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Roll</v>
-      </c>
-      <c r="F13" s="27" t="s">
+      <c r="E13" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="27"/>
-      <c r="H13" s="8">
+      <c r="F13" s="27"/>
+      <c r="G13" s="8">
         <v>1370</v>
       </c>
-      <c r="I13" s="8"/>
-      <c r="J13" s="10">
+      <c r="H13" s="8"/>
+      <c r="I13" s="10">
         <v>11.4</v>
       </c>
-      <c r="K13" s="20" t="str">
+      <c r="J13" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per metre</v>
       </c>
-      <c r="L13" s="27" t="s">
+      <c r="K13" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M13" s="28" t="s">
+      <c r="L13" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" x14ac:dyDescent="0.35">
       <c r="A14" s="33" t="s">
         <v>118</v>
       </c>
@@ -5093,33 +5003,29 @@
       <c r="D14" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Roll</v>
-      </c>
-      <c r="F14" s="27" t="s">
+      <c r="E14" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="G14" s="27"/>
-      <c r="H14" s="8">
+      <c r="F14" s="27"/>
+      <c r="G14" s="8">
         <v>1067</v>
       </c>
-      <c r="I14" s="8"/>
-      <c r="J14" s="10">
+      <c r="H14" s="8"/>
+      <c r="I14" s="10">
         <v>5.6</v>
       </c>
-      <c r="K14" s="20" t="str">
+      <c r="J14" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per metre</v>
       </c>
-      <c r="L14" s="27" t="s">
+      <c r="K14" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M14" s="28" t="s">
+      <c r="L14" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" x14ac:dyDescent="0.35">
       <c r="A15" s="33" t="s">
         <v>120</v>
       </c>
@@ -5132,35 +5038,31 @@
       <c r="D15" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="E15" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Sheet</v>
-      </c>
-      <c r="F15" s="27" t="s">
+      <c r="E15" s="27" t="s">
         <v>122</v>
       </c>
-      <c r="G15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="8">
+        <v>320</v>
+      </c>
       <c r="H15" s="8">
-        <v>320</v>
-      </c>
-      <c r="I15" s="8">
         <v>450</v>
       </c>
-      <c r="J15" s="10">
+      <c r="I15" s="10">
         <v>0.18</v>
       </c>
-      <c r="K15" s="20" t="str">
+      <c r="J15" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
-      <c r="L15" s="27" t="s">
+      <c r="K15" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M15" s="28" t="s">
+      <c r="L15" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" x14ac:dyDescent="0.35">
       <c r="A16" s="33" t="s">
         <v>242</v>
       </c>
@@ -5173,29 +5075,25 @@
       <c r="D16" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="E16" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Roll</v>
-      </c>
+      <c r="E16" s="27"/>
       <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
+      <c r="G16" s="8"/>
       <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="10">
+      <c r="I16" s="10">
         <v>0</v>
       </c>
-      <c r="K16" s="20" t="str">
+      <c r="J16" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per metre</v>
       </c>
-      <c r="L16" s="27" t="s">
+      <c r="K16" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M16" s="28" t="s">
+      <c r="L16" s="28" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" x14ac:dyDescent="0.35">
       <c r="A17" s="33" t="s">
         <v>245</v>
       </c>
@@ -5208,56 +5106,52 @@
       <c r="D17" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Family]]="","",IFERROR(INDEX(tblPaperFamilies[Measurement basis],MATCH(tblPapers[[#This Row],[Family]],tblPaperFamilies[Family],0)),"?"))</f>
-        <v>Sheet</v>
-      </c>
+      <c r="E17" s="27"/>
       <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
+      <c r="G17" s="8"/>
       <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="10">
+      <c r="I17" s="10">
         <v>0</v>
       </c>
-      <c r="K17" s="20" t="str">
+      <c r="J17" s="20" t="str">
         <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
         <v>£ per sheet</v>
       </c>
-      <c r="L17" s="27" t="s">
+      <c r="K17" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M17" s="28" t="s">
+      <c r="L17" s="28" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Supplied by student" error="Choose Yes or No." promptTitle="Supplied by student" prompt="Yes only for the two 'Supplied' catalogue rows - paper cost always computes to zero for these regardless of Cost." sqref="M7:M17" xr:uid="{2ED70CBA-D9C3-4CB5-A147-78652DAACDC7}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Supplied by student" error="Choose Yes or No." promptTitle="Supplied by student" prompt="Yes only for the two 'Supplied' catalogue rows - paper cost always computes to zero for these regardless of Cost." sqref="L7:L17" xr:uid="{2ED70CBA-D9C3-4CB5-A147-78652DAACDC7}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C2003" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>lstPaperTypes</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper family" error="The family decides whether this stock is measured in sheets or metres, and which printers can use it." promptTitle="Paper family" prompt="The family decides whether this stock is measured in sheets or metres, and which printers can use it." sqref="D7:D2003" xr:uid="{00000000-0002-0000-0300-000001000000}">
-      <formula1>lstFamilies</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Measure" error="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." promptTitle="Measure" prompt="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." sqref="D7:D2003" xr:uid="{00000000-0002-0000-0300-000001000000}">
+      <formula1>"Sheet,Roll"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Size mode" error="Standard fills the size from the standard sizes list. Custom sheet takes width and height directly. Roll takes the roll width only." promptTitle="Size mode" prompt="Standard fills the size from the standard sizes list. Custom sheet takes width and height directly. Roll takes the roll width only." sqref="F7:F2003" xr:uid="{00000000-0002-0000-0300-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Size mode" error="Standard fills the size from the standard sizes list. Custom sheet takes width and height directly. Roll takes the roll width only." promptTitle="Size mode" prompt="Standard fills the size from the standard sizes list. Custom sheet takes width and height directly. Roll takes the roll width only." sqref="E7:E2003" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>"Standard,Custom sheet,Roll"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G7:G2003" xr:uid="{00000000-0002-0000-0300-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7:F2003" xr:uid="{00000000-0002-0000-0300-000003000000}">
       <formula1>lstStandardSizes</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres. For roll stock, enter the roll width only." promptTitle="Dimension" prompt="Enter the size in millimetres. For roll stock, enter the roll width only." sqref="H7:H2003" xr:uid="{00000000-0002-0000-0300-000004000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres. For roll stock, enter the roll width only." promptTitle="Dimension" prompt="Enter the size in millimetres. For roll stock, enter the roll width only." sqref="G7:G2003" xr:uid="{00000000-0002-0000-0300-000004000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres." promptTitle="Dimension" prompt="Enter the size in millimetres." sqref="I7:I2003" xr:uid="{00000000-0002-0000-0300-000005000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres." promptTitle="Dimension" prompt="Enter the size in millimetres." sqref="H7:H2003" xr:uid="{00000000-0002-0000-0300-000005000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Cost" error="Cost per sheet for sheet stock, or cost per metre for roll stock. The Cost unit column shows which applies." promptTitle="Cost" prompt="Cost per sheet for sheet stock, or cost per metre for roll stock. The Cost unit column shows which applies." sqref="J7:J2003" xr:uid="{00000000-0002-0000-0300-000006000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Cost" error="Cost per sheet for sheet stock, or cost per metre for roll stock. The Cost unit column shows which applies." promptTitle="Cost" prompt="Cost per sheet for sheet stock, or cost per metre for roll stock. The Cost unit column shows which applies." sqref="I7:I2003" xr:uid="{00000000-0002-0000-0300-000006000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L7:L2003" xr:uid="{00000000-0002-0000-0300-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K7:K2003" xr:uid="{00000000-0002-0000-0300-000007000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5271,7 +5165,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
@@ -5280,35 +5174,32 @@
     <col min="4" max="4" width="60.7265625" customWidth="1"/>
     <col min="6" max="6" width="22.7265625" customWidth="1"/>
     <col min="7" max="7" width="9.7265625" customWidth="1"/>
-    <col min="9" max="9" width="16.7265625" customWidth="1"/>
-    <col min="10" max="10" width="20.7265625" customWidth="1"/>
-    <col min="11" max="11" width="46.7265625" customWidth="1"/>
-    <col min="13" max="13" width="12.7265625" customWidth="1"/>
-    <col min="14" max="15" width="11.7265625" customWidth="1"/>
-    <col min="17" max="17" width="18.7265625" customWidth="1"/>
-    <col min="18" max="18" width="9.7265625" customWidth="1"/>
-    <col min="20" max="20" width="20.7265625" customWidth="1"/>
+    <col min="9" max="9" width="12.7265625" customWidth="1"/>
+    <col min="10" max="11" width="11.7265625" customWidth="1"/>
+    <col min="13" max="13" width="18.7265625" customWidth="1"/>
+    <col min="14" max="14" width="9.7265625" customWidth="1"/>
+    <col min="16" max="16" width="20.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="T3" s="2" t="s">
+    <row r="3" x14ac:dyDescent="0.35">
+      <c r="P3" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -5316,16 +5207,13 @@
         <v>34</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q4" s="3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
@@ -5345,31 +5233,22 @@
         <v>36</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q5" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="R5" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
@@ -5389,31 +5268,22 @@
         <v>38</v>
       </c>
       <c r="I6" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="J6" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="K6" s="27" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="J6" s="8">
+        <v>841</v>
+      </c>
+      <c r="K6" s="8">
+        <v>1189</v>
       </c>
       <c r="M6" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="N6" s="8">
-        <v>841</v>
-      </c>
-      <c r="O6" s="8">
-        <v>1189</v>
-      </c>
-      <c r="Q6" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="R6" s="27" t="s">
+      <c r="N6" s="27" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="7" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>11</v>
       </c>
@@ -5431,31 +5301,22 @@
         <v>38</v>
       </c>
       <c r="I7" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="J7" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="K7" s="27" t="s">
-        <v>51</v>
+        <v>58</v>
+      </c>
+      <c r="J7" s="8">
+        <v>594</v>
+      </c>
+      <c r="K7" s="8">
+        <v>841</v>
       </c>
       <c r="M7" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="N7" s="8">
-        <v>594</v>
-      </c>
-      <c r="O7" s="8">
-        <v>841</v>
-      </c>
-      <c r="Q7" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="R7" s="27" t="s">
+      <c r="N7" s="27" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="8" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>14</v>
       </c>
@@ -5474,23 +5335,23 @@
       <c r="G8" s="27" t="s">
         <v>38</v>
       </c>
+      <c r="I8" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="J8" s="8">
+        <v>420</v>
+      </c>
+      <c r="K8" s="8">
+        <v>594</v>
+      </c>
       <c r="M8" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="N8" s="8">
-        <v>420</v>
-      </c>
-      <c r="O8" s="8">
-        <v>594</v>
-      </c>
-      <c r="Q8" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="R8" s="27" t="s">
+      <c r="N8" s="27" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="9" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>18</v>
       </c>
@@ -5507,23 +5368,23 @@
       <c r="G9" s="27" t="s">
         <v>38</v>
       </c>
+      <c r="I9" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="J9" s="8">
+        <v>297</v>
+      </c>
+      <c r="K9" s="8">
+        <v>420</v>
+      </c>
       <c r="M9" s="27" t="s">
-        <v>60</v>
-      </c>
-      <c r="N9" s="8">
-        <v>297</v>
-      </c>
-      <c r="O9" s="8">
-        <v>420</v>
-      </c>
-      <c r="Q9" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="R9" s="27" t="s">
+      <c r="N9" s="27" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>21</v>
       </c>
@@ -5542,17 +5403,17 @@
       <c r="G10" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M10" s="27" t="s">
+      <c r="I10" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="N10" s="8">
+      <c r="J10" s="8">
         <v>210</v>
       </c>
-      <c r="O10" s="8">
+      <c r="K10" s="8">
         <v>297</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="11" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>25</v>
       </c>
@@ -5571,17 +5432,17 @@
       <c r="G11" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="M11" s="27" t="s">
+      <c r="I11" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="N11" s="8">
+      <c r="J11" s="8">
         <v>320</v>
       </c>
-      <c r="O11" s="8">
+      <c r="K11" s="8">
         <v>450</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="12" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>28</v>
       </c>
@@ -5595,7 +5456,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="13" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>31</v>
       </c>
@@ -5609,7 +5470,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="14" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>214</v>
       </c>
@@ -5623,7 +5484,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="15" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>217</v>
       </c>
@@ -5637,7 +5498,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="16" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>220</v>
       </c>
@@ -5651,7 +5512,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="17" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>224</v>
       </c>
@@ -5663,7 +5524,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>227</v>
       </c>
@@ -5677,7 +5538,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="19" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>230</v>
       </c>
@@ -5691,7 +5552,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>234</v>
       </c>
@@ -5707,22 +5568,18 @@
     </row>
   </sheetData>
   <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G6:G2000 R6:R2000" xr:uid="{00000000-0002-0000-0000-000001000000}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G6:G2000 N6:N2000" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres." promptTitle="Dimension" prompt="Enter the size in millimetres." sqref="N6:O2000" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres." promptTitle="Dimension" prompt="Enter the size in millimetres." sqref="J6:K2000" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Measurement basis" error="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." promptTitle="Measurement basis" prompt="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." sqref="J6:J1999" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>"Sheet,Roll"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="5">
+  <tableParts count="4">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
   </tableParts>

</xml_diff>

<commit_message>
Fix number formats, dropdown range and column widths on Printers/Papers
- Printers: Cost per m2 now GBP 2dp; Max roll width mm #,##0; Max sheet
  size General (currency format had smeared onto both, in cells and in
  the tblPrinters column dxfs).
- Printers: Yes/No dropdown moved from F11:F2001 to G7:G2001 (Active).
- Column widths tidied on Printers and Papers.
- CHANGELOG entry added.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QY4SDmfhp22Z4nSruXi2Ga
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -1147,7 +1147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1294,6 +1294,22 @@
     <xf numFmtId="22" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1561,7 +1577,7 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1580,7 +1596,7 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -1599,7 +1615,7 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
       <border outline="0">
         <left style="medium">
           <color rgb="FFBFBFBF"/>
@@ -4502,8 +4518,9 @@
     <col min="2" max="2" width="30.7265625" customWidth="1"/>
     <col min="3" max="3" width="17.7265625" customWidth="1"/>
     <col min="4" max="4" width="13.7265625" customWidth="1"/>
-    <col min="5" max="5" width="34.7265625" customWidth="1"/>
-    <col min="6" max="6" width="9.7265625" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" customWidth="1"/>
+    <col min="6" max="6" width="14.7265625" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
@@ -4557,13 +4574,13 @@
       <c r="C7" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="47">
         <v>2.85</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="48">
         <v>1370</v>
       </c>
-      <c r="F7" s="26"/>
+      <c r="F7" s="50"/>
       <c r="G7" s="27" t="s">
         <v>38</v>
       </c>
@@ -4578,13 +4595,13 @@
       <c r="C8" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="47">
         <v>2.4</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="49">
         <v>610</v>
       </c>
-      <c r="F8" s="26"/>
+      <c r="F8" s="50"/>
       <c r="G8" s="27" t="s">
         <v>38</v>
       </c>
@@ -4599,11 +4616,11 @@
       <c r="C9" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="47">
         <v>0.95</v>
       </c>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26" t="s">
+      <c r="E9" s="49"/>
+      <c r="F9" s="50" t="s">
         <v>58</v>
       </c>
       <c r="G9" s="27" t="s">
@@ -4620,13 +4637,13 @@
       <c r="C10" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="23">
+      <c r="D10" s="47">
         <v>1.75</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="49">
         <v>1370</v>
       </c>
-      <c r="F10" s="26"/>
+      <c r="F10" s="50"/>
       <c r="G10" s="27" t="s">
         <v>38</v>
       </c>
@@ -4641,7 +4658,7 @@
     <dataValidation type="decimal" operator="greaterThanOrEqual" showInputMessage="1" showErrorMessage="1" errorTitle="Consumable cost" error="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." promptTitle="Consumable cost" prompt="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." sqref="D7:D2001" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F11:F2001 G7:G10" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G7:G2001" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Max roll width mm" error="Enter 0 or more, in millimetres." promptTitle="Max roll width mm" prompt="The widest roll stock this printer can take, in millimetres. Leave blank if this printer cannot print on roll stock." sqref="E7:E10" xr:uid="{C0A2668E-6A17-4354-874C-F8907F30987B}">
@@ -4664,13 +4681,18 @@
   <dimension ref="A1:M17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" customWidth="1"/>
+    <col min="1" max="1" width="15.7265625" customWidth="1"/>
     <col min="2" max="2" width="34.7265625" customWidth="1"/>
-    <col min="3" max="5" width="14.7265625" customWidth="1"/>
-    <col min="6" max="6" width="13.7265625" customWidth="1"/>
-    <col min="7" max="9" width="10.7265625" customWidth="1"/>
+    <col min="3" max="3" width="17.7265625" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="8" max="8" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="10.7265625" customWidth="1"/>
     <col min="10" max="10" width="14.7265625" customWidth="1"/>
     <col min="11" max="11" width="9.7265625" customWidth="1"/>
+    <col min="12" max="12" width="14.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Drop EnsureCatalogIdSettings; trim InitialiseWorkbook's per-sheet loop
EnsureCatalogIdSettings is removed: no workbook in the wild predates catalogue IDs, so the three counter rows (TECH_ID_HWM, PRINTER_ID_HWM, STOCK_ID_HWM) now ship in PrintCosts.xlsx with their SET_ names, like the other settings. SetCatalogHwm no longer re-seeds a missing counter.

InitialiseWorkbook's location loop no longer repeats the steps RefreshLocations (which ends the run) already performs per sheet: defaults, roll unit, printers/job-count display, below-table validation, BindColumns, reduced view, cost columns, and the final RepositionLocationButtons. Column widths now precede the view/visibility pass instead of following it.

32/32 tests pass (3 via the runner's retry).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\pj-exp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23F7D237-0C1E-419A-BA9C-9AF4DD2F3A50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30789ADB-78C4-4CF3-BB63-90FD3435BBB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,10 +55,13 @@
     <definedName name="SET_LOC_REDUCED_COLUMNS">Settings!$C$19</definedName>
     <definedName name="SET_LOC_REDUCED_VIEW">Settings!$C$18</definedName>
     <definedName name="SET_ORG">Settings!$C$8</definedName>
+    <definedName name="SET_PRINTER_ID_HWM">Settings!$C$22</definedName>
     <definedName name="SET_ROUND_DP">Settings!$C$11</definedName>
     <definedName name="SET_SCHEMA">Settings!$C$12</definedName>
     <definedName name="SET_SITE_ID">Settings!$C$6</definedName>
     <definedName name="SET_SITE_NAME">Settings!$C$7</definedName>
+    <definedName name="SET_STOCK_ID_HWM">Settings!$C$23</definedName>
+    <definedName name="SET_TECH_ID_HWM">Settings!$C$21</definedName>
   </definedNames>
   <calcPr calcId="191029" calcOnSave="0"/>
   <extLst>
@@ -78,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="257">
   <si>
     <t>Settings</t>
   </si>
@@ -822,6 +825,33 @@
   </si>
   <si>
     <t>Adam Shailer</t>
+  </si>
+  <si>
+    <t>TECH_ID_HWM</t>
+  </si>
+  <si>
+    <t>Last technician ID number</t>
+  </si>
+  <si>
+    <t>Read-only. The highest TechID number issued at this site. Only ever rises, so an ID is never reused.</t>
+  </si>
+  <si>
+    <t>PRINTER_ID_HWM</t>
+  </si>
+  <si>
+    <t>Last printer ID number</t>
+  </si>
+  <si>
+    <t>Read-only. The highest PrinterID number issued at this site. Only ever rises, so an ID is never reused.</t>
+  </si>
+  <si>
+    <t>STOCK_ID_HWM</t>
+  </si>
+  <si>
+    <t>Last paper ID number</t>
+  </si>
+  <si>
+    <t>Read-only. The highest StockID number issued at this site. Only ever rises, so an ID is never reused.</t>
   </si>
 </sst>
 </file>
@@ -982,7 +1012,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1107,11 +1137,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1262,6 +1305,10 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2265,8 +2312,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A5:D20" totalsRowShown="0">
-  <autoFilter ref="A5:D20" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A5:D23" totalsRowShown="0">
+  <autoFilter ref="A5:D23" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key" dataDxfId="76"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Setting" dataDxfId="75"/>
@@ -5060,7 +5107,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
@@ -5459,6 +5506,42 @@
       </c>
       <c r="D20" s="26" t="s">
         <v>226</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="C21" s="48"/>
+      <c r="D21" s="26" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="C22" s="48"/>
+      <c r="D22" s="26" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="C23" s="48"/>
+      <c r="D23" s="26" t="s">
+        <v>256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bake the final layout into PrintCosts.xlsx
The template now ships what setup used to build on every run: the
LOC_MINIMAL_COLUMNS and REPORT_HEADING settings rows (in display order, with
SET_ names, current labels, notes and defaults), current version and schema
stamps, the two location header gap rows, the three Settings button-band rows
with the stale P2:P3 text cleared, D1:D2 cleared, roll-unit-aware Unit / Area m2 /
Paper Cost formulas, no stray validation below the job table, no built-in
Supplied rows in tblPapers, Supplied by student defaulted, and catalogue IDs
with their counters on the sample rows.

Made by running the workbook's own setup routines on a temp copy; a rebuild
from this file matches a rebuild from the old template apart from the hidden
LOC_RollUnitApplied name. Code is unchanged; step 2 removes the upgraders.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\claude\C--Users-adash-OneDrive-Development-OfficeApps-PrintJob\97da5acd-fb69-4037-ad89-90b60a7c50c7\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30789ADB-78C4-4CF3-BB63-90FD3435BBB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F0EF5AC-E533-4946-8786-E4DD940772F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,17 +26,17 @@
   </sheets>
   <definedNames>
     <definedName name="LOC_Code" localSheetId="0">'Example Print Room'!$AM$2</definedName>
-    <definedName name="LOC_DefDisCons" localSheetId="0">'Example Print Room'!$B$7</definedName>
-    <definedName name="LOC_DefDisPaper" localSheetId="0">'Example Print Room'!$B$6</definedName>
-    <definedName name="LOC_DefPaper" localSheetId="0">'Example Print Room'!$B$5</definedName>
-    <definedName name="LOC_DefPrinter" localSheetId="0">'Example Print Room'!$B$4</definedName>
-    <definedName name="LOC_DefTech" localSheetId="0">'Example Print Room'!$B$3</definedName>
+    <definedName name="LOC_DefDisCons" localSheetId="0">'Example Print Room'!$B$9</definedName>
+    <definedName name="LOC_DefDisPaper" localSheetId="0">'Example Print Room'!$B$8</definedName>
+    <definedName name="LOC_DefPaper" localSheetId="0">'Example Print Room'!$B$6</definedName>
+    <definedName name="LOC_DefPrinter" localSheetId="0">'Example Print Room'!$B$5</definedName>
+    <definedName name="LOC_DefTech" localSheetId="0">'Example Print Room'!$B$4</definedName>
     <definedName name="LOC_Dept" localSheetId="0">'Example Print Room'!$B$2</definedName>
-    <definedName name="LOC_Export" localSheetId="0">'Example Print Room'!$AM$6</definedName>
+    <definedName name="LOC_Export" localSheetId="0">'Example Print Room'!$AM$8</definedName>
     <definedName name="LOC_Name" localSheetId="0">'Example Print Room'!$B$1</definedName>
-    <definedName name="LOC_Printers" localSheetId="0">'Example Print Room'!$AM$7</definedName>
-    <definedName name="LOC_RollUnit" localSheetId="0">'Example Print Room'!$B$9</definedName>
-    <definedName name="LOC_Status" localSheetId="0">'Example Print Room'!$AM$5</definedName>
+    <definedName name="LOC_Printers" localSheetId="0">'Example Print Room'!$AM$9</definedName>
+    <definedName name="LOC_RollUnit" localSheetId="0">'Example Print Room'!$B$11</definedName>
+    <definedName name="LOC_Status" localSheetId="0">'Example Print Room'!$AM$6</definedName>
     <definedName name="lstConsumables">tblConsumables[Consumable type]</definedName>
     <definedName name="lstPaperTypes">tblPaperTypes[Paper type]</definedName>
     <definedName name="lstPrinters">tblPrinters[Model]</definedName>
@@ -44,24 +44,26 @@
     <definedName name="lstStocks">tblPapers[Description]</definedName>
     <definedName name="lstTechnicians">tblTechnicians[Name]</definedName>
     <definedName name="RNG_STD_SIZES">tblStandardSizes[Size name]</definedName>
-    <definedName name="SET_APP_VER">Settings!$C$14</definedName>
-    <definedName name="SET_BUILT">Settings!$C$15</definedName>
-    <definedName name="SET_BUILT_BY">Settings!$C$16</definedName>
-    <definedName name="SET_COST_COLS_HIDDEN">Settings!$C$20</definedName>
-    <definedName name="SET_CURRENCY">Settings!$C$10</definedName>
-    <definedName name="SET_DEPT">Settings!$C$9</definedName>
-    <definedName name="SET_EXPORT_FOLDER">Settings!$C$17</definedName>
-    <definedName name="SET_LASTREF">Settings!$C$13</definedName>
-    <definedName name="SET_LOC_REDUCED_COLUMNS">Settings!$C$19</definedName>
-    <definedName name="SET_LOC_REDUCED_VIEW">Settings!$C$18</definedName>
-    <definedName name="SET_ORG">Settings!$C$8</definedName>
-    <definedName name="SET_PRINTER_ID_HWM">Settings!$C$22</definedName>
-    <definedName name="SET_ROUND_DP">Settings!$C$11</definedName>
-    <definedName name="SET_SCHEMA">Settings!$C$12</definedName>
-    <definedName name="SET_SITE_ID">Settings!$C$6</definedName>
-    <definedName name="SET_SITE_NAME">Settings!$C$7</definedName>
-    <definedName name="SET_STOCK_ID_HWM">Settings!$C$23</definedName>
-    <definedName name="SET_TECH_ID_HWM">Settings!$C$21</definedName>
+    <definedName name="SET_APP_VER">Settings!$C$17</definedName>
+    <definedName name="SET_BUILT">Settings!$C$18</definedName>
+    <definedName name="SET_BUILT_BY">Settings!$C$19</definedName>
+    <definedName name="SET_COST_COLS_HIDDEN">Settings!$C$24</definedName>
+    <definedName name="SET_CURRENCY">Settings!$C$13</definedName>
+    <definedName name="SET_DEPT">Settings!$C$12</definedName>
+    <definedName name="SET_EXPORT_FOLDER">Settings!$C$20</definedName>
+    <definedName name="SET_LASTREF">Settings!$C$16</definedName>
+    <definedName name="SET_LOC_MINIMAL_COLUMNS">Settings!$C$23</definedName>
+    <definedName name="SET_LOC_REDUCED_COLUMNS">Settings!$C$22</definedName>
+    <definedName name="SET_LOC_REDUCED_VIEW">Settings!$C$21</definedName>
+    <definedName name="SET_ORG">Settings!$C$11</definedName>
+    <definedName name="SET_PRINTER_ID_HWM">Settings!$C$26</definedName>
+    <definedName name="SET_REPORT_HEADING">Settings!$C$28</definedName>
+    <definedName name="SET_ROUND_DP">Settings!$C$14</definedName>
+    <definedName name="SET_SCHEMA">Settings!$C$15</definedName>
+    <definedName name="SET_SITE_ID">Settings!$C$9</definedName>
+    <definedName name="SET_SITE_NAME">Settings!$C$10</definedName>
+    <definedName name="SET_STOCK_ID_HWM">Settings!$C$27</definedName>
+    <definedName name="SET_TECH_ID_HWM">Settings!$C$25</definedName>
   </definedNames>
   <calcPr calcId="191029" calcOnSave="0"/>
   <extLst>
@@ -81,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="275">
   <si>
     <t>Settings</t>
   </si>
@@ -269,12 +271,6 @@
     <t>Latex</t>
   </si>
   <si>
-    <t>Commands</t>
-  </si>
-  <si>
-    <t>Buttons appear here once InitialiseWorkbook has been run.</t>
-  </si>
-  <si>
     <t>Print Technicians</t>
   </si>
   <si>
@@ -491,12 +487,6 @@
     <t>PRINTLOC/v1</t>
   </si>
   <si>
-    <t>Print room configuration</t>
-  </si>
-  <si>
-    <t>Defaults seed each new print job. Changing them afterwards never alters rows that already exist.</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -722,9 +712,6 @@
     <t>Read-only.</t>
   </si>
   <si>
-    <t>0.10.0</t>
-  </si>
-  <si>
     <t>EXPORT_FOLDER</t>
   </si>
   <si>
@@ -737,24 +724,12 @@
     <t>LOC_REDUCED_VIEW</t>
   </si>
   <si>
-    <t>Reduced location view</t>
-  </si>
-  <si>
-    <t>Yes hides the columns named in the setting below on every location sheet (toggled by the button on each one). No shows every column.</t>
-  </si>
-  <si>
     <t>LOC_REDUCED_COLUMNS</t>
   </si>
   <si>
     <t>Reduced view - hidden columns</t>
   </si>
   <si>
-    <t>Semicolon-separated column headers hidden by the reduced view above. Edit this list to change which columns it hides - no rebuild needed.</t>
-  </si>
-  <si>
-    <t>Status;Job ID;Printer;Area m2;Disregard Paper;Disregard Consumable;S_SchemaVer</t>
-  </si>
-  <si>
     <t>COST_COLS_HIDDEN</t>
   </si>
   <si>
@@ -779,15 +754,6 @@
     <t>Supplied by student</t>
   </si>
   <si>
-    <t>Supplied (Roll)</t>
-  </si>
-  <si>
-    <t>Student supplied</t>
-  </si>
-  <si>
-    <t>Supplied (Sheet)</t>
-  </si>
-  <si>
     <t>Paid</t>
   </si>
   <si>
@@ -852,6 +818,96 @@
   </si>
   <si>
     <t>Read-only. The highest StockID number issued at this site. Only ever rises, so an ID is never reused.</t>
+  </si>
+  <si>
+    <t>0.10.21</t>
+  </si>
+  <si>
+    <t>Location column view</t>
+  </si>
+  <si>
+    <t>Which columns location sheets show: All, Reduced or Minimal. Set by the Show columns drop-down on each location sheet; applies to every location.</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Semicolon-separated column headers hidden by the Reduced view. Edit to change what it hides - no rebuild needed. Minimal hides these as well.</t>
+  </si>
+  <si>
+    <t>Status;Job ID;Area m2;S_SchemaVer</t>
+  </si>
+  <si>
+    <t>LOC_MINIMAL_COLUMNS</t>
+  </si>
+  <si>
+    <t>Minimal view - extra hidden columns</t>
+  </si>
+  <si>
+    <t>Semicolon-separated column headers the Minimal view hides IN ADDITION to the Reduced list above (Minimal always includes Reduced). Edit to change - no rebuild needed.</t>
+  </si>
+  <si>
+    <t>Printer;Disregard Paper;Disregard Consumable;Print Width mm;Sheet size</t>
+  </si>
+  <si>
+    <t>REPORT_HEADING</t>
+  </si>
+  <si>
+    <t>Report heading</t>
+  </si>
+  <si>
+    <t>The heading printed at the top of an exported Reports report. Leave blank for 'Print job report'.</t>
+  </si>
+  <si>
+    <t>Print job report</t>
+  </si>
+  <si>
+    <t>UNI-TCH-0001</t>
+  </si>
+  <si>
+    <t>UNI-TCH-0002</t>
+  </si>
+  <si>
+    <t>UNI-TCH-0003</t>
+  </si>
+  <si>
+    <t>UNI-PRN-0001</t>
+  </si>
+  <si>
+    <t>UNI-PRN-0002</t>
+  </si>
+  <si>
+    <t>UNI-PRN-0003</t>
+  </si>
+  <si>
+    <t>UNI-PRN-0004</t>
+  </si>
+  <si>
+    <t>UNI-STK-0001</t>
+  </si>
+  <si>
+    <t>UNI-STK-0002</t>
+  </si>
+  <si>
+    <t>UNI-STK-0003</t>
+  </si>
+  <si>
+    <t>UNI-STK-0004</t>
+  </si>
+  <si>
+    <t>UNI-STK-0005</t>
+  </si>
+  <si>
+    <t>UNI-STK-0006</t>
+  </si>
+  <si>
+    <t>UNI-STK-0007</t>
+  </si>
+  <si>
+    <t>UNI-STK-0008</t>
+  </si>
+  <si>
+    <t>UNI-STK-0009</t>
   </si>
 </sst>
 </file>
@@ -2185,8 +2241,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_MAIN" displayName="tblJobs_MAIN" ref="A15:AH27" totalsRowShown="0">
-  <autoFilter ref="A15:AH27" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_MAIN" displayName="tblJobs_MAIN" ref="A17:AH29" totalsRowShown="0">
+  <autoFilter ref="A17:AH29" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="34">
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Date/Time" dataDxfId="62"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="61"/>
@@ -2195,7 +2251,7 @@
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="58"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="57"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="56">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Qty" dataDxfId="55"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Print Width mm" dataDxfId="54"/>
@@ -2203,10 +2259,10 @@
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Disregard Paper" dataDxfId="52"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Disregard Consumable" dataDxfId="51"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Area m2" dataDxfId="50">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="49">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="48">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</calculatedColumnFormula>
@@ -2289,8 +2345,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:L17" totalsRowShown="0" dataDxfId="15">
-  <autoFilter ref="A6:L17" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:L15" totalsRowShown="0" dataDxfId="15">
+  <autoFilter ref="A6:L15" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="14"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Description" dataDxfId="13"/>
@@ -2312,8 +2368,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A5:D23" totalsRowShown="0">
-  <autoFilter ref="A5:D23" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A8:D28" totalsRowShown="0">
+  <autoFilter ref="A8:D28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key" dataDxfId="76"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Setting" dataDxfId="75"/>
@@ -2325,8 +2381,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblPaperTypes" displayName="tblPaperTypes" ref="F5:G11" totalsRowShown="0" dataDxfId="72">
-  <autoFilter ref="F5:G11" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblPaperTypes" displayName="tblPaperTypes" ref="F8:G14" totalsRowShown="0" dataDxfId="72">
+  <autoFilter ref="F8:G14" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Paper type" dataDxfId="71"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Active" dataDxfId="70"/>
@@ -2336,8 +2392,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="tblStandardSizes" displayName="tblStandardSizes" ref="I5:K11" totalsRowShown="0" dataDxfId="69">
-  <autoFilter ref="I5:K11" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="tblStandardSizes" displayName="tblStandardSizes" ref="I8:K14" totalsRowShown="0" dataDxfId="69">
+  <autoFilter ref="I8:K14" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Size name" dataDxfId="68"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Width mm" dataDxfId="67"/>
@@ -2348,8 +2404,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="tblConsumables" displayName="tblConsumables" ref="M5:N9" totalsRowShown="0" dataDxfId="65">
-  <autoFilter ref="M5:N9" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="tblConsumables" displayName="tblConsumables" ref="M8:N12" totalsRowShown="0" dataDxfId="65">
+  <autoFilter ref="M8:N12" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Consumable type" dataDxfId="64"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Active" dataDxfId="63"/>
@@ -2666,7 +2722,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr codeName="Sheet10"/>
-  <dimension ref="A1:AZ27"/>
+  <dimension ref="A1:AZ29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.6328125" customWidth="1"/>
@@ -2705,19 +2761,16 @@
   <sheetData>
     <row r="1" spans="1:52" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="AL1" s="18" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="AZ1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:52" x14ac:dyDescent="0.35">
@@ -2727,470 +2780,255 @@
       <c r="B2" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>137</v>
-      </c>
       <c r="AL2" s="18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="AM2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="B3" s="32"/>
-      <c r="D3" s="2"/>
-    </row>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="3" spans="1:52" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="B4" s="33"/>
+        <v>225</v>
+      </c>
+      <c r="B4" s="32"/>
+      <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>239</v>
+        <v>226</v>
       </c>
       <c r="B5" s="33"/>
-      <c r="AL5" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>134</v>
-      </c>
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
+      <c r="A6" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="AL6" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="AM6" t="s">
         <v>132</v>
       </c>
-      <c r="AL6" s="42" t="s">
-        <v>245</v>
-      </c>
-      <c r="AM6" s="28" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
-        <v>132</v>
-      </c>
-      <c r="AL7" s="18" t="s">
-        <v>182</v>
-      </c>
-      <c r="AM7" t="s">
-        <v>199</v>
-      </c>
-    </row>
+    </row>
+    <row r="7" spans="1:52" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="AL8" s="19" t="s">
-        <v>181</v>
+      <c r="B8" t="s">
+        <v>130</v>
+      </c>
+      <c r="AL8" s="42" t="s">
+        <v>233</v>
+      </c>
+      <c r="AM8" s="28" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="B9" s="32" t="s">
-        <v>241</v>
+      <c r="B9" t="s">
+        <v>130</v>
+      </c>
+      <c r="AL9" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="B10" s="5" t="str">
+      <c r="AL10" s="19" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="11" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="12" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="B12" s="5" t="str">
         <f>_xlfn.LET(_xlpm.list,LOC_Printers,_xlpm.n,IF(_xlpm.list="",0,LEN(_xlpm.list)-LEN(SUBSTITUTE(_xlpm.list,";",""))+1),IF(_xlpm.n=0,"0 printers ()",_xlpm.n&amp;" printer"&amp;IF(_xlpm.n=1,"","s")&amp;" ("&amp;SUBSTITUTE(_xlpm.list,";",", ")&amp;")"))</f>
         <v>3 printers (Epson SureColor P9500, HP DesignJet Z9+, Xerox Versant 180)</v>
       </c>
     </row>
-    <row r="11" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A11" s="27" t="s">
-        <v>243</v>
-      </c>
-      <c r="B11">
+    <row r="13" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A13" s="27" t="s">
+        <v>231</v>
+      </c>
+      <c r="B13">
         <f>ROWS(tblJobs_MAIN[])</f>
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="G13" s="29"/>
-      <c r="I13" s="29"/>
-      <c r="K13" s="29"/>
-      <c r="M13" s="2"/>
-    </row>
-    <row r="15" spans="1:52" ht="29" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="A15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="I15" s="29"/>
+      <c r="K15" s="29"/>
+      <c r="M15" s="2"/>
+    </row>
+    <row r="17" spans="1:34" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="H17" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="I17" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="J17" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="K17" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="L17" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="M17" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="H15" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I15" s="4" t="s">
+      <c r="N17" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="J15" s="23" t="s">
-        <v>244</v>
-      </c>
-      <c r="K15" s="4" t="s">
+      <c r="O17" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="L15" s="4" t="s">
+      <c r="P17" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="Q17" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="N15" s="4" t="s">
+      <c r="R17" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="O15" s="4" t="s">
+      <c r="S17" s="23" t="s">
+        <v>223</v>
+      </c>
+      <c r="T17" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="U17" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="V17" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W17" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="P15" s="4" t="s">
+      <c r="X17" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="Q15" s="4" t="s">
+      <c r="Y17" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="R15" s="4" t="s">
+      <c r="Z17" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="S15" s="23" t="s">
-        <v>235</v>
-      </c>
-      <c r="T15" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="U15" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="V15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="W15" s="4" t="s">
+      <c r="AA17" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="X15" s="4" t="s">
+      <c r="AB17" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="Y15" s="4" t="s">
+      <c r="AC17" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="Z15" s="4" t="s">
+      <c r="AD17" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="AA15" s="4" t="s">
+      <c r="AE17" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="AB15" s="4" t="s">
+      <c r="AF17" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="AC15" s="4" t="s">
+      <c r="AG17" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="AD15" s="4" t="s">
+      <c r="AH17" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="AE15" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="AF15" s="4" t="s">
+    </row>
+    <row r="18" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A18" s="11">
+        <v>46280.425000000003</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="AG15" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="AH15" s="4" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="16" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="A16" s="11">
-        <v>46280.425000000003</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="C16" s="12">
+      <c r="C18" s="12">
         <v>2201884</v>
       </c>
-      <c r="D16" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="G16" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+      <c r="D18" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="G18" s="9" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
-      <c r="H16" s="13">
+      <c r="H18" s="13">
         <v>100</v>
       </c>
-      <c r="I16" s="36"/>
-      <c r="J16" s="39"/>
-      <c r="K16" s="37" t="s">
-        <v>132</v>
-      </c>
-      <c r="L16" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="M16" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
+      <c r="I18" s="36"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="L18" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="M18" s="14">
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>14.400000000000002</v>
       </c>
-      <c r="N16" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+      <c r="N18" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>31</v>
       </c>
-      <c r="O16" s="15">
+      <c r="O18" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
         <v>13.68</v>
       </c>
-      <c r="P16" s="15">
+      <c r="P18" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
         <v>44.68</v>
-      </c>
-      <c r="Q16" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>0</v>
-      </c>
-      <c r="R16" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>44.68</v>
-      </c>
-      <c r="S16" s="34"/>
-      <c r="T16" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
-        <v>OK</v>
-      </c>
-      <c r="U16" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="V16" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="W16" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
-        <v/>
-      </c>
-      <c r="X16" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="Y16" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="Z16" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="AA16" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="AB16" s="17">
-        <v>0.31</v>
-      </c>
-      <c r="AC16" s="16">
-        <v>320</v>
-      </c>
-      <c r="AD16" s="16">
-        <v>450</v>
-      </c>
-      <c r="AE16" s="17">
-        <v>0.95</v>
-      </c>
-      <c r="AF16" s="16">
-        <v>46280.425000000003</v>
-      </c>
-      <c r="AG16" s="16" t="s">
-        <v>171</v>
-      </c>
-      <c r="AH16" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="A17" s="11">
-        <v>46280.611111111109</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="C17" s="12">
-        <v>2201884</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="E17" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="F17" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="G17" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>metres</v>
-      </c>
-      <c r="H17" s="13">
-        <v>12</v>
-      </c>
-      <c r="I17" s="36"/>
-      <c r="J17" s="39"/>
-      <c r="K17" s="37" t="s">
-        <v>132</v>
-      </c>
-      <c r="L17" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="M17" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>10.968</v>
-      </c>
-      <c r="N17" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>105</v>
-      </c>
-      <c r="O17" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>31.26</v>
-      </c>
-      <c r="P17" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>136.26</v>
-      </c>
-      <c r="Q17" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>0</v>
-      </c>
-      <c r="R17" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>136.26</v>
-      </c>
-      <c r="S17" s="35"/>
-      <c r="T17" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
-        <v>OK</v>
-      </c>
-      <c r="U17" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="V17" s="12" t="s">
-        <v>173</v>
-      </c>
-      <c r="W17" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
-        <v/>
-      </c>
-      <c r="X17" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="Y17" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="Z17" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="AA17" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="AB17" s="17">
-        <v>8.75</v>
-      </c>
-      <c r="AC17" s="16">
-        <v>914</v>
-      </c>
-      <c r="AD17" s="16"/>
-      <c r="AE17" s="17">
-        <v>2.85</v>
-      </c>
-      <c r="AF17" s="16">
-        <v>46280.611111111109</v>
-      </c>
-      <c r="AG17" s="16" t="s">
-        <v>171</v>
-      </c>
-      <c r="AH17" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="A18" s="11">
-        <v>46281.461805555555</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="C18" s="12">
-        <v>2203110</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="E18" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="G18" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>metres</v>
-      </c>
-      <c r="H18" s="13">
-        <v>12</v>
-      </c>
-      <c r="I18" s="36">
-        <v>600</v>
-      </c>
-      <c r="J18" s="39"/>
-      <c r="K18" s="37" t="s">
-        <v>132</v>
-      </c>
-      <c r="L18" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="M18" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>7.1999999999999993</v>
-      </c>
-      <c r="N18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>105</v>
-      </c>
-      <c r="O18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>20.52</v>
-      </c>
-      <c r="P18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>125.52</v>
       </c>
       <c r="Q18" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
@@ -3198,50 +3036,52 @@
       </c>
       <c r="R18" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>125.52</v>
-      </c>
-      <c r="S18" s="35"/>
+        <v>44.68</v>
+      </c>
+      <c r="S18" s="34"/>
       <c r="T18" s="9" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
         <v>OK</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="V18" s="12" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="W18" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="X18" s="16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Y18" s="16" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="Z18" s="16" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="AA18" s="16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AB18" s="17">
-        <v>8.75</v>
+        <v>0.31</v>
       </c>
       <c r="AC18" s="16">
-        <v>914</v>
-      </c>
-      <c r="AD18" s="16"/>
+        <v>320</v>
+      </c>
+      <c r="AD18" s="16">
+        <v>450</v>
+      </c>
       <c r="AE18" s="17">
-        <v>2.85</v>
+        <v>0.95</v>
       </c>
       <c r="AF18" s="16">
-        <v>46281.461805555555</v>
+        <v>46280.425000000003</v>
       </c>
       <c r="AG18" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH18" s="16">
         <v>1</v>
@@ -3249,61 +3089,61 @@
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A19" s="11">
-        <v>46281.638888888891</v>
+        <v>46280.611111111109</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C19" s="12">
-        <v>2203110</v>
+        <v>2201884</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>69</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>106</v>
       </c>
       <c r="G19" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="H19" s="13">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I19" s="36"/>
       <c r="J19" s="39"/>
       <c r="K19" s="37" t="s">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="L19" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="M19" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>3.05</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>10.968</v>
       </c>
       <c r="N19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>15.5</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>105</v>
       </c>
       <c r="O19" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>8.69</v>
+        <v>31.26</v>
       </c>
       <c r="P19" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>24.189999999999998</v>
+        <v>136.26</v>
       </c>
       <c r="Q19" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>15.499999999999998</v>
+        <v>0</v>
       </c>
       <c r="R19" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>8.69</v>
+        <v>136.26</v>
       </c>
       <c r="S19" s="35"/>
       <c r="T19" s="9" t="str">
@@ -3311,17 +3151,17 @@
         <v>OK</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="V19" s="12" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="W19" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="X19" s="16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Y19" s="16" t="s">
         <v>105</v>
@@ -3333,20 +3173,20 @@
         <v>45</v>
       </c>
       <c r="AB19" s="17">
-        <v>3.1</v>
+        <v>8.75</v>
       </c>
       <c r="AC19" s="16">
-        <v>610</v>
+        <v>914</v>
       </c>
       <c r="AD19" s="16"/>
       <c r="AE19" s="17">
         <v>2.85</v>
       </c>
       <c r="AF19" s="16">
-        <v>46281.638888888891</v>
+        <v>46280.611111111109</v>
       </c>
       <c r="AG19" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH19" s="16">
         <v>1</v>
@@ -3354,61 +3194,63 @@
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A20" s="11">
-        <v>46282.381944444445</v>
+        <v>46281.461805555555</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="C20" s="12">
-        <v>2204521</v>
+        <v>2203110</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G20" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>sheets</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <v>metres</v>
       </c>
       <c r="H20" s="13">
-        <v>25</v>
-      </c>
-      <c r="I20" s="36"/>
+        <v>12</v>
+      </c>
+      <c r="I20" s="36">
+        <v>600</v>
+      </c>
       <c r="J20" s="39"/>
       <c r="K20" s="37" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L20" s="12" t="s">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="M20" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>3.1184999999999996</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>7.1999999999999993</v>
       </c>
       <c r="N20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>2.25</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>105</v>
       </c>
       <c r="O20" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>2.96</v>
+        <v>20.52</v>
       </c>
       <c r="P20" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>5.21</v>
+        <v>125.52</v>
       </c>
       <c r="Q20" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>2.96</v>
+        <v>0</v>
       </c>
       <c r="R20" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>2.25</v>
+        <v>125.52</v>
       </c>
       <c r="S20" s="35"/>
       <c r="T20" s="9" t="str">
@@ -3416,44 +3258,42 @@
         <v>OK</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="V20" s="12" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="W20" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="X20" s="16" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="Y20" s="16" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="Z20" s="16" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AA20" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AB20" s="17">
-        <v>0.09</v>
+        <v>8.75</v>
       </c>
       <c r="AC20" s="16">
-        <v>297</v>
-      </c>
-      <c r="AD20" s="16">
-        <v>420</v>
-      </c>
+        <v>914</v>
+      </c>
+      <c r="AD20" s="16"/>
       <c r="AE20" s="17">
-        <v>0.95</v>
+        <v>2.85</v>
       </c>
       <c r="AF20" s="16">
-        <v>46282.381944444445</v>
+        <v>46281.461805555555</v>
       </c>
       <c r="AG20" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH20" s="16">
         <v>1</v>
@@ -3461,61 +3301,61 @@
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A21" s="11">
-        <v>46282.559027777781</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>183</v>
+        <v>46281.638888888891</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>171</v>
       </c>
       <c r="C21" s="12">
-        <v>2204521</v>
+        <v>2203110</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G21" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>sheets</v>
+        <v>104</v>
+      </c>
+      <c r="G21" s="9" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <v>metres</v>
       </c>
       <c r="H21" s="13">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="I21" s="36"/>
       <c r="J21" s="39"/>
-      <c r="K21" s="38" t="s">
-        <v>132</v>
+      <c r="K21" s="37" t="s">
+        <v>38</v>
       </c>
       <c r="L21" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="M21" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>2.16</v>
+        <v>130</v>
+      </c>
+      <c r="M21" s="14">
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>3.05</v>
       </c>
       <c r="N21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>2.7</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>15.5</v>
       </c>
       <c r="O21" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>2.0499999999999998</v>
+        <v>8.69</v>
       </c>
       <c r="P21" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>4.75</v>
+        <v>24.189999999999998</v>
       </c>
       <c r="Q21" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>0</v>
+        <v>15.499999999999998</v>
       </c>
       <c r="R21" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>4.75</v>
+        <v>8.69</v>
       </c>
       <c r="S21" s="35"/>
       <c r="T21" s="9" t="str">
@@ -3523,44 +3363,42 @@
         <v>OK</v>
       </c>
       <c r="U21" s="5" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="V21" s="12" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="W21" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="X21" s="16" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="Y21" s="16" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="Z21" s="16" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="AA21" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AB21" s="17">
-        <v>0.18</v>
+        <v>3.1</v>
       </c>
       <c r="AC21" s="16">
-        <v>320</v>
-      </c>
-      <c r="AD21" s="16">
-        <v>450</v>
-      </c>
+        <v>610</v>
+      </c>
+      <c r="AD21" s="16"/>
       <c r="AE21" s="17">
-        <v>0.95</v>
+        <v>2.85</v>
       </c>
       <c r="AF21" s="16">
-        <v>46282.559027777781</v>
+        <v>46281.638888888891</v>
       </c>
       <c r="AG21" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH21" s="16">
         <v>1</v>
@@ -3568,10 +3406,10 @@
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A22" s="11">
-        <v>46282.666666666664</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>183</v>
+        <v>46282.381944444445</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>179</v>
       </c>
       <c r="C22" s="12">
         <v>2204521</v>
@@ -3580,49 +3418,49 @@
         <v>71</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="G22" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>metres</v>
+        <v>102</v>
+      </c>
+      <c r="G22" s="9" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <v>sheets</v>
       </c>
       <c r="H22" s="13">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="I22" s="36"/>
       <c r="J22" s="39"/>
-      <c r="K22" s="38" t="s">
-        <v>132</v>
+      <c r="K22" s="37" t="s">
+        <v>130</v>
       </c>
       <c r="L22" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="M22" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>10.96</v>
+        <v>38</v>
+      </c>
+      <c r="M22" s="14">
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>3.1184999999999996</v>
       </c>
       <c r="N22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>91.2</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>2.25</v>
       </c>
       <c r="O22" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>19.18</v>
+        <v>2.96</v>
       </c>
       <c r="P22" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>110.38</v>
+        <v>5.21</v>
       </c>
       <c r="Q22" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
-        <v>0</v>
+        <v>2.96</v>
       </c>
       <c r="R22" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>110.38</v>
+        <v>2.25</v>
       </c>
       <c r="S22" s="35"/>
       <c r="T22" s="9" t="str">
@@ -3630,42 +3468,44 @@
         <v>OK</v>
       </c>
       <c r="U22" s="5" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="V22" s="12" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="W22" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="X22" s="16" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="Y22" s="16" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="Z22" s="16" t="s">
         <v>70</v>
       </c>
       <c r="AA22" s="16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AB22" s="17">
-        <v>11.4</v>
+        <v>0.09</v>
       </c>
       <c r="AC22" s="16">
-        <v>1370</v>
-      </c>
-      <c r="AD22" s="16"/>
+        <v>297</v>
+      </c>
+      <c r="AD22" s="16">
+        <v>420</v>
+      </c>
       <c r="AE22" s="17">
-        <v>1.75</v>
+        <v>0.95</v>
       </c>
       <c r="AF22" s="16">
-        <v>46282.666666666664</v>
+        <v>46282.381944444445</v>
       </c>
       <c r="AG22" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH22" s="16">
         <v>1</v>
@@ -3673,51 +3513,53 @@
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46283.427083333336</v>
-      </c>
-      <c r="B23" s="11"/>
+        <v>46282.559027777781</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>179</v>
+      </c>
       <c r="C23" s="12">
-        <v>2205077</v>
+        <v>2204521</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E23" s="12" t="s">
         <v>83</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="G23" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>metres</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <v>sheets</v>
       </c>
       <c r="H23" s="13">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I23" s="36"/>
       <c r="J23" s="39"/>
       <c r="K23" s="38" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L23" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="M23" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>1.83</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>2.16</v>
       </c>
       <c r="N23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>9.3000000000000007</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>2.7</v>
       </c>
       <c r="O23" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>4.3899999999999997</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="P23" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>13.690000000000001</v>
+        <v>4.75</v>
       </c>
       <c r="Q23" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
@@ -3725,7 +3567,7 @@
       </c>
       <c r="R23" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>13.690000000000001</v>
+        <v>4.75</v>
       </c>
       <c r="S23" s="35"/>
       <c r="T23" s="9" t="str">
@@ -3733,10 +3575,10 @@
         <v>OK</v>
       </c>
       <c r="U23" s="5" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="V23" s="12" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="W23" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
@@ -3746,29 +3588,31 @@
         <v>82</v>
       </c>
       <c r="Y23" s="16" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="Z23" s="16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA23" s="16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AB23" s="17">
-        <v>3.1</v>
+        <v>0.18</v>
       </c>
       <c r="AC23" s="16">
-        <v>610</v>
-      </c>
-      <c r="AD23" s="16"/>
+        <v>320</v>
+      </c>
+      <c r="AD23" s="16">
+        <v>450</v>
+      </c>
       <c r="AE23" s="17">
-        <v>2.4</v>
+        <v>0.95</v>
       </c>
       <c r="AF23" s="16">
-        <v>46283.427083333336</v>
+        <v>46282.559027777781</v>
       </c>
       <c r="AG23" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH23" s="16">
         <v>1</v>
@@ -3776,51 +3620,53 @@
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A24" s="11">
-        <v>46283.486111111109</v>
+        <v>46282.666666666664</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="C24" s="12"/>
+        <v>179</v>
+      </c>
+      <c r="C24" s="12">
+        <v>2204521</v>
+      </c>
       <c r="D24" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E24" s="12" t="s">
         <v>85</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="G24" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
-        <v>sheets</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <v>metres</v>
       </c>
       <c r="H24" s="13">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="I24" s="36"/>
       <c r="J24" s="39"/>
       <c r="K24" s="38" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L24" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="M24" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>7.4843999999999991</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>10.96</v>
       </c>
       <c r="N24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>7.2</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>91.2</v>
       </c>
       <c r="O24" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>7.11</v>
+        <v>19.18</v>
       </c>
       <c r="P24" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>14.31</v>
+        <v>110.38</v>
       </c>
       <c r="Q24" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
@@ -3828,7 +3674,7 @@
       </c>
       <c r="R24" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>14.31</v>
+        <v>110.38</v>
       </c>
       <c r="S24" s="35"/>
       <c r="T24" s="9" t="str">
@@ -3836,10 +3682,10 @@
         <v>OK</v>
       </c>
       <c r="U24" s="5" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="V24" s="12" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="W24" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
@@ -3849,31 +3695,29 @@
         <v>84</v>
       </c>
       <c r="Y24" s="16" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="Z24" s="16" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AA24" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AB24" s="17">
-        <v>0.24</v>
+        <v>11.4</v>
       </c>
       <c r="AC24" s="16">
-        <v>420</v>
-      </c>
-      <c r="AD24" s="16">
-        <v>594</v>
-      </c>
+        <v>1370</v>
+      </c>
+      <c r="AD24" s="16"/>
       <c r="AE24" s="17">
-        <v>0.95</v>
+        <v>1.75</v>
       </c>
       <c r="AF24" s="16">
-        <v>46283.486111111109</v>
+        <v>46282.666666666664</v>
       </c>
       <c r="AG24" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH24" s="16">
         <v>1</v>
@@ -3881,53 +3725,51 @@
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46283.638888888891</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>183</v>
-      </c>
+        <v>46283.427083333336</v>
+      </c>
+      <c r="B25" s="11"/>
       <c r="C25" s="12">
-        <v>2204521</v>
+        <v>2205077</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E25" s="12" t="s">
         <v>81</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="G25" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="H25" s="13">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="I25" s="36"/>
       <c r="J25" s="39"/>
       <c r="K25" s="38" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L25" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="M25" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>21.34</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>1.83</v>
       </c>
       <c r="N25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>112</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>9.3000000000000007</v>
       </c>
       <c r="O25" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>60.82</v>
+        <v>4.3899999999999997</v>
       </c>
       <c r="P25" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>172.82</v>
+        <v>13.690000000000001</v>
       </c>
       <c r="Q25" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
@@ -3935,7 +3777,7 @@
       </c>
       <c r="R25" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>172.82</v>
+        <v>13.690000000000001</v>
       </c>
       <c r="S25" s="35"/>
       <c r="T25" s="9" t="str">
@@ -3943,10 +3785,10 @@
         <v>OK</v>
       </c>
       <c r="U25" s="5" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="V25" s="12" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="W25" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
@@ -3956,29 +3798,29 @@
         <v>80</v>
       </c>
       <c r="Y25" s="16" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="Z25" s="16" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="AA25" s="16" t="s">
         <v>45</v>
       </c>
       <c r="AB25" s="17">
-        <v>5.6</v>
+        <v>3.1</v>
       </c>
       <c r="AC25" s="16">
-        <v>1067</v>
+        <v>610</v>
       </c>
       <c r="AD25" s="16"/>
       <c r="AE25" s="17">
-        <v>2.85</v>
+        <v>2.4</v>
       </c>
       <c r="AF25" s="16">
-        <v>46283.638888888891</v>
+        <v>46283.427083333336</v>
       </c>
       <c r="AG25" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH25" s="16">
         <v>1</v>
@@ -3986,53 +3828,51 @@
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A26" s="11">
-        <v>46284.34375</v>
+        <v>46283.486111111109</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="C26" s="12">
-        <v>2203110</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="C26" s="12"/>
       <c r="D26" s="12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G26" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
       <c r="H26" s="13">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I26" s="36"/>
       <c r="J26" s="39"/>
       <c r="K26" s="38" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L26" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="M26" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>19.982159999999997</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>7.4843999999999991</v>
       </c>
       <c r="N26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>16.8</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>7.2</v>
       </c>
       <c r="O26" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>18.98</v>
+        <v>7.11</v>
       </c>
       <c r="P26" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>35.78</v>
+        <v>14.31</v>
       </c>
       <c r="Q26" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
@@ -4040,7 +3880,7 @@
       </c>
       <c r="R26" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>35.78</v>
+        <v>14.31</v>
       </c>
       <c r="S26" s="35"/>
       <c r="T26" s="9" t="str">
@@ -4048,44 +3888,44 @@
         <v>OK</v>
       </c>
       <c r="U26" s="5" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="V26" s="12" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="W26" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="X26" s="16" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="Y26" s="16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="Z26" s="16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA26" s="16" t="s">
         <v>44</v>
       </c>
       <c r="AB26" s="17">
-        <v>0.42</v>
+        <v>0.24</v>
       </c>
       <c r="AC26" s="16">
+        <v>420</v>
+      </c>
+      <c r="AD26" s="16">
         <v>594</v>
-      </c>
-      <c r="AD26" s="16">
-        <v>841</v>
       </c>
       <c r="AE26" s="17">
         <v>0.95</v>
       </c>
       <c r="AF26" s="16">
-        <v>46284.34375</v>
+        <v>46283.486111111109</v>
       </c>
       <c r="AG26" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH26" s="16">
         <v>1</v>
@@ -4093,51 +3933,53 @@
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46284.395833333336</v>
-      </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="12"/>
+        <v>46283.638888888891</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="C27" s="12">
+        <v>2204521</v>
+      </c>
       <c r="D27" s="12" t="s">
         <v>69</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G27" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets","metres"))</f>
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="H27" s="13">
-        <v>12</v>
-      </c>
-      <c r="I27" s="36">
-        <v>1200</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="I27" s="36"/>
       <c r="J27" s="39"/>
       <c r="K27" s="38" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L27" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="M27" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]))</f>
-        <v>14.399999999999999</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>21.34</v>
       </c>
       <c r="N27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
-        <v>105</v>
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>112</v>
       </c>
       <c r="O27" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
-        <v>41.04</v>
+        <v>60.82</v>
       </c>
       <c r="P27" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
-        <v>146.04</v>
+        <v>172.82</v>
       </c>
       <c r="Q27" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
@@ -4145,28 +3987,28 @@
       </c>
       <c r="R27" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
-        <v>146.04</v>
+        <v>172.82</v>
       </c>
       <c r="S27" s="35"/>
       <c r="T27" s="9" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
-        <v>Student name or number required; Print width exceeds stock width</v>
+        <v>OK</v>
       </c>
       <c r="U27" s="5" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="V27" s="12" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="W27" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
-        <v>; Student name or number required; Print width exceeds stock width</v>
+        <v/>
       </c>
       <c r="X27" s="16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Y27" s="16" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="Z27" s="16" t="s">
         <v>68</v>
@@ -4175,67 +4017,262 @@
         <v>45</v>
       </c>
       <c r="AB27" s="17">
-        <v>8.75</v>
+        <v>5.6</v>
       </c>
       <c r="AC27" s="16">
-        <v>914</v>
+        <v>1067</v>
       </c>
       <c r="AD27" s="16"/>
       <c r="AE27" s="17">
         <v>2.85</v>
       </c>
       <c r="AF27" s="16">
-        <v>46284.395833333336</v>
+        <v>46283.638888888891</v>
       </c>
       <c r="AG27" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AH27" s="16">
         <v>1</v>
       </c>
     </row>
+    <row r="28" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A28" s="11">
+        <v>46284.34375</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C28" s="12">
+        <v>2203110</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="G28" s="20" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <v>sheets</v>
+      </c>
+      <c r="H28" s="13">
+        <v>40</v>
+      </c>
+      <c r="I28" s="36"/>
+      <c r="J28" s="39"/>
+      <c r="K28" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="L28" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="M28" s="21">
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>19.982159999999997</v>
+      </c>
+      <c r="N28" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>16.8</v>
+      </c>
+      <c r="O28" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <v>18.98</v>
+      </c>
+      <c r="P28" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <v>35.78</v>
+      </c>
+      <c r="Q28" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <v>0</v>
+      </c>
+      <c r="R28" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <v>35.78</v>
+      </c>
+      <c r="S28" s="35"/>
+      <c r="T28" s="9" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+        <v>OK</v>
+      </c>
+      <c r="U28" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="V28" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="W28" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <v/>
+      </c>
+      <c r="X28" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y28" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z28" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA28" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB28" s="17">
+        <v>0.42</v>
+      </c>
+      <c r="AC28" s="16">
+        <v>594</v>
+      </c>
+      <c r="AD28" s="16">
+        <v>841</v>
+      </c>
+      <c r="AE28" s="17">
+        <v>0.95</v>
+      </c>
+      <c r="AF28" s="16">
+        <v>46284.34375</v>
+      </c>
+      <c r="AG28" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="AH28" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A29" s="11">
+        <v>46284.395833333336</v>
+      </c>
+      <c r="B29" s="11"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="G29" s="20" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <v>metres</v>
+      </c>
+      <c r="H29" s="13">
+        <v>12</v>
+      </c>
+      <c r="I29" s="36">
+        <v>1200</v>
+      </c>
+      <c r="J29" s="39"/>
+      <c r="K29" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="L29" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="M29" s="21">
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <v>14.399999999999999</v>
+      </c>
+      <c r="N29" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <v>105</v>
+      </c>
+      <c r="O29" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+        <v>41.04</v>
+      </c>
+      <c r="P29" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+        <v>146.04</v>
+      </c>
+      <c r="Q29" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <v>0</v>
+      </c>
+      <c r="R29" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+        <v>146.04</v>
+      </c>
+      <c r="S29" s="35"/>
+      <c r="T29" s="9" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+        <v>Student name or number required; Print width exceeds stock width</v>
+      </c>
+      <c r="U29" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="V29" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="W29" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <v>; Student name or number required; Print width exceeds stock width</v>
+      </c>
+      <c r="X29" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y29" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="Z29" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA29" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB29" s="17">
+        <v>8.75</v>
+      </c>
+      <c r="AC29" s="16">
+        <v>914</v>
+      </c>
+      <c r="AD29" s="16"/>
+      <c r="AE29" s="17">
+        <v>2.85</v>
+      </c>
+      <c r="AF29" s="16">
+        <v>46284.395833333336</v>
+      </c>
+      <c r="AG29" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="AH29" s="16">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
-  <conditionalFormatting sqref="T16:T27">
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <conditionalFormatting sqref="T18:T29">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>AND(T16&lt;&gt;"",T16&lt;&gt;"OK")</formula>
+      <formula>AND(T18&lt;&gt;"",T18&lt;&gt;"OK")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Technician" error="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." promptTitle="Technician" prompt="Choose from the active technicians. Inactive technicians stay on historical records but cannot be selected for new jobs." sqref="D28:D2010" xr:uid="{00000000-0002-0000-0900-000000000000}">
-      <formula1>lstTechnicians</formula1>
+  <dataValidations count="7">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date and time" error="Date and time the print was produced. Use the Now button to stamp the current date and time." promptTitle="Date and time" prompt="Date and time the print was produced. Use the Now button to stamp the current date and time." sqref="A18:A29" xr:uid="{00000000-0002-0000-0900-000007000000}">
+      <formula1>36526</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Only printers available at this print room may be selected." promptTitle="Printer" prompt="Only printers available at this print room may be selected." sqref="E28:E2010" xr:uid="{00000000-0002-0000-0900-000001000000}">
-      <formula1>lstPrinters</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L18:L29 K18:K29" xr:uid="{00000000-0002-0000-0900-000003000000}">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." promptTitle="Paper stock" prompt="The list is limited to stocks whose paper family the selected printer supports. Choose a printer first." sqref="F28:F2010" xr:uid="{00000000-0002-0000-0900-000002000000}">
-      <formula1>lstStocks</formula1>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Roll length unit" error="Choose Metres or Centimetres." promptTitle="Roll length unit" prompt="How a roll job's length is typed into Qty on this sheet. Always converted to, and stored as, metres regardless of this setting - Sheet stock is unaffected." sqref="B11" xr:uid="{DDF6FDDC-C744-4D90-987F-9EBAA10EE831}">
+      <formula1>"Metres,Centimetres"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle="Quantity" error="Sheets for sheet stock, metres for roll stock. Must be greater than zero." promptTitle="Quantity" prompt="Sheets for sheet stock, metres for roll stock. Must be greater than zero." sqref="H28:H2010" xr:uid="{00000000-0002-0000-0900-000005000000}">
+    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle="Qty" error="Sheets for sheet stock, metres for roll stock. Must be greater than zero." promptTitle="Qty" prompt="Sheets for sheet stock, metres for roll stock. Must be greater than zero." sqref="H18:H29" xr:uid="{0EB6289D-94A2-4A20-A725-132ACF4AC0B0}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Print width" error="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." promptTitle="Print width" prompt="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." sqref="I28:I2010" xr:uid="{00000000-0002-0000-0900-000006000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Print width" error="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." promptTitle="Print width" prompt="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width. Required for 'Supplied (Roll)'." sqref="I18:I29" xr:uid="{1894B910-050C-4C3A-8489-9F7A13C9685D}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date and time" error="Date and time the print was produced. Use the Now button to stamp the current date and time." promptTitle="Date and time" prompt="Date and time the print was produced. Use the Now button to stamp the current date and time." sqref="A16:A2010" xr:uid="{00000000-0002-0000-0900-000007000000}">
-      <formula1>36526</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J28:K2010 K16:K27 L16:L27" xr:uid="{00000000-0002-0000-0900-000003000000}">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Roll length unit" error="Choose Metres or Centimetres." promptTitle="Roll length unit" prompt="How a roll job's length is typed into Qty on this sheet. Always converted to, and stored as, metres regardless of this setting - Sheet stock is unaffected." sqref="B9" xr:uid="{DDF6FDDC-C744-4D90-987F-9EBAA10EE831}">
-      <formula1>"Metres,Centimetres"</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle="Qty" error="Sheets for sheet stock, metres for roll stock. Must be greater than zero." promptTitle="Qty" prompt="Sheets for sheet stock, metres for roll stock. Must be greater than zero." sqref="H16:H27" xr:uid="{0EB6289D-94A2-4A20-A725-132ACF4AC0B0}">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Print width" error="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." promptTitle="Print width" prompt="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width. Required for 'Supplied (Roll)'." sqref="I16:I27" xr:uid="{1894B910-050C-4C3A-8489-9F7A13C9685D}">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Sheet size" error="Choose one of the standard sizes listed on Settings." promptTitle="Sheet size" prompt="Required only for 'Supplied (Sheet)' - the nearest standard size to the sheet the student brought. Ignored for every other paper stock." sqref="J16:J27" xr:uid="{974A2940-850F-46E7-B729-C14D6A820BB6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Sheet size" error="Choose one of the standard sizes listed on Settings." promptTitle="Sheet size" prompt="Required only for 'Supplied (Sheet)' - the nearest standard size to the sheet the student brought. Ignored for every other paper stock." sqref="J18:J29" xr:uid="{974A2940-850F-46E7-B729-C14D6A820BB6}">
       <formula1>RNG_STD_SIZES</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paid" error="Choose Yes or No." promptTitle="Paid" prompt="Whether this chargeable cost has been paid. Blank means not recorded either way and counts as unpaid in totals." sqref="S16:S27" xr:uid="{A827598F-CA17-4532-A2B4-E4329BE2650A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paid" error="Choose Yes or No." promptTitle="Paid" prompt="Whether this chargeable cost has been paid. Blank means not recorded either way and counts as unpaid in totals." sqref="S18:S29" xr:uid="{A827598F-CA17-4532-A2B4-E4329BE2650A}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4250,103 +4287,103 @@
           <x14:formula1>
             <xm:f>_Work!$G$2:$G$4</xm:f>
           </x14:formula1>
-          <xm:sqref>D16:D27</xm:sqref>
+          <xm:sqref>D18:D29</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="Choose one of the listed options. Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family HP Latex 335 supports - picking one clears the printer instead." promptTitle="Paper stock" prompt="Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family HP Latex 335 supports - picking one clears the printer instead." xr:uid="{C8525DE8-70D2-4939-AE53-09B8E996F529}">
           <x14:formula1>
             <xm:f>_Work!$J$2:$J$12</xm:f>
           </x14:formula1>
-          <xm:sqref>F22</xm:sqref>
+          <xm:sqref>F24</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="Choose one of the listed options. Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family HP DesignJet Z9+ supports - picking one clears the printer instead." promptTitle="Paper stock" prompt="Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family HP DesignJet Z9+ supports - picking one clears the printer instead." xr:uid="{804CCC33-3817-4F3E-94F4-8A56C88B24CB}">
           <x14:formula1>
             <xm:f>_Work!$K$2:$K$12</xm:f>
           </x14:formula1>
-          <xm:sqref>F23</xm:sqref>
+          <xm:sqref>F25</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="Choose one of the listed options. Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family Xerox Versant 180 supports - picking one clears the printer instead." promptTitle="Paper stock" prompt="Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family Xerox Versant 180 supports - picking one clears the printer instead." xr:uid="{4A0AEE34-9D74-46CA-A391-1496C855AAAF}">
           <x14:formula1>
             <xm:f>_Work!$L$2:$L$12</xm:f>
           </x14:formula1>
-          <xm:sqref>F16 F20:F21 F24 F26</xm:sqref>
+          <xm:sqref>F18 F22:F23 F26 F28</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="Choose one of the listed options. Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family Epson SureColor P9500 supports - picking one clears the printer instead." promptTitle="Paper stock" prompt="Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family Epson SureColor P9500 supports - picking one clears the printer instead." xr:uid="{32B928B8-1766-4CED-B621-7AB9984EA332}">
           <x14:formula1>
             <xm:f>_Work!$M$2:$M$12</xm:f>
           </x14:formula1>
-          <xm:sqref>F17:F19 F25 F27</xm:sqref>
+          <xm:sqref>F19:F21 F27 F29</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Gloss 200gsm SRA3 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Gloss 200gsm SRA3 sheet' - picking one clears the paper stock instead." xr:uid="{3D72609D-7821-40D1-B4E0-9A17A762D7B9}">
           <x14:formula1>
             <xm:f>_Work!$N$2:$N$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E16</xm:sqref>
+          <xm:sqref>E18</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Uncoated 120gsm A3 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Uncoated 120gsm A3 sheet' - picking one clears the paper stock instead." xr:uid="{ADA2925B-D9CE-483D-A3CB-F6887904EC42}">
           <x14:formula1>
             <xm:f>_Work!$O$2:$O$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E20</xm:sqref>
+          <xm:sqref>E22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Gloss offcut 320x450 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Gloss offcut 320x450 sheet' - picking one clears the paper stock instead." xr:uid="{012D11A0-C356-4599-BC4D-DC0EE936279D}">
           <x14:formula1>
             <xm:f>_Work!$P$2:$P$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E21</xm:sqref>
+          <xm:sqref>E23</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Vinyl self-adhesive 1370mm roll' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Vinyl self-adhesive 1370mm roll' - picking one clears the paper stock instead." xr:uid="{8B127D0B-FEBC-4EAD-9A1C-1213E7673F7A}">
           <x14:formula1>
             <xm:f>_Work!$Q$2:$Q$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E22</xm:sqref>
+          <xm:sqref>E24</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Satin photo 610mm roll' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Satin photo 610mm roll' - picking one clears the paper stock instead." xr:uid="{9C71BD25-2544-420E-9FD9-6BBB323309B0}">
           <x14:formula1>
             <xm:f>_Work!$R$2:$R$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E19 E23</xm:sqref>
+          <xm:sqref>E21 E25</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm A2 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm A2 sheet' - picking one clears the paper stock instead." xr:uid="{67197FBA-1C2E-4D3C-ACB9-817976B15DF1}">
           <x14:formula1>
             <xm:f>_Work!$S$2:$S$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E24</xm:sqref>
+          <xm:sqref>E26</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm 1067mm roll' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm 1067mm roll' - picking one clears the paper stock instead." xr:uid="{8CFA56E2-9A8D-460B-A5B6-7BDFEC59376E}">
           <x14:formula1>
             <xm:f>_Work!$T$2:$T$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E25</xm:sqref>
+          <xm:sqref>E27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm A1 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm A1 sheet' - picking one clears the paper stock instead." xr:uid="{D369D7DE-B42A-4E5A-915B-58A90399AD45}">
           <x14:formula1>
             <xm:f>_Work!$U$2:$U$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E26</xm:sqref>
+          <xm:sqref>E28</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Canvas 914mm roll' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Canvas 914mm roll' - picking one clears the paper stock instead." xr:uid="{C4698F5D-DDE1-4E72-8DD1-0CFA5F7A883D}">
           <x14:formula1>
             <xm:f>_Work!$V$2:$V$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E17:E18 E27</xm:sqref>
+          <xm:sqref>E19:E20 E29</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Default technician" error="Choose one of the listed options. Pre-fills each new print job's Technician until Clear defaults is used." promptTitle="Default technician" prompt="Pre-fills each new print job's Technician until Clear defaults is used." xr:uid="{4692C48D-8984-4261-BBD5-05992933E720}">
           <x14:formula1>
             <xm:f>_Work!$G$2:$G$4</xm:f>
           </x14:formula1>
-          <xm:sqref>B3</xm:sqref>
+          <xm:sqref>B4</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="Choose one of the listed options. Every active stock compatible with a printer at this print room." promptTitle="Paper stock" prompt="Every active stock compatible with a printer at this print room." xr:uid="{A7A0E1B4-A8AC-413E-87D0-F11BD62E60D6}">
           <x14:formula1>
             <xm:f>_Work!$H$2:$H$12</xm:f>
           </x14:formula1>
-          <xm:sqref>B5</xm:sqref>
+          <xm:sqref>B6</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room." promptTitle="Printer" prompt="Every active printer permitted at this print room." xr:uid="{F880BA63-A334-4F88-A95C-6BF163632FD8}">
           <x14:formula1>
             <xm:f>_Work!$I$2:$I$4</xm:f>
           </x14:formula1>
-          <xm:sqref>B4</xm:sqref>
+          <xm:sqref>B5</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4366,11 +4403,11 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4389,20 +4426,20 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>19</v>
@@ -4412,9 +4449,11 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="30"/>
+      <c r="A7" s="30" t="s">
+        <v>259</v>
+      </c>
       <c r="B7" s="24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>20</v>
@@ -4424,9 +4463,11 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="30"/>
+      <c r="A8" s="30" t="s">
+        <v>260</v>
+      </c>
       <c r="B8" s="24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>20</v>
@@ -4436,19 +4477,21 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="30"/>
+      <c r="A9" s="30" t="s">
+        <v>261</v>
+      </c>
       <c r="B9" s="24" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D9" s="24" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Active" error="Set to No to retire a technician. Existing records keep working; the name stops appearing for new print jobs." promptTitle="Active" prompt="Set to No to retire a technician. Existing records keep working; the name stops appearing for new print jobs." sqref="D7:D2001" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Yes,No"</formula1>
@@ -4477,17 +4520,17 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="H4" s="2" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -4495,31 +4538,33 @@
     </row>
     <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="30"/>
+      <c r="A7" s="30" t="s">
+        <v>262</v>
+      </c>
       <c r="B7" s="24" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>58</v>
@@ -4536,9 +4581,11 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="30"/>
+      <c r="A8" s="30" t="s">
+        <v>263</v>
+      </c>
       <c r="B8" s="24" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>58</v>
@@ -4555,9 +4602,11 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="30"/>
+      <c r="A9" s="30" t="s">
+        <v>264</v>
+      </c>
       <c r="B9" s="24" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>59</v>
@@ -4574,9 +4623,11 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="30"/>
+      <c r="A10" s="30" t="s">
+        <v>265</v>
+      </c>
       <c r="B10" s="24" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>61</v>
@@ -4593,7 +4644,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <phoneticPr fontId="11" type="noConversion"/>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C2001" xr:uid="{00000000-0002-0000-0200-000000000000}">
@@ -4622,7 +4673,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.7265625" customWidth="1"/>
@@ -4639,17 +4690,17 @@
   <sheetData>
     <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="M4" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -4657,22 +4708,22 @@
     </row>
     <row r="6" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>48</v>
@@ -4681,22 +4732,24 @@
         <v>49</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>36</v>
       </c>
       <c r="L6" s="22" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" s="30"/>
+      <c r="A7" s="30" t="s">
+        <v>266</v>
+      </c>
       <c r="B7" s="24" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>40</v>
@@ -4705,7 +4758,7 @@
         <v>44</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F7" s="24" t="s">
         <v>51</v>
@@ -4727,13 +4780,15 @@
         <v>38</v>
       </c>
       <c r="L7" s="25" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" s="30"/>
+      <c r="A8" s="30" t="s">
+        <v>267</v>
+      </c>
       <c r="B8" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>40</v>
@@ -4742,7 +4797,7 @@
         <v>44</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F8" s="24" t="s">
         <v>52</v>
@@ -4764,13 +4819,15 @@
         <v>38</v>
       </c>
       <c r="L8" s="25" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" s="30"/>
+      <c r="A9" s="30" t="s">
+        <v>268</v>
+      </c>
       <c r="B9" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>39</v>
@@ -4779,7 +4836,7 @@
         <v>44</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F9" s="24" t="s">
         <v>55</v>
@@ -4801,13 +4858,15 @@
         <v>38</v>
       </c>
       <c r="L9" s="25" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="30"/>
+      <c r="A10" s="30" t="s">
+        <v>269</v>
+      </c>
       <c r="B10" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>43</v>
@@ -4816,7 +4875,7 @@
         <v>44</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F10" s="24" t="s">
         <v>53</v>
@@ -4838,13 +4897,15 @@
         <v>38</v>
       </c>
       <c r="L10" s="25" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" s="30"/>
+      <c r="A11" s="30" t="s">
+        <v>270</v>
+      </c>
       <c r="B11" s="24" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>42</v>
@@ -4871,13 +4932,15 @@
         <v>38</v>
       </c>
       <c r="L11" s="25" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A12" s="30"/>
+      <c r="A12" s="30" t="s">
+        <v>271</v>
+      </c>
       <c r="B12" s="24" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>41</v>
@@ -4904,13 +4967,15 @@
         <v>38</v>
       </c>
       <c r="L12" s="25" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13" s="30"/>
+      <c r="A13" s="30" t="s">
+        <v>272</v>
+      </c>
       <c r="B13" s="24" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>37</v>
@@ -4937,13 +5002,15 @@
         <v>38</v>
       </c>
       <c r="L13" s="25" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" s="30"/>
+      <c r="A14" s="30" t="s">
+        <v>273</v>
+      </c>
       <c r="B14" s="24" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>40</v>
@@ -4970,13 +5037,15 @@
         <v>38</v>
       </c>
       <c r="L14" s="25" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A15" s="30"/>
+      <c r="A15" s="30" t="s">
+        <v>274</v>
+      </c>
       <c r="B15" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>39</v>
@@ -4985,7 +5054,7 @@
         <v>44</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F15" s="24"/>
       <c r="G15" s="8">
@@ -5005,95 +5074,37 @@
         <v>38</v>
       </c>
       <c r="L15" s="25" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A16" s="30"/>
-      <c r="B16" s="24" t="s">
-        <v>232</v>
-      </c>
-      <c r="C16" s="24" t="s">
-        <v>233</v>
-      </c>
-      <c r="D16" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="10">
-        <v>0</v>
-      </c>
-      <c r="J16" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
-        <v>£ per metre</v>
-      </c>
-      <c r="K16" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="L16" s="25" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A17" s="30"/>
-      <c r="B17" s="24" t="s">
-        <v>234</v>
-      </c>
-      <c r="C17" s="24" t="s">
-        <v>233</v>
-      </c>
-      <c r="D17" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="10">
-        <v>0</v>
-      </c>
-      <c r="J17" s="20" t="str">
-        <f>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</f>
-        <v>£ per sheet</v>
-      </c>
-      <c r="K17" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="L17" s="25" t="s">
-        <v>38</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Supplied by student" error="Choose Yes or No." promptTitle="Supplied by student" prompt="Yes only for the two 'Supplied' catalogue rows - paper cost always computes to zero for these regardless of Cost." sqref="L7:L17" xr:uid="{2ED70CBA-D9C3-4CB5-A147-78652DAACDC7}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Supplied by student" error="Choose Yes or No." promptTitle="Supplied by student" prompt="Yes only for the two 'Supplied' catalogue rows - paper cost always computes to zero for these regardless of Cost." sqref="L7:L15" xr:uid="{2ED70CBA-D9C3-4CB5-A147-78652DAACDC7}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C2003" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C2001" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>lstPaperTypes</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Measure" error="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." promptTitle="Measure" prompt="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." sqref="D7:D2003" xr:uid="{00000000-0002-0000-0300-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Measure" error="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." promptTitle="Measure" prompt="Sheet stock is counted in sheets; roll stock is counted in metres. This choice drives how the workbook measures and prices the stock." sqref="D7:D2001" xr:uid="{00000000-0002-0000-0300-000001000000}">
       <formula1>"Sheet,Roll"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Size mode" error="Standard fills the size from the standard sizes list. Custom sheet takes width and height directly. Roll takes the roll width only." promptTitle="Size mode" prompt="Standard fills the size from the standard sizes list. Custom sheet takes width and height directly. Roll takes the roll width only." sqref="E7:E2003" xr:uid="{00000000-0002-0000-0300-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Size mode" error="Standard fills the size from the standard sizes list. Custom sheet takes width and height directly. Roll takes the roll width only." promptTitle="Size mode" prompt="Standard fills the size from the standard sizes list. Custom sheet takes width and height directly. Roll takes the roll width only." sqref="E7:E2001" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>"Standard,Custom sheet,Roll"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7:F2003" xr:uid="{00000000-0002-0000-0300-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7:F2001" xr:uid="{00000000-0002-0000-0300-000003000000}">
       <formula1>lstStandardSizes</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres. For roll stock, enter the roll width only." promptTitle="Dimension" prompt="Enter the size in millimetres. For roll stock, enter the roll width only." sqref="G7:G2003" xr:uid="{00000000-0002-0000-0300-000004000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres. For roll stock, enter the roll width only." promptTitle="Dimension" prompt="Enter the size in millimetres. For roll stock, enter the roll width only." sqref="G7:G2001" xr:uid="{00000000-0002-0000-0300-000004000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres." promptTitle="Dimension" prompt="Enter the size in millimetres." sqref="H7:H2003" xr:uid="{00000000-0002-0000-0300-000005000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres." promptTitle="Dimension" prompt="Enter the size in millimetres." sqref="H7:H2001" xr:uid="{00000000-0002-0000-0300-000005000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Cost" error="Cost per sheet for sheet stock, or cost per metre for roll stock. The Cost unit column shows which applies." promptTitle="Cost" prompt="Cost per sheet for sheet stock, or cost per metre for roll stock. The Cost unit column shows which applies." sqref="I7:I2003" xr:uid="{00000000-0002-0000-0300-000006000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Cost" error="Cost per sheet for sheet stock, or cost per metre for roll stock. The Cost unit column shows which applies." promptTitle="Cost" prompt="Cost per sheet for sheet stock, or cost per metre for roll stock. The Cost unit column shows which applies." sqref="I7:I2001" xr:uid="{00000000-0002-0000-0300-000006000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K7:K2003" xr:uid="{00000000-0002-0000-0300-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K7:K2001" xr:uid="{00000000-0002-0000-0300-000007000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5107,7 +5118,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
@@ -5132,195 +5143,102 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="P2" s="3" t="s">
-        <v>62</v>
-      </c>
+      <c r="P2" s="3"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="P3" s="2" t="s">
-        <v>63</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="P3" s="3"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2"/>
+      <c r="P4" s="3"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A5" s="2"/>
+      <c r="P5" s="3"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P6" s="2"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M7" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I8" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J8" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K8" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M8" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="N8" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="5" t="s">
+    <row r="9" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D9" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F9" s="24" t="s">
         <v>37</v>
-      </c>
-      <c r="G6" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="8">
-        <v>841</v>
-      </c>
-      <c r="K6" s="8">
-        <v>1189</v>
-      </c>
-      <c r="M6" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="N6" s="24" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="26"/>
-      <c r="F7" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="I7" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="J7" s="8">
-        <v>594</v>
-      </c>
-      <c r="K7" s="8">
-        <v>841</v>
-      </c>
-      <c r="M7" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="N7" s="24" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="I8" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="J8" s="8">
-        <v>420</v>
-      </c>
-      <c r="K8" s="8">
-        <v>594</v>
-      </c>
-      <c r="M8" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="N8" s="24" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="26"/>
-      <c r="F9" s="24" t="s">
-        <v>41</v>
       </c>
       <c r="G9" s="24" t="s">
         <v>38</v>
       </c>
       <c r="I9" s="24" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="J9" s="8">
-        <v>297</v>
+        <v>841</v>
       </c>
       <c r="K9" s="8">
-        <v>420</v>
+        <v>1189</v>
       </c>
       <c r="M9" s="24" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="N9" s="24" t="s">
         <v>38</v>
@@ -5328,229 +5246,364 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>24</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="D10" s="26"/>
       <c r="F10" s="24" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G10" s="24" t="s">
         <v>38</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="J10" s="8">
-        <v>210</v>
+        <v>594</v>
       </c>
       <c r="K10" s="8">
-        <v>297</v>
+        <v>841</v>
+      </c>
+      <c r="M10" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="N10" s="24" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="7">
-        <v>2</v>
+        <v>15</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G11" s="24" t="s">
         <v>38</v>
       </c>
       <c r="I11" s="24" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="J11" s="8">
-        <v>320</v>
+        <v>420</v>
       </c>
       <c r="K11" s="8">
-        <v>450</v>
+        <v>594</v>
+      </c>
+      <c r="M11" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="N11" s="24" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="40">
-        <v>1.2</v>
-      </c>
-      <c r="D12" s="26" t="s">
-        <v>30</v>
+        <v>19</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="26"/>
+      <c r="F12" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="I12" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" s="8">
+        <v>297</v>
+      </c>
+      <c r="K12" s="8">
+        <v>420</v>
+      </c>
+      <c r="M12" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="N12" s="24" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="43">
-        <v>46294.403460648151</v>
+        <v>22</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>33</v>
+        <v>24</v>
+      </c>
+      <c r="F13" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="G13" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="I13" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="J13" s="8">
+        <v>210</v>
+      </c>
+      <c r="K13" s="8">
+        <v>297</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>204</v>
+        <v>25</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="C14" s="40" t="s">
-        <v>213</v>
+        <v>26</v>
+      </c>
+      <c r="C14" s="7">
+        <v>2</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>206</v>
+        <v>27</v>
+      </c>
+      <c r="F14" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="I14" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="J14" s="8">
+        <v>320</v>
+      </c>
+      <c r="K14" s="8">
+        <v>450</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>207</v>
+        <v>28</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="C15" s="43">
-        <v>46294.403460648151</v>
+        <v>29</v>
+      </c>
+      <c r="C15" s="40">
+        <v>1.3</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>209</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>210</v>
+        <v>31</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="C16" s="40" t="s">
-        <v>247</v>
+        <v>32</v>
+      </c>
+      <c r="C16" s="43">
+        <v>46294.403460648151</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="C17" s="7"/>
+        <v>201</v>
+      </c>
+      <c r="C17" s="40" t="s">
+        <v>245</v>
+      </c>
       <c r="D17" s="26" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>217</v>
+        <v>203</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>132</v>
+        <v>204</v>
+      </c>
+      <c r="C18" s="43">
+        <v>46294.403460648151</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>223</v>
+        <v>207</v>
+      </c>
+      <c r="C19" s="40" t="s">
+        <v>235</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>132</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="C20" s="7"/>
       <c r="D20" s="26" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="D21" s="26" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="D22" s="26" t="s">
         <v>249</v>
       </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="26" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
+    </row>
+    <row r="23" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B23" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="C22" s="48"/>
-      <c r="D22" s="26" t="s">
+      <c r="C23" s="48" t="s">
+        <v>254</v>
+      </c>
+      <c r="D23" s="26" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A23" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="B23" s="6" t="s">
+    <row r="24" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="D24" s="26" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A25" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C25" s="48">
+        <v>3</v>
+      </c>
+      <c r="D25" s="26" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A26" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="C26" s="48">
+        <v>4</v>
+      </c>
+      <c r="D26" s="26" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="C27" s="48">
+        <v>9</v>
+      </c>
+      <c r="D27" s="26" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="C23" s="48"/>
-      <c r="D23" s="26" t="s">
+      <c r="B28" s="6" t="s">
         <v>256</v>
       </c>
+      <c r="C28" s="48" t="s">
+        <v>258</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>257</v>
+      </c>
     </row>
   </sheetData>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G6:G2000 N6:N2000" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G9:G2003 N9:N2003" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres." promptTitle="Dimension" prompt="Enter the size in millimetres." sqref="J6:K2000" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres." promptTitle="Dimension" prompt="Enter the size in millimetres." sqref="J9:K2003" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -5584,48 +5637,48 @@
   <sheetData>
     <row r="1" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>122</v>
-      </c>
       <c r="I1" s="22" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="J1" s="22" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="K1" s="22" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="22" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D2" s="22" t="s">
         <v>20</v>
@@ -5647,7 +5700,7 @@
       <c r="K2" s="22"/>
     </row>
   </sheetData>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -5661,7 +5714,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5672,7 +5725,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5685,23 +5738,23 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>127</v>
-      </c>
     </row>
   </sheetData>
-  <sheetProtection formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
0.10.25: Reports Go to record, Clear all filters, Toggle Paid, new filters
- Reports: Go to record, Clear all filters, Has notes and Min/Max cost
  filters; header buttons drawn and kept in place like the room sheets'.
- Paid on Reports is now changed with a Toggle Paid button acting on the
  selected row(s); the Paid cells are read-only. In-place editing is gone
  because Excel for Mac delivers no VBA callbacks after a dropdown pick until
  the next click, leaving the spilled table blank (#SPILL!).
- Fix Delete visible records after a file rename (button names / HealButtons).
- Mac notice before restoring from an older workbook; column widths follow
  PrintCosts.xlsx; tests updated (test-togglepaid, test-reportsnav,
  test-summaryformat renamed from test-phase8).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NAQB3F5peB8rQeTpNgXCTe
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -2732,18 +2732,18 @@
     <col min="5" max="5" width="24.7265625" customWidth="1"/>
     <col min="6" max="6" width="30.7265625" customWidth="1"/>
     <col min="7" max="8" width="7.08984375" customWidth="1"/>
-    <col min="9" max="9" width="17.08984375" customWidth="1"/>
-    <col min="10" max="10" width="15.7265625" customWidth="1"/>
-    <col min="11" max="12" width="18.453125" customWidth="1"/>
+    <col min="9" max="9" width="12.86" customWidth="1"/>
+    <col min="10" max="10" width="10.71" customWidth="1"/>
+    <col min="11" max="12" width="14.29" customWidth="1"/>
     <col min="13" max="13" width="8.453125" customWidth="1"/>
-    <col min="14" max="14" width="15.7265625" customWidth="1"/>
+    <col min="14" max="14" width="12.86" customWidth="1"/>
     <col min="15" max="16" width="12.7265625" customWidth="1"/>
-    <col min="17" max="17" width="15.7265625" customWidth="1"/>
-    <col min="18" max="18" width="30.7265625" customWidth="1"/>
+    <col min="17" max="17" width="14.29" customWidth="1"/>
+    <col min="18" max="18" width="14.29" customWidth="1"/>
     <col min="19" max="19" width="5.6328125" customWidth="1"/>
-    <col min="20" max="20" width="34.7265625" customWidth="1"/>
+    <col min="20" max="20" width="12.86" customWidth="1"/>
     <col min="21" max="21" width="14.1796875" customWidth="1"/>
-    <col min="22" max="22" width="11.7265625" customWidth="1" collapsed="1"/>
+    <col min="22" max="22" width="42.86" customWidth="1" collapsed="1"/>
     <col min="23" max="24" width="11.7265625" hidden="1" customWidth="1"/>
     <col min="25" max="25" width="13.7265625" hidden="1" customWidth="1"/>
     <col min="26" max="26" width="10.7265625" hidden="1" customWidth="1"/>

</xml_diff>

<commit_message>
0.11.0 (2/7) template: multi-pass columns, printer colour mode, summaryBelow
apply-multipass-template.ps1 is the re-runnable record of the template change
(job table +11 columns, LOC_* block moved to AW:AX, Printers Colour mode and
Template cost, Risograph type, MULTIPASS_COLS_HIDDEN, schema 1.4 stamp).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\claude\C--Users-adash-OneDrive-Development-OfficeApps-PrintJob\97da5acd-fb69-4037-ad89-90b60a7c50c7\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F0EF5AC-E533-4946-8786-E4DD940772F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A63511-F932-4C50-B688-8D925626494D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,18 +25,18 @@
     <sheet name="_Picker" sheetId="9" state="veryHidden" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="LOC_Code" localSheetId="0">'Example Print Room'!$AM$2</definedName>
+    <definedName name="LOC_Code" localSheetId="0">'Example Print Room'!$AX$2</definedName>
     <definedName name="LOC_DefDisCons" localSheetId="0">'Example Print Room'!$B$9</definedName>
     <definedName name="LOC_DefDisPaper" localSheetId="0">'Example Print Room'!$B$8</definedName>
     <definedName name="LOC_DefPaper" localSheetId="0">'Example Print Room'!$B$6</definedName>
     <definedName name="LOC_DefPrinter" localSheetId="0">'Example Print Room'!$B$5</definedName>
     <definedName name="LOC_DefTech" localSheetId="0">'Example Print Room'!$B$4</definedName>
     <definedName name="LOC_Dept" localSheetId="0">'Example Print Room'!$B$2</definedName>
-    <definedName name="LOC_Export" localSheetId="0">'Example Print Room'!$AM$8</definedName>
+    <definedName name="LOC_Export" localSheetId="0">'Example Print Room'!$AX$8</definedName>
     <definedName name="LOC_Name" localSheetId="0">'Example Print Room'!$B$1</definedName>
-    <definedName name="LOC_Printers" localSheetId="0">'Example Print Room'!$AM$9</definedName>
+    <definedName name="LOC_Printers" localSheetId="0">'Example Print Room'!$AX$9</definedName>
     <definedName name="LOC_RollUnit" localSheetId="0">'Example Print Room'!$B$11</definedName>
-    <definedName name="LOC_Status" localSheetId="0">'Example Print Room'!$AM$6</definedName>
+    <definedName name="LOC_Status" localSheetId="0">'Example Print Room'!$AX$6</definedName>
     <definedName name="lstConsumables">tblConsumables[Consumable type]</definedName>
     <definedName name="lstPaperTypes">tblPaperTypes[Paper type]</definedName>
     <definedName name="lstPrinters">tblPrinters[Model]</definedName>
@@ -55,15 +55,16 @@
     <definedName name="SET_LOC_MINIMAL_COLUMNS">Settings!$C$23</definedName>
     <definedName name="SET_LOC_REDUCED_COLUMNS">Settings!$C$22</definedName>
     <definedName name="SET_LOC_REDUCED_VIEW">Settings!$C$21</definedName>
+    <definedName name="SET_MULTIPASS_COLS_HIDDEN">Settings!$C$25</definedName>
     <definedName name="SET_ORG">Settings!$C$11</definedName>
-    <definedName name="SET_PRINTER_ID_HWM">Settings!$C$26</definedName>
-    <definedName name="SET_REPORT_HEADING">Settings!$C$28</definedName>
+    <definedName name="SET_PRINTER_ID_HWM">Settings!$C$27</definedName>
+    <definedName name="SET_REPORT_HEADING">Settings!$C$29</definedName>
     <definedName name="SET_ROUND_DP">Settings!$C$14</definedName>
     <definedName name="SET_SCHEMA">Settings!$C$15</definedName>
     <definedName name="SET_SITE_ID">Settings!$C$9</definedName>
     <definedName name="SET_SITE_NAME">Settings!$C$10</definedName>
-    <definedName name="SET_STOCK_ID_HWM">Settings!$C$27</definedName>
-    <definedName name="SET_TECH_ID_HWM">Settings!$C$25</definedName>
+    <definedName name="SET_STOCK_ID_HWM">Settings!$C$28</definedName>
+    <definedName name="SET_TECH_ID_HWM">Settings!$C$26</definedName>
   </definedNames>
   <calcPr calcId="191029" calcOnSave="0"/>
   <extLst>
@@ -83,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="294">
   <si>
     <t>Settings</t>
   </si>
@@ -835,9 +836,6 @@
     <t>Semicolon-separated column headers hidden by the Reduced view. Edit to change what it hides - no rebuild needed. Minimal hides these as well.</t>
   </si>
   <si>
-    <t>Status;Job ID;Area m2;S_SchemaVer</t>
-  </si>
-  <si>
     <t>LOC_MINIMAL_COLUMNS</t>
   </si>
   <si>
@@ -908,6 +906,66 @@
   </si>
   <si>
     <t>UNI-STK-0009</t>
+  </si>
+  <si>
+    <t>Passes</t>
+  </si>
+  <si>
+    <t>Colour</t>
+  </si>
+  <si>
+    <t>Set-up Cost</t>
+  </si>
+  <si>
+    <t>Row Type</t>
+  </si>
+  <si>
+    <t>Parent</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>H_Ink</t>
+  </si>
+  <si>
+    <t>H_Setup</t>
+  </si>
+  <si>
+    <t>H_Notices</t>
+  </si>
+  <si>
+    <t>S_SetupCost</t>
+  </si>
+  <si>
+    <t>S_ColourID</t>
+  </si>
+  <si>
+    <t>Job</t>
+  </si>
+  <si>
+    <t>Colour mode</t>
+  </si>
+  <si>
+    <t>Template cost</t>
+  </si>
+  <si>
+    <t>single pass</t>
+  </si>
+  <si>
+    <t>Risograph</t>
+  </si>
+  <si>
+    <t>MULTIPASS_COLS_HIDDEN</t>
+  </si>
+  <si>
+    <t>Hide multi-pass columns</t>
+  </si>
+  <si>
+    <t>Yes hides the multi-pass columns (Passes, Colour, Row Type, Parent, Pass) on every location sheet (toggled by the button on each one). No shows them. The Set-up Cost column belongs to the cost detail setting instead.</t>
+  </si>
+  <si>
+    <t>Status;Job ID;Area m2;S_SchemaVer;Passes;Colour;Row Type;Parent;Pass</t>
   </si>
 </sst>
 </file>
@@ -1210,7 +1268,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1365,17 +1423,400 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="77">
+  <dxfs count="90">
     <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <right style="medium">
+          <color rgb="FFBFBFBF"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="#,##0.###"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
@@ -1632,17 +2073,6 @@
       <font>
         <color rgb="FF808080"/>
       </font>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFD9D9D9"/>
@@ -1719,24 +2149,6 @@
           <bgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -1843,34 +2255,6 @@
         <i/>
         <color rgb="FF595959"/>
       </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
       <numFmt numFmtId="167" formatCode="#,##0.000"/>
       <fill>
         <patternFill patternType="solid">
@@ -1997,26 +2381,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -2241,61 +2605,80 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_MAIN" displayName="tblJobs_MAIN" ref="A17:AH29" totalsRowShown="0">
-  <autoFilter ref="A17:AH29" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
-  <tableColumns count="34">
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Date/Time" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Student No" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="Technician" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_MAIN" displayName="tblJobs_MAIN" ref="A17:AS29" totalsRowShown="0">
+  <autoFilter ref="A17:AS29" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
+  <tableColumns count="45">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Date/Time" dataDxfId="75"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="74"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Student No" dataDxfId="73"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="Technician" dataDxfId="72"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="14"/>
+    <tableColumn id="25" xr3:uid="{09F3ECAE-609E-455B-9BA8-2E241E8FAF46}" name="Passes" dataDxfId="12">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="36" xr3:uid="{3444712F-EA34-42DA-B9B5-0EBBE8952B8B}" name="Colour" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="71"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="70">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Qty" dataDxfId="55"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Print Width mm" dataDxfId="54"/>
-    <tableColumn id="35" xr3:uid="{E6BF4E83-281D-4CCB-8342-85AB57046527}" name="Sheet size" dataDxfId="53"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Disregard Paper" dataDxfId="52"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Disregard Consumable" dataDxfId="51"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Area m2" dataDxfId="50">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Qty" dataDxfId="69"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Print Width mm" dataDxfId="68"/>
+    <tableColumn id="35" xr3:uid="{E6BF4E83-281D-4CCB-8342-85AB57046527}" name="Sheet size" dataDxfId="67"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Disregard Paper" dataDxfId="66"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Disregard Consumable" dataDxfId="65"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Area m2" dataDxfId="64">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="49">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="63">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="48">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</calculatedColumnFormula>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="8">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="47">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</calculatedColumnFormula>
+    <tableColumn id="37" xr3:uid="{9D5B92B2-8D8C-4AB8-B4C8-729D5FEC16B3}" name="Set-up Cost" dataDxfId="6">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Disregarded" dataDxfId="46">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="7">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Disregarded" dataDxfId="62">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" name="Chargeable Cost" dataDxfId="45">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</calculatedColumnFormula>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" name="Chargeable Cost" dataDxfId="61">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="34" xr3:uid="{9C12E379-305A-4AA1-8D70-0BFC2C6CF3C5}" name="Paid" dataDxfId="44"/>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Status" dataDxfId="43">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</calculatedColumnFormula>
+    <tableColumn id="34" xr3:uid="{9C12E379-305A-4AA1-8D70-0BFC2C6CF3C5}" name="Paid" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Status" dataDxfId="59">
+      <calculatedColumnFormula>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Job ID" dataDxfId="42"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="41"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="40">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Job ID" dataDxfId="58"/>
+    <tableColumn id="38" xr3:uid="{4D2F43D5-36A3-4912-BABA-E130C7C2146E}" name="Row Type" dataDxfId="18"/>
+    <tableColumn id="39" xr3:uid="{5A1BB7C9-ECFF-4CC8-8500-3A293A25528C}" name="Parent" dataDxfId="11"/>
+    <tableColumn id="40" xr3:uid="{3E507CE4-6A67-46A5-BB60-7B729C2D5A26}" name="Pass" dataDxfId="9"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="10"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="57">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="39"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="38"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="37"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="36"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="35"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="34"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="33"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="32"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="31"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="30"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="29"/>
+    <tableColumn id="41" xr3:uid="{82AE4E46-EF17-494F-A090-ADA99BEE4E30}" name="H_Ink" dataDxfId="17">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="42" xr3:uid="{7A8AEB6A-0F1F-4F77-9521-2D3285156496}" name="H_Setup" dataDxfId="16">
+      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="43" xr3:uid="{4F21AC66-121A-48B2-991A-1B25B7F679A0}" name="H_Notices" dataDxfId="15"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="56"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="55"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="54"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="53"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="52"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="51"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="50"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="5"/>
+    <tableColumn id="44" xr3:uid="{473158C1-5A71-4BCD-9231-D8A93A8E6E06}" name="S_SetupCost" dataDxfId="3"/>
+    <tableColumn id="45" xr3:uid="{AE04C717-F979-427D-9DE7-1B4ED6904D05}" name="S_ColourID" dataDxfId="4"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="49"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="48"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2316,99 +2699,101 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblTechnicians" displayName="tblTechnicians" ref="A6:D9" totalsRowShown="0" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblTechnicians" displayName="tblTechnicians" ref="A6:D9" totalsRowShown="0" dataDxfId="46">
   <autoFilter ref="A6:D9" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Name" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Department" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Active" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Name" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Department" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Active" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblPrinters" displayName="tblPrinters" ref="A6:G10" totalsRowShown="0" dataDxfId="23">
-  <autoFilter ref="A6:G10" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Model" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Consumable type" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{27EBC752-1CF1-48B9-B798-05BFAB38AF84}" name="Max roll width mm" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{78D66AB2-9A7B-410A-92C1-2CCFD2C22414}" name="Max sheet size" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Active" dataDxfId="16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblPrinters" displayName="tblPrinters" ref="A6:I10" totalsRowShown="0" dataDxfId="41">
+  <autoFilter ref="A6:I10" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Model" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Consumable type" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{15CEC00B-A782-4C1F-9D8C-FC4996A5205D}" name="Colour mode" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{59F8E22B-28C7-46F1-991A-38D5C4091FF4}" name="Template cost" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{27EBC752-1CF1-48B9-B798-05BFAB38AF84}" name="Max roll width mm" dataDxfId="36"/>
+    <tableColumn id="8" xr3:uid="{78D66AB2-9A7B-410A-92C1-2CCFD2C22414}" name="Max sheet size" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Active" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:L15" totalsRowShown="0" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:L15" totalsRowShown="0" dataDxfId="33">
   <autoFilter ref="A6:L15" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Description" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Paper type" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Measure" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Size mode" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Std. size" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Width mm" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Height mm" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Cost" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Cost unit" dataDxfId="5">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Description" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Paper type" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Measure" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Size mode" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Std. size" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Width mm" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Height mm" dataDxfId="25"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Cost" dataDxfId="24"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Cost unit" dataDxfId="23">
       <calculatedColumnFormula>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Active" dataDxfId="4"/>
-    <tableColumn id="13" xr3:uid="{62AE4E30-01F2-4D26-B1F8-C8FD5BF6FCC9}" name="Supplied by student" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Active" dataDxfId="22"/>
+    <tableColumn id="13" xr3:uid="{62AE4E30-01F2-4D26-B1F8-C8FD5BF6FCC9}" name="Supplied by student" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A8:D28" totalsRowShown="0">
-  <autoFilter ref="A8:D28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSettings" displayName="tblSettings" ref="A8:D29" totalsRowShown="0">
+  <autoFilter ref="A8:D29" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key" dataDxfId="76"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Setting" dataDxfId="75"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Value" dataDxfId="74"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Notes" dataDxfId="73"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Key" dataDxfId="89"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Setting" dataDxfId="88"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Value" dataDxfId="87"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Notes" dataDxfId="86"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblPaperTypes" displayName="tblPaperTypes" ref="F8:G14" totalsRowShown="0" dataDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblPaperTypes" displayName="tblPaperTypes" ref="F8:G14" totalsRowShown="0" dataDxfId="85">
   <autoFilter ref="F8:G14" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Paper type" dataDxfId="71"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Active" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Paper type" dataDxfId="84"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Active" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="tblStandardSizes" displayName="tblStandardSizes" ref="I8:K14" totalsRowShown="0" dataDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="tblStandardSizes" displayName="tblStandardSizes" ref="I8:K14" totalsRowShown="0" dataDxfId="82">
   <autoFilter ref="I8:K14" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Size name" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Width mm" dataDxfId="67"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Height mm" dataDxfId="66"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Size name" dataDxfId="81"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Width mm" dataDxfId="80"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Height mm" dataDxfId="79"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="tblConsumables" displayName="tblConsumables" ref="M8:N12" totalsRowShown="0" dataDxfId="65">
-  <autoFilter ref="M8:N12" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="tblConsumables" displayName="tblConsumables" ref="M8:N13" totalsRowShown="0" dataDxfId="78">
+  <autoFilter ref="M8:N13" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Consumable type" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Active" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Consumable type" dataDxfId="77"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Active" dataDxfId="76"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2423,8 +2808,8 @@
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Name"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Department"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="Rows"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="First date" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Last date" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="First date" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Last date" dataDxfId="19"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="State"/>
     <tableColumn id="9" xr3:uid="{F307D930-BB9C-468F-AC38-00DA61DF508D}" name="Last export"/>
     <tableColumn id="10" xr3:uid="{B7692E42-45DD-48C6-8B10-C3C464C1B69D}" name="Export sig"/>
@@ -2721,7 +3106,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <sheetPr codeName="Sheet10"/>
+  <sheetPr codeName="Sheet10">
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
   <dimension ref="A1:AZ29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2730,32 +3117,33 @@
     <col min="3" max="3" width="13.7265625" customWidth="1"/>
     <col min="4" max="4" width="18.7265625" customWidth="1"/>
     <col min="5" max="5" width="24.7265625" customWidth="1"/>
-    <col min="6" max="6" width="30.7265625" customWidth="1"/>
-    <col min="7" max="8" width="7.08984375" customWidth="1"/>
-    <col min="9" max="9" width="12.86" customWidth="1"/>
-    <col min="10" max="10" width="10.71" customWidth="1"/>
-    <col min="11" max="12" width="14.29" customWidth="1"/>
-    <col min="13" max="13" width="8.453125" customWidth="1"/>
-    <col min="14" max="14" width="12.86" customWidth="1"/>
-    <col min="15" max="16" width="12.7265625" customWidth="1"/>
-    <col min="17" max="17" width="14.29" customWidth="1"/>
-    <col min="18" max="18" width="14.29" customWidth="1"/>
-    <col min="19" max="19" width="5.6328125" customWidth="1"/>
-    <col min="20" max="20" width="12.86" customWidth="1"/>
-    <col min="21" max="21" width="14.1796875" customWidth="1"/>
-    <col min="22" max="22" width="42.86" customWidth="1" collapsed="1"/>
-    <col min="23" max="24" width="11.7265625" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="13.7265625" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="10.7265625" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="13.7265625" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="14.7265625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="8.1796875" customWidth="1"/>
+    <col min="7" max="7" width="16.6328125" customWidth="1"/>
+    <col min="8" max="8" width="30.7265625" customWidth="1"/>
+    <col min="9" max="10" width="7.08984375" customWidth="1"/>
+    <col min="11" max="11" width="12.81640625" customWidth="1"/>
+    <col min="12" max="12" width="10.7265625" customWidth="1"/>
+    <col min="13" max="14" width="14.26953125" customWidth="1"/>
+    <col min="15" max="15" width="8.453125" customWidth="1"/>
+    <col min="16" max="16" width="12.81640625" customWidth="1"/>
+    <col min="17" max="19" width="12.7265625" customWidth="1"/>
+    <col min="20" max="21" width="14.26953125" customWidth="1"/>
+    <col min="22" max="22" width="5.6328125" customWidth="1" collapsed="1"/>
+    <col min="23" max="23" width="12.81640625" customWidth="1"/>
+    <col min="24" max="24" width="14.1796875" customWidth="1"/>
+    <col min="25" max="25" width="9.1796875" customWidth="1"/>
+    <col min="26" max="26" width="14.6328125" customWidth="1"/>
+    <col min="27" max="27" width="6.6328125" customWidth="1"/>
+    <col min="28" max="28" width="42.81640625" customWidth="1"/>
     <col min="29" max="29" width="12.7265625" hidden="1" customWidth="1"/>
     <col min="30" max="30" width="16.7265625" hidden="1" customWidth="1"/>
     <col min="31" max="31" width="14.7265625" hidden="1" customWidth="1"/>
     <col min="32" max="32" width="11.7265625" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="0" hidden="1" customWidth="1" collapsed="1"/>
-    <col min="34" max="34" width="8.7265625" customWidth="1"/>
-    <col min="36" max="36" width="29.90625" customWidth="1"/>
+    <col min="33" max="33" width="8.7265625" hidden="1" customWidth="1" collapsed="1"/>
+    <col min="34" max="34" width="8.7265625" hidden="1" customWidth="1"/>
+    <col min="35" max="35" width="0" hidden="1" customWidth="1"/>
+    <col min="36" max="36" width="29.90625" hidden="1" customWidth="1"/>
+    <col min="37" max="44" width="0" hidden="1" customWidth="1"/>
     <col min="52" max="52" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2766,7 +3154,7 @@
       <c r="B1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="AL1" s="18" t="s">
+      <c r="AW1" s="18" t="s">
         <v>176</v>
       </c>
       <c r="AZ1" t="s">
@@ -2780,10 +3168,10 @@
       <c r="B2" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="AL2" s="18" t="s">
+      <c r="AW2" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AX2" t="s">
         <v>129</v>
       </c>
     </row>
@@ -2806,10 +3194,10 @@
         <v>227</v>
       </c>
       <c r="B6" s="33"/>
-      <c r="AL6" s="18" t="s">
+      <c r="AW6" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="AM6" t="s">
+      <c r="AX6" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2818,10 +3206,10 @@
       <c r="B8" t="s">
         <v>130</v>
       </c>
-      <c r="AL8" s="42" t="s">
+      <c r="AW8" s="42" t="s">
         <v>233</v>
       </c>
-      <c r="AM8" s="28" t="s">
+      <c r="AX8" s="28" t="s">
         <v>234</v>
       </c>
     </row>
@@ -2829,15 +3217,15 @@
       <c r="B9" t="s">
         <v>130</v>
       </c>
-      <c r="AL9" s="18" t="s">
+      <c r="AW9" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="AM9" t="s">
+      <c r="AX9" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.35">
-      <c r="AL10" s="19" t="s">
+      <c r="AW10" s="19" t="s">
         <v>177</v>
       </c>
     </row>
@@ -2876,7 +3264,7 @@
       <c r="K15" s="29"/>
       <c r="M15" s="2"/>
     </row>
-    <row r="17" spans="1:34" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:45" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>136</v>
       </c>
@@ -2893,94 +3281,127 @@
         <v>140</v>
       </c>
       <c r="F17" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="H17" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="I17" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="J17" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="K17" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="J17" s="23" t="s">
+      <c r="L17" s="23" t="s">
         <v>232</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="M17" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="L17" s="4" t="s">
+      <c r="N17" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="O17" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="N17" s="4" t="s">
+      <c r="P17" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="O17" s="4" t="s">
+      <c r="Q17" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="P17" s="4" t="s">
+      <c r="R17" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="S17" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="Q17" s="4" t="s">
+      <c r="T17" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="R17" s="4" t="s">
+      <c r="U17" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="S17" s="23" t="s">
+      <c r="V17" s="23" t="s">
         <v>223</v>
       </c>
-      <c r="T17" s="4" t="s">
+      <c r="W17" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="U17" s="4" t="s">
+      <c r="X17" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="V17" s="4" t="s">
+      <c r="Y17" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="Z17" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA17" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="AB17" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="W17" s="4" t="s">
+      <c r="AC17" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="X17" s="4" t="s">
+      <c r="AD17" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="AE17" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="AF17" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="AG17" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="Y17" s="4" t="s">
+      <c r="AH17" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="Z17" s="4" t="s">
+      <c r="AI17" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="AA17" s="4" t="s">
+      <c r="AJ17" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="AB17" s="4" t="s">
+      <c r="AK17" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="AC17" s="4" t="s">
+      <c r="AL17" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="AD17" s="4" t="s">
+      <c r="AM17" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="AE17" s="4" t="s">
+      <c r="AN17" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="AF17" s="4" t="s">
+      <c r="AO17" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="AP17" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="AQ17" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="AG17" s="4" t="s">
+      <c r="AR17" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="AH17" s="4" t="s">
+      <c r="AS17" s="4" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
         <v>46280.425000000003</v>
       </c>
@@ -2996,98 +3417,123 @@
       <c r="E18" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="G18" s="9" t="str">
+      <c r="I18" s="9" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
-      <c r="H18" s="13">
+      <c r="J18" s="13">
         <v>100</v>
       </c>
-      <c r="I18" s="36"/>
-      <c r="J18" s="39"/>
-      <c r="K18" s="37" t="s">
+      <c r="K18" s="36"/>
+      <c r="L18" s="39"/>
+      <c r="M18" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="L18" s="12" t="s">
+      <c r="N18" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M18" s="14">
+      <c r="O18" s="14">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>14.400000000000002</v>
       </c>
-      <c r="N18" s="15">
+      <c r="P18" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>31</v>
       </c>
-      <c r="O18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q18" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>13.68</v>
       </c>
-      <c r="P18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R18" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S18" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>44.68</v>
       </c>
-      <c r="Q18" s="15">
+      <c r="T18" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U18" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>44.68</v>
       </c>
-      <c r="S18" s="34"/>
-      <c r="T18" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V18" s="34"/>
+      <c r="W18" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U18" s="5" t="s">
+      <c r="X18" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="V18" s="12" t="s">
+      <c r="Y18" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z18" s="5"/>
+      <c r="AA18" s="49"/>
+      <c r="AB18" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="W18" s="16" t="str">
+      <c r="AC18" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X18" s="16" t="s">
+      <c r="AD18" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE18" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF18" s="16"/>
+      <c r="AG18" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="Y18" s="16" t="s">
+      <c r="AH18" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="Z18" s="16" t="s">
+      <c r="AI18" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="AA18" s="16" t="s">
+      <c r="AJ18" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="AB18" s="17">
+      <c r="AK18" s="17">
         <v>0.31</v>
       </c>
-      <c r="AC18" s="16">
+      <c r="AL18" s="16">
         <v>320</v>
       </c>
-      <c r="AD18" s="16">
+      <c r="AM18" s="16">
         <v>450</v>
       </c>
-      <c r="AE18" s="17">
+      <c r="AN18" s="17">
         <v>0.95</v>
       </c>
-      <c r="AF18" s="16">
+      <c r="AO18" s="17"/>
+      <c r="AP18" s="16"/>
+      <c r="AQ18" s="16">
         <v>46280.425000000003</v>
       </c>
-      <c r="AG18" s="16" t="s">
+      <c r="AR18" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH18" s="16">
+      <c r="AS18" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A19" s="11">
         <v>46280.611111111109</v>
       </c>
@@ -3103,96 +3549,121 @@
       <c r="E19" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G19" s="9" t="str">
+      <c r="I19" s="9" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
-      <c r="H19" s="13">
+      <c r="J19" s="13">
         <v>12</v>
       </c>
-      <c r="I19" s="36"/>
-      <c r="J19" s="39"/>
-      <c r="K19" s="37" t="s">
+      <c r="K19" s="36"/>
+      <c r="L19" s="39"/>
+      <c r="M19" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="L19" s="12" t="s">
+      <c r="N19" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M19" s="14">
+      <c r="O19" s="14">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>10.968</v>
       </c>
-      <c r="N19" s="15">
+      <c r="P19" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>105</v>
       </c>
-      <c r="O19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q19" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>31.26</v>
       </c>
-      <c r="P19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R19" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S19" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>136.26</v>
       </c>
-      <c r="Q19" s="15">
+      <c r="T19" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U19" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>136.26</v>
       </c>
-      <c r="S19" s="35"/>
-      <c r="T19" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V19" s="35"/>
+      <c r="W19" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U19" s="5" t="s">
+      <c r="X19" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="V19" s="12" t="s">
+      <c r="Y19" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z19" s="5"/>
+      <c r="AA19" s="49"/>
+      <c r="AB19" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="W19" s="16" t="str">
+      <c r="AC19" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X19" s="16" t="s">
+      <c r="AD19" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE19" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF19" s="16"/>
+      <c r="AG19" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="Y19" s="16" t="s">
+      <c r="AH19" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="Z19" s="16" t="s">
+      <c r="AI19" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AA19" s="16" t="s">
+      <c r="AJ19" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="AB19" s="17">
+      <c r="AK19" s="17">
         <v>8.75</v>
       </c>
-      <c r="AC19" s="16">
+      <c r="AL19" s="16">
         <v>914</v>
       </c>
-      <c r="AD19" s="16"/>
-      <c r="AE19" s="17">
+      <c r="AM19" s="16"/>
+      <c r="AN19" s="17">
         <v>2.85</v>
       </c>
-      <c r="AF19" s="16">
+      <c r="AO19" s="17"/>
+      <c r="AP19" s="16"/>
+      <c r="AQ19" s="16">
         <v>46280.611111111109</v>
       </c>
-      <c r="AG19" s="16" t="s">
+      <c r="AR19" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH19" s="16">
+      <c r="AS19" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A20" s="11">
         <v>46281.461805555555</v>
       </c>
@@ -3208,98 +3679,123 @@
       <c r="E20" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G20" s="9" t="str">
+      <c r="I20" s="9" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
-      <c r="H20" s="13">
+      <c r="J20" s="13">
         <v>12</v>
       </c>
-      <c r="I20" s="36">
+      <c r="K20" s="36">
         <v>600</v>
       </c>
-      <c r="J20" s="39"/>
-      <c r="K20" s="37" t="s">
+      <c r="L20" s="39"/>
+      <c r="M20" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="L20" s="12" t="s">
+      <c r="N20" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M20" s="14">
+      <c r="O20" s="14">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>7.1999999999999993</v>
       </c>
-      <c r="N20" s="15">
+      <c r="P20" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>105</v>
       </c>
-      <c r="O20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q20" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>20.52</v>
       </c>
-      <c r="P20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R20" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S20" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>125.52</v>
       </c>
-      <c r="Q20" s="15">
+      <c r="T20" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U20" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>125.52</v>
       </c>
-      <c r="S20" s="35"/>
-      <c r="T20" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V20" s="35"/>
+      <c r="W20" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U20" s="5" t="s">
+      <c r="X20" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="V20" s="12" t="s">
+      <c r="Y20" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z20" s="5"/>
+      <c r="AA20" s="49"/>
+      <c r="AB20" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="W20" s="16" t="str">
+      <c r="AC20" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X20" s="16" t="s">
+      <c r="AD20" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE20" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF20" s="16"/>
+      <c r="AG20" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="Y20" s="16" t="s">
+      <c r="AH20" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="Z20" s="16" t="s">
+      <c r="AI20" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AA20" s="16" t="s">
+      <c r="AJ20" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="AB20" s="17">
+      <c r="AK20" s="17">
         <v>8.75</v>
       </c>
-      <c r="AC20" s="16">
+      <c r="AL20" s="16">
         <v>914</v>
       </c>
-      <c r="AD20" s="16"/>
-      <c r="AE20" s="17">
+      <c r="AM20" s="16"/>
+      <c r="AN20" s="17">
         <v>2.85</v>
       </c>
-      <c r="AF20" s="16">
+      <c r="AO20" s="17"/>
+      <c r="AP20" s="16"/>
+      <c r="AQ20" s="16">
         <v>46281.461805555555</v>
       </c>
-      <c r="AG20" s="16" t="s">
+      <c r="AR20" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH20" s="16">
+      <c r="AS20" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A21" s="11">
         <v>46281.638888888891</v>
       </c>
@@ -3315,96 +3811,121 @@
       <c r="E21" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="G21" s="9" t="str">
+      <c r="I21" s="9" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
-      <c r="H21" s="13">
+      <c r="J21" s="13">
         <v>5</v>
       </c>
-      <c r="I21" s="36"/>
-      <c r="J21" s="39"/>
-      <c r="K21" s="37" t="s">
+      <c r="K21" s="36"/>
+      <c r="L21" s="39"/>
+      <c r="M21" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="L21" s="12" t="s">
+      <c r="N21" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M21" s="14">
+      <c r="O21" s="14">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>3.05</v>
       </c>
-      <c r="N21" s="15">
+      <c r="P21" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>15.5</v>
       </c>
-      <c r="O21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q21" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>8.69</v>
       </c>
-      <c r="P21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R21" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S21" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>24.189999999999998</v>
       </c>
-      <c r="Q21" s="15">
+      <c r="T21" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>15.499999999999998</v>
       </c>
-      <c r="R21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U21" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>8.69</v>
       </c>
-      <c r="S21" s="35"/>
-      <c r="T21" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V21" s="35"/>
+      <c r="W21" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U21" s="5" t="s">
+      <c r="X21" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="V21" s="12" t="s">
+      <c r="Y21" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z21" s="5"/>
+      <c r="AA21" s="49"/>
+      <c r="AB21" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="W21" s="16" t="str">
+      <c r="AC21" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X21" s="16" t="s">
+      <c r="AD21" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE21" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF21" s="16"/>
+      <c r="AG21" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="Y21" s="16" t="s">
+      <c r="AH21" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="Z21" s="16" t="s">
+      <c r="AI21" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="AA21" s="16" t="s">
+      <c r="AJ21" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="AB21" s="17">
+      <c r="AK21" s="17">
         <v>3.1</v>
       </c>
-      <c r="AC21" s="16">
+      <c r="AL21" s="16">
         <v>610</v>
       </c>
-      <c r="AD21" s="16"/>
-      <c r="AE21" s="17">
+      <c r="AM21" s="16"/>
+      <c r="AN21" s="17">
         <v>2.85</v>
       </c>
-      <c r="AF21" s="16">
+      <c r="AO21" s="17"/>
+      <c r="AP21" s="16"/>
+      <c r="AQ21" s="16">
         <v>46281.638888888891</v>
       </c>
-      <c r="AG21" s="16" t="s">
+      <c r="AR21" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH21" s="16">
+      <c r="AS21" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A22" s="11">
         <v>46282.381944444445</v>
       </c>
@@ -3420,98 +3941,123 @@
       <c r="E22" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G22" s="9" t="str">
+      <c r="I22" s="9" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
-      <c r="H22" s="13">
+      <c r="J22" s="13">
         <v>25</v>
       </c>
-      <c r="I22" s="36"/>
-      <c r="J22" s="39"/>
-      <c r="K22" s="37" t="s">
+      <c r="K22" s="36"/>
+      <c r="L22" s="39"/>
+      <c r="M22" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="L22" s="12" t="s">
+      <c r="N22" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="M22" s="14">
+      <c r="O22" s="14">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>3.1184999999999996</v>
       </c>
-      <c r="N22" s="15">
+      <c r="P22" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>2.25</v>
       </c>
-      <c r="O22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q22" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>2.96</v>
       </c>
-      <c r="P22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R22" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S22" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>5.21</v>
       </c>
-      <c r="Q22" s="15">
+      <c r="T22" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>2.96</v>
       </c>
-      <c r="R22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U22" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>2.25</v>
       </c>
-      <c r="S22" s="35"/>
-      <c r="T22" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V22" s="35"/>
+      <c r="W22" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U22" s="5" t="s">
+      <c r="X22" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="V22" s="12" t="s">
+      <c r="Y22" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z22" s="5"/>
+      <c r="AA22" s="49"/>
+      <c r="AB22" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="W22" s="16" t="str">
+      <c r="AC22" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X22" s="16" t="s">
+      <c r="AD22" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE22" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF22" s="16"/>
+      <c r="AG22" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="Y22" s="16" t="s">
+      <c r="AH22" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="Z22" s="16" t="s">
+      <c r="AI22" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="AA22" s="16" t="s">
+      <c r="AJ22" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="AB22" s="17">
+      <c r="AK22" s="17">
         <v>0.09</v>
       </c>
-      <c r="AC22" s="16">
+      <c r="AL22" s="16">
         <v>297</v>
       </c>
-      <c r="AD22" s="16">
+      <c r="AM22" s="16">
         <v>420</v>
       </c>
-      <c r="AE22" s="17">
+      <c r="AN22" s="17">
         <v>0.95</v>
       </c>
-      <c r="AF22" s="16">
+      <c r="AO22" s="17"/>
+      <c r="AP22" s="16"/>
+      <c r="AQ22" s="16">
         <v>46282.381944444445</v>
       </c>
-      <c r="AG22" s="16" t="s">
+      <c r="AR22" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH22" s="16">
+      <c r="AS22" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
         <v>46282.559027777781</v>
       </c>
@@ -3527,98 +4073,123 @@
       <c r="E23" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="F23" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="G23" s="20" t="str">
+      <c r="I23" s="20" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
-      <c r="H23" s="13">
+      <c r="J23" s="13">
         <v>15</v>
       </c>
-      <c r="I23" s="36"/>
-      <c r="J23" s="39"/>
-      <c r="K23" s="38" t="s">
+      <c r="K23" s="36"/>
+      <c r="L23" s="39"/>
+      <c r="M23" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="L23" s="12" t="s">
+      <c r="N23" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M23" s="21">
+      <c r="O23" s="21">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>2.16</v>
       </c>
-      <c r="N23" s="15">
+      <c r="P23" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>2.7</v>
       </c>
-      <c r="O23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q23" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>2.0499999999999998</v>
       </c>
-      <c r="P23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R23" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S23" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>4.75</v>
       </c>
-      <c r="Q23" s="15">
+      <c r="T23" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U23" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>4.75</v>
       </c>
-      <c r="S23" s="35"/>
-      <c r="T23" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V23" s="35"/>
+      <c r="W23" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U23" s="5" t="s">
+      <c r="X23" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="V23" s="12" t="s">
+      <c r="Y23" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z23" s="5"/>
+      <c r="AA23" s="49"/>
+      <c r="AB23" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="W23" s="16" t="str">
+      <c r="AC23" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X23" s="16" t="s">
+      <c r="AD23" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE23" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF23" s="16"/>
+      <c r="AG23" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="Y23" s="16" t="s">
+      <c r="AH23" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="Z23" s="16" t="s">
+      <c r="AI23" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="AA23" s="16" t="s">
+      <c r="AJ23" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="AB23" s="17">
+      <c r="AK23" s="17">
         <v>0.18</v>
       </c>
-      <c r="AC23" s="16">
+      <c r="AL23" s="16">
         <v>320</v>
       </c>
-      <c r="AD23" s="16">
+      <c r="AM23" s="16">
         <v>450</v>
       </c>
-      <c r="AE23" s="17">
+      <c r="AN23" s="17">
         <v>0.95</v>
       </c>
-      <c r="AF23" s="16">
+      <c r="AO23" s="17"/>
+      <c r="AP23" s="16"/>
+      <c r="AQ23" s="16">
         <v>46282.559027777781</v>
       </c>
-      <c r="AG23" s="16" t="s">
+      <c r="AR23" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH23" s="16">
+      <c r="AS23" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A24" s="11">
         <v>46282.666666666664</v>
       </c>
@@ -3634,96 +4205,121 @@
       <c r="E24" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="F24" s="12" t="s">
+      <c r="F24" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="G24" s="20" t="str">
+      <c r="I24" s="20" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
-      <c r="H24" s="13">
+      <c r="J24" s="13">
         <v>8</v>
       </c>
-      <c r="I24" s="36"/>
-      <c r="J24" s="39"/>
-      <c r="K24" s="38" t="s">
+      <c r="K24" s="36"/>
+      <c r="L24" s="39"/>
+      <c r="M24" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="L24" s="12" t="s">
+      <c r="N24" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M24" s="21">
+      <c r="O24" s="21">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>10.96</v>
       </c>
-      <c r="N24" s="15">
+      <c r="P24" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>91.2</v>
       </c>
-      <c r="O24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q24" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>19.18</v>
       </c>
-      <c r="P24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R24" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S24" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>110.38</v>
       </c>
-      <c r="Q24" s="15">
+      <c r="T24" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U24" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>110.38</v>
       </c>
-      <c r="S24" s="35"/>
-      <c r="T24" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V24" s="35"/>
+      <c r="W24" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U24" s="5" t="s">
+      <c r="X24" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="V24" s="12" t="s">
+      <c r="Y24" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z24" s="5"/>
+      <c r="AA24" s="49"/>
+      <c r="AB24" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="W24" s="16" t="str">
+      <c r="AC24" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X24" s="16" t="s">
+      <c r="AD24" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE24" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF24" s="16"/>
+      <c r="AG24" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="Y24" s="16" t="s">
+      <c r="AH24" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="Z24" s="16" t="s">
+      <c r="AI24" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AA24" s="16" t="s">
+      <c r="AJ24" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="AB24" s="17">
+      <c r="AK24" s="17">
         <v>11.4</v>
       </c>
-      <c r="AC24" s="16">
+      <c r="AL24" s="16">
         <v>1370</v>
       </c>
-      <c r="AD24" s="16"/>
-      <c r="AE24" s="17">
+      <c r="AM24" s="16"/>
+      <c r="AN24" s="17">
         <v>1.75</v>
       </c>
-      <c r="AF24" s="16">
+      <c r="AO24" s="17"/>
+      <c r="AP24" s="16"/>
+      <c r="AQ24" s="16">
         <v>46282.666666666664</v>
       </c>
-      <c r="AG24" s="16" t="s">
+      <c r="AR24" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH24" s="16">
+      <c r="AS24" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
         <v>46283.427083333336</v>
       </c>
@@ -3737,96 +4333,121 @@
       <c r="E25" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="G25" s="20" t="str">
+      <c r="I25" s="20" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
-      <c r="H25" s="13">
+      <c r="J25" s="13">
         <v>3</v>
       </c>
-      <c r="I25" s="36"/>
-      <c r="J25" s="39"/>
-      <c r="K25" s="38" t="s">
+      <c r="K25" s="36"/>
+      <c r="L25" s="39"/>
+      <c r="M25" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="L25" s="12" t="s">
+      <c r="N25" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M25" s="21">
+      <c r="O25" s="21">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>1.83</v>
       </c>
-      <c r="N25" s="15">
+      <c r="P25" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>9.3000000000000007</v>
       </c>
-      <c r="O25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q25" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>4.3899999999999997</v>
       </c>
-      <c r="P25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R25" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S25" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>13.690000000000001</v>
       </c>
-      <c r="Q25" s="15">
+      <c r="T25" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U25" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>13.690000000000001</v>
       </c>
-      <c r="S25" s="35"/>
-      <c r="T25" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V25" s="35"/>
+      <c r="W25" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U25" s="5" t="s">
+      <c r="X25" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="V25" s="12" t="s">
+      <c r="Y25" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z25" s="5"/>
+      <c r="AA25" s="49"/>
+      <c r="AB25" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="W25" s="16" t="str">
+      <c r="AC25" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X25" s="16" t="s">
+      <c r="AD25" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE25" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF25" s="16"/>
+      <c r="AG25" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="Y25" s="16" t="s">
+      <c r="AH25" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="Z25" s="16" t="s">
+      <c r="AI25" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="AA25" s="16" t="s">
+      <c r="AJ25" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="AB25" s="17">
+      <c r="AK25" s="17">
         <v>3.1</v>
       </c>
-      <c r="AC25" s="16">
+      <c r="AL25" s="16">
         <v>610</v>
       </c>
-      <c r="AD25" s="16"/>
-      <c r="AE25" s="17">
+      <c r="AM25" s="16"/>
+      <c r="AN25" s="17">
         <v>2.4</v>
       </c>
-      <c r="AF25" s="16">
+      <c r="AO25" s="17"/>
+      <c r="AP25" s="16"/>
+      <c r="AQ25" s="16">
         <v>46283.427083333336</v>
       </c>
-      <c r="AG25" s="16" t="s">
+      <c r="AR25" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH25" s="16">
+      <c r="AS25" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A26" s="11">
         <v>46283.486111111109</v>
       </c>
@@ -3840,98 +4461,123 @@
       <c r="E26" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="F26" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="G26" s="20" t="str">
+      <c r="I26" s="20" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
-      <c r="H26" s="13">
+      <c r="J26" s="13">
         <v>30</v>
       </c>
-      <c r="I26" s="36"/>
-      <c r="J26" s="39"/>
-      <c r="K26" s="38" t="s">
+      <c r="K26" s="36"/>
+      <c r="L26" s="39"/>
+      <c r="M26" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="L26" s="12" t="s">
+      <c r="N26" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M26" s="21">
+      <c r="O26" s="21">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>7.4843999999999991</v>
       </c>
-      <c r="N26" s="15">
+      <c r="P26" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>7.2</v>
       </c>
-      <c r="O26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q26" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>7.11</v>
       </c>
-      <c r="P26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R26" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S26" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>14.31</v>
       </c>
-      <c r="Q26" s="15">
+      <c r="T26" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U26" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>14.31</v>
       </c>
-      <c r="S26" s="35"/>
-      <c r="T26" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V26" s="35"/>
+      <c r="W26" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U26" s="5" t="s">
+      <c r="X26" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="V26" s="12" t="s">
+      <c r="Y26" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z26" s="5"/>
+      <c r="AA26" s="49"/>
+      <c r="AB26" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="W26" s="16" t="str">
+      <c r="AC26" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X26" s="16" t="s">
+      <c r="AD26" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE26" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF26" s="16"/>
+      <c r="AG26" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="Y26" s="16" t="s">
+      <c r="AH26" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="Z26" s="16" t="s">
+      <c r="AI26" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="AA26" s="16" t="s">
+      <c r="AJ26" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="AB26" s="17">
+      <c r="AK26" s="17">
         <v>0.24</v>
       </c>
-      <c r="AC26" s="16">
+      <c r="AL26" s="16">
         <v>420</v>
       </c>
-      <c r="AD26" s="16">
+      <c r="AM26" s="16">
         <v>594</v>
       </c>
-      <c r="AE26" s="17">
+      <c r="AN26" s="17">
         <v>0.95</v>
       </c>
-      <c r="AF26" s="16">
+      <c r="AO26" s="17"/>
+      <c r="AP26" s="16"/>
+      <c r="AQ26" s="16">
         <v>46283.486111111109</v>
       </c>
-      <c r="AG26" s="16" t="s">
+      <c r="AR26" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH26" s="16">
+      <c r="AS26" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
         <v>46283.638888888891</v>
       </c>
@@ -3947,96 +4593,121 @@
       <c r="E27" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="F27" s="12" t="s">
+      <c r="F27" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="G27" s="20" t="str">
+      <c r="I27" s="20" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
-      <c r="H27" s="13">
+      <c r="J27" s="13">
         <v>20</v>
       </c>
-      <c r="I27" s="36"/>
-      <c r="J27" s="39"/>
-      <c r="K27" s="38" t="s">
+      <c r="K27" s="36"/>
+      <c r="L27" s="39"/>
+      <c r="M27" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="L27" s="12" t="s">
+      <c r="N27" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M27" s="21">
+      <c r="O27" s="21">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>21.34</v>
       </c>
-      <c r="N27" s="15">
+      <c r="P27" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>112</v>
       </c>
-      <c r="O27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q27" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>60.82</v>
       </c>
-      <c r="P27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R27" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S27" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>172.82</v>
       </c>
-      <c r="Q27" s="15">
+      <c r="T27" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U27" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>172.82</v>
       </c>
-      <c r="S27" s="35"/>
-      <c r="T27" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V27" s="35"/>
+      <c r="W27" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U27" s="5" t="s">
+      <c r="X27" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="V27" s="12" t="s">
+      <c r="Y27" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z27" s="5"/>
+      <c r="AA27" s="49"/>
+      <c r="AB27" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="W27" s="16" t="str">
+      <c r="AC27" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X27" s="16" t="s">
+      <c r="AD27" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE27" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF27" s="16"/>
+      <c r="AG27" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="Y27" s="16" t="s">
+      <c r="AH27" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="Z27" s="16" t="s">
+      <c r="AI27" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AA27" s="16" t="s">
+      <c r="AJ27" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="AB27" s="17">
+      <c r="AK27" s="17">
         <v>5.6</v>
       </c>
-      <c r="AC27" s="16">
+      <c r="AL27" s="16">
         <v>1067</v>
       </c>
-      <c r="AD27" s="16"/>
-      <c r="AE27" s="17">
+      <c r="AM27" s="16"/>
+      <c r="AN27" s="17">
         <v>2.85</v>
       </c>
-      <c r="AF27" s="16">
+      <c r="AO27" s="17"/>
+      <c r="AP27" s="16"/>
+      <c r="AQ27" s="16">
         <v>46283.638888888891</v>
       </c>
-      <c r="AG27" s="16" t="s">
+      <c r="AR27" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH27" s="16">
+      <c r="AS27" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A28" s="11">
         <v>46284.34375</v>
       </c>
@@ -4052,98 +4723,123 @@
       <c r="E28" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F28" s="12" t="s">
+      <c r="F28" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="G28" s="20" t="str">
+      <c r="I28" s="20" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
-      <c r="H28" s="13">
+      <c r="J28" s="13">
         <v>40</v>
       </c>
-      <c r="I28" s="36"/>
-      <c r="J28" s="39"/>
-      <c r="K28" s="38" t="s">
+      <c r="K28" s="36"/>
+      <c r="L28" s="39"/>
+      <c r="M28" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="L28" s="12" t="s">
+      <c r="N28" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M28" s="21">
+      <c r="O28" s="21">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>19.982159999999997</v>
       </c>
-      <c r="N28" s="15">
+      <c r="P28" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>16.8</v>
       </c>
-      <c r="O28" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q28" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>18.98</v>
       </c>
-      <c r="P28" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R28" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S28" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>35.78</v>
       </c>
-      <c r="Q28" s="15">
+      <c r="T28" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R28" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U28" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>35.78</v>
       </c>
-      <c r="S28" s="35"/>
-      <c r="T28" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V28" s="35"/>
+      <c r="W28" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
-      <c r="U28" s="5" t="s">
+      <c r="X28" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="V28" s="12" t="s">
+      <c r="Y28" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z28" s="5"/>
+      <c r="AA28" s="49"/>
+      <c r="AB28" s="12" t="s">
         <v>194</v>
       </c>
-      <c r="W28" s="16" t="str">
+      <c r="AC28" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
-      <c r="X28" s="16" t="s">
+      <c r="AD28" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE28" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF28" s="16"/>
+      <c r="AG28" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="Y28" s="16" t="s">
+      <c r="AH28" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="Z28" s="16" t="s">
+      <c r="AI28" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="AA28" s="16" t="s">
+      <c r="AJ28" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="AB28" s="17">
+      <c r="AK28" s="17">
         <v>0.42</v>
       </c>
-      <c r="AC28" s="16">
+      <c r="AL28" s="16">
         <v>594</v>
       </c>
-      <c r="AD28" s="16">
+      <c r="AM28" s="16">
         <v>841</v>
       </c>
-      <c r="AE28" s="17">
+      <c r="AN28" s="17">
         <v>0.95</v>
       </c>
-      <c r="AF28" s="16">
+      <c r="AO28" s="17"/>
+      <c r="AP28" s="16"/>
+      <c r="AQ28" s="16">
         <v>46284.34375</v>
       </c>
-      <c r="AG28" s="16" t="s">
+      <c r="AR28" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH28" s="16">
+      <c r="AS28" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
         <v>46284.395833333336</v>
       </c>
@@ -4155,124 +4851,149 @@
       <c r="E29" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="12" t="s">
+      <c r="F29" s="49" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v/>
+      </c>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G29" s="20" t="str">
+      <c r="I29" s="20" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
-      <c r="H29" s="13">
+      <c r="J29" s="13">
         <v>12</v>
       </c>
-      <c r="I29" s="36">
+      <c r="K29" s="36">
         <v>1200</v>
       </c>
-      <c r="J29" s="39"/>
-      <c r="K29" s="38" t="s">
+      <c r="L29" s="39"/>
+      <c r="M29" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="L29" s="12" t="s">
+      <c r="N29" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="M29" s="21">
+      <c r="O29" s="21">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>14.399999999999999</v>
       </c>
-      <c r="N29" s="15">
+      <c r="P29" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>105</v>
       </c>
-      <c r="O29" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP))</f>
+      <c r="Q29" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
         <v>41.04</v>
       </c>
-      <c r="P29" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]])</f>
+      <c r="R29" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <v>0</v>
+      </c>
+      <c r="S29" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
         <v>146.04</v>
       </c>
-      <c r="Q29" s="15">
+      <c r="T29" s="15">
         <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
-      <c r="R29" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]))</f>
+      <c r="U29" s="15">
+        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
         <v>146.04</v>
       </c>
-      <c r="S29" s="35"/>
-      <c r="T29" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[H_Issues]]="","OK",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255)))</f>
+      <c r="V29" s="35"/>
+      <c r="W29" s="9" t="str">
+        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>Student name or number required; Print width exceeds stock width</v>
       </c>
-      <c r="U29" s="5" t="s">
+      <c r="X29" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="V29" s="12" t="s">
+      <c r="Y29" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="Z29" s="5"/>
+      <c r="AA29" s="49"/>
+      <c r="AB29" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="W29" s="16" t="str">
+      <c r="AC29" s="16" t="str">
         <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v>; Student name or number required; Print width exceeds stock width</v>
       </c>
-      <c r="X29" s="16" t="s">
+      <c r="AD29" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <v/>
+      </c>
+      <c r="AE29" s="16" t="str">
+        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <v/>
+      </c>
+      <c r="AF29" s="16"/>
+      <c r="AG29" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="Y29" s="16" t="s">
+      <c r="AH29" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="Z29" s="16" t="s">
+      <c r="AI29" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="AA29" s="16" t="s">
+      <c r="AJ29" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="AB29" s="17">
+      <c r="AK29" s="17">
         <v>8.75</v>
       </c>
-      <c r="AC29" s="16">
+      <c r="AL29" s="16">
         <v>914</v>
       </c>
-      <c r="AD29" s="16"/>
-      <c r="AE29" s="17">
+      <c r="AM29" s="16"/>
+      <c r="AN29" s="17">
         <v>2.85</v>
       </c>
-      <c r="AF29" s="16">
+      <c r="AO29" s="17"/>
+      <c r="AP29" s="16"/>
+      <c r="AQ29" s="16">
         <v>46284.395833333336</v>
       </c>
-      <c r="AG29" s="16" t="s">
+      <c r="AR29" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="AH29" s="16">
+      <c r="AS29" s="16">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
-  <conditionalFormatting sqref="T18:T29">
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <conditionalFormatting sqref="W18:W29">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>AND(T18&lt;&gt;"",T18&lt;&gt;"OK")</formula>
+      <formula>AND(W18&lt;&gt;"",W18&lt;&gt;"OK")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="7">
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Date and time" error="Date and time the print was produced. Use the Now button to stamp the current date and time." promptTitle="Date and time" prompt="Date and time the print was produced. Use the Now button to stamp the current date and time." sqref="A18:A29" xr:uid="{00000000-0002-0000-0900-000007000000}">
       <formula1>36526</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L18:L29 K18:K29" xr:uid="{00000000-0002-0000-0900-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N18:N29 M18:M29" xr:uid="{00000000-0002-0000-0900-000003000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Roll length unit" error="Choose Metres or Centimetres." promptTitle="Roll length unit" prompt="How a roll job's length is typed into Qty on this sheet. Always converted to, and stored as, metres regardless of this setting - Sheet stock is unaffected." sqref="B11" xr:uid="{DDF6FDDC-C744-4D90-987F-9EBAA10EE831}">
       <formula1>"Metres,Centimetres"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle="Qty" error="Sheets for sheet stock, metres for roll stock. Must be greater than zero." promptTitle="Qty" prompt="Sheets for sheet stock, metres for roll stock. Must be greater than zero." sqref="H18:H29" xr:uid="{0EB6289D-94A2-4A20-A725-132ACF4AC0B0}">
+    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle="Qty" error="Sheets for sheet stock, metres for roll stock. Must be greater than zero." promptTitle="Qty" prompt="Sheets for sheet stock, metres for roll stock. Must be greater than zero." sqref="J18:J29" xr:uid="{0EB6289D-94A2-4A20-A725-132ACF4AC0B0}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Print width" error="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." promptTitle="Print width" prompt="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width. Required for 'Supplied (Roll)'." sqref="I18:I29" xr:uid="{1894B910-050C-4C3A-8489-9F7A13C9685D}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Print width" error="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width." promptTitle="Print width" prompt="Optional, roll stock only, in millimetres. Leave blank to use the full width of the roll. It must not exceed the stock width. Required for 'Supplied (Roll)'." sqref="K18:K29" xr:uid="{1894B910-050C-4C3A-8489-9F7A13C9685D}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Sheet size" error="Choose one of the standard sizes listed on Settings." promptTitle="Sheet size" prompt="Required only for 'Supplied (Sheet)' - the nearest standard size to the sheet the student brought. Ignored for every other paper stock." sqref="J18:J29" xr:uid="{974A2940-850F-46E7-B729-C14D6A820BB6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Sheet size" error="Choose one of the standard sizes listed on Settings." promptTitle="Sheet size" prompt="Required only for 'Supplied (Sheet)' - the nearest standard size to the sheet the student brought. Ignored for every other paper stock." sqref="L18:L29" xr:uid="{974A2940-850F-46E7-B729-C14D6A820BB6}">
       <formula1>RNG_STD_SIZES</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paid" error="Choose Yes or No." promptTitle="Paid" prompt="Whether this chargeable cost has been paid. Blank means not recorded either way and counts as unpaid in totals." sqref="S18:S29" xr:uid="{A827598F-CA17-4532-A2B4-E4329BE2650A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paid" error="Choose Yes or No." promptTitle="Paid" prompt="Whether this chargeable cost has been paid. Blank means not recorded either way and counts as unpaid in totals." sqref="V18:V29" xr:uid="{A827598F-CA17-4532-A2B4-E4329BE2650A}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4293,79 +5014,79 @@
           <x14:formula1>
             <xm:f>_Work!$J$2:$J$12</xm:f>
           </x14:formula1>
-          <xm:sqref>F24</xm:sqref>
+          <xm:sqref>H24</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="Choose one of the listed options. Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family HP DesignJet Z9+ supports - picking one clears the printer instead." promptTitle="Paper stock" prompt="Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family HP DesignJet Z9+ supports - picking one clears the printer instead." xr:uid="{804CCC33-3817-4F3E-94F4-8A56C88B24CB}">
           <x14:formula1>
             <xm:f>_Work!$K$2:$K$12</xm:f>
           </x14:formula1>
-          <xm:sqref>F25</xm:sqref>
+          <xm:sqref>H25</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="Choose one of the listed options. Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family Xerox Versant 180 supports - picking one clears the printer instead." promptTitle="Paper stock" prompt="Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family Xerox Versant 180 supports - picking one clears the printer instead." xr:uid="{4A0AEE34-9D74-46CA-A391-1496C855AAAF}">
           <x14:formula1>
             <xm:f>_Work!$L$2:$L$12</xm:f>
           </x14:formula1>
-          <xm:sqref>F18 F22:F23 F26 F28</xm:sqref>
+          <xm:sqref>H18 H22:H23 H26 H28</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Paper stock" error="Choose one of the listed options. Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family Epson SureColor P9500 supports - picking one clears the printer instead." promptTitle="Paper stock" prompt="Every active stock compatible with a printer at this print room. Stocks marked '(unavailable)' are not in a family Epson SureColor P9500 supports - picking one clears the printer instead." xr:uid="{32B928B8-1766-4CED-B621-7AB9984EA332}">
           <x14:formula1>
             <xm:f>_Work!$M$2:$M$12</xm:f>
           </x14:formula1>
-          <xm:sqref>F19:F21 F27 F29</xm:sqref>
+          <xm:sqref>H19:H21 H27 H29</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Gloss 200gsm SRA3 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Gloss 200gsm SRA3 sheet' - picking one clears the paper stock instead." xr:uid="{3D72609D-7821-40D1-B4E0-9A17A762D7B9}">
           <x14:formula1>
             <xm:f>_Work!$N$2:$N$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E18</xm:sqref>
+          <xm:sqref>E18:G18</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Uncoated 120gsm A3 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Uncoated 120gsm A3 sheet' - picking one clears the paper stock instead." xr:uid="{ADA2925B-D9CE-483D-A3CB-F6887904EC42}">
           <x14:formula1>
             <xm:f>_Work!$O$2:$O$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E22</xm:sqref>
+          <xm:sqref>E22:G22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Gloss offcut 320x450 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Gloss offcut 320x450 sheet' - picking one clears the paper stock instead." xr:uid="{012D11A0-C356-4599-BC4D-DC0EE936279D}">
           <x14:formula1>
             <xm:f>_Work!$P$2:$P$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E23</xm:sqref>
+          <xm:sqref>E23:G23</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Vinyl self-adhesive 1370mm roll' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Vinyl self-adhesive 1370mm roll' - picking one clears the paper stock instead." xr:uid="{8B127D0B-FEBC-4EAD-9A1C-1213E7673F7A}">
           <x14:formula1>
             <xm:f>_Work!$Q$2:$Q$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E24</xm:sqref>
+          <xm:sqref>E24:G24</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Satin photo 610mm roll' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Satin photo 610mm roll' - picking one clears the paper stock instead." xr:uid="{9C71BD25-2544-420E-9FD9-6BBB323309B0}">
           <x14:formula1>
             <xm:f>_Work!$R$2:$R$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E21 E25</xm:sqref>
+          <xm:sqref>E21:G21 E25:G25</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm A2 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm A2 sheet' - picking one clears the paper stock instead." xr:uid="{67197FBA-1C2E-4D3C-ACB9-817976B15DF1}">
           <x14:formula1>
             <xm:f>_Work!$S$2:$S$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E26</xm:sqref>
+          <xm:sqref>E26:G26</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm 1067mm roll' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm 1067mm roll' - picking one clears the paper stock instead." xr:uid="{8CFA56E2-9A8D-460B-A5B6-7BDFEC59376E}">
           <x14:formula1>
             <xm:f>_Work!$T$2:$T$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E27</xm:sqref>
+          <xm:sqref>E27:G27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm A1 sheet' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Matte 180gsm A1 sheet' - picking one clears the paper stock instead." xr:uid="{D369D7DE-B42A-4E5A-915B-58A90399AD45}">
           <x14:formula1>
             <xm:f>_Work!$U$2:$U$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E28</xm:sqref>
+          <xm:sqref>E28:G28</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Printer" error="Choose one of the listed options. Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Canvas 914mm roll' - picking one clears the paper stock instead." promptTitle="Printer" prompt="Every active printer permitted at this print room. Printers marked '(unavailable)' don't support 'Canvas 914mm roll' - picking one clears the paper stock instead." xr:uid="{C4698F5D-DDE1-4E72-8DD1-0CFA5F7A883D}">
           <x14:formula1>
             <xm:f>_Work!$V$2:$V$4</xm:f>
           </x14:formula1>
-          <xm:sqref>E19:E20 E29</xm:sqref>
+          <xm:sqref>E19:G20 E29:G29</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Default technician" error="Choose one of the listed options. Pre-fills each new print job's Technician until Clear defaults is used." promptTitle="Default technician" prompt="Pre-fills each new print job's Technician until Clear defaults is used." xr:uid="{4692C48D-8984-4261-BBD5-05992933E720}">
           <x14:formula1>
@@ -4407,7 +5128,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4450,7 +5171,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="30" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B7" s="24" t="s">
         <v>67</v>
@@ -4464,7 +5185,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="30" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>69</v>
@@ -4478,7 +5199,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="30" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>71</v>
@@ -4491,7 +5212,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Active" error="Set to No to retire a technician. Existing records keep working; the name stops appearing for new print jobs." promptTitle="Active" prompt="Set to No to retire a technician. Existing records keep working; the name stops appearing for new print jobs." sqref="D7:D2001" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Yes,No"</formula1>
@@ -4507,36 +5228,37 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
     <col min="2" max="2" width="30.7265625" customWidth="1"/>
     <col min="3" max="3" width="17.7265625" customWidth="1"/>
     <col min="4" max="4" width="13.7265625" customWidth="1"/>
-    <col min="5" max="6" width="14.7265625" customWidth="1"/>
-    <col min="7" max="7" width="9.7265625" customWidth="1"/>
+    <col min="5" max="6" width="14.6328125" customWidth="1"/>
+    <col min="7" max="8" width="14.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="H4" s="2" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>75</v>
       </c>
@@ -4549,19 +5271,25 @@
       <c r="D6" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="G6" s="23" t="s">
         <v>219</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="H6" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="I6" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="30" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B7" s="24" t="s">
         <v>79</v>
@@ -4572,17 +5300,21 @@
       <c r="D7" s="44">
         <v>2.85</v>
       </c>
-      <c r="E7" s="45">
+      <c r="E7" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="F7" s="44"/>
+      <c r="G7" s="45">
         <v>1370</v>
       </c>
-      <c r="F7" s="47"/>
-      <c r="G7" s="24" t="s">
+      <c r="H7" s="47"/>
+      <c r="I7" s="24" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="30" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>81</v>
@@ -4593,17 +5325,21 @@
       <c r="D8" s="44">
         <v>2.4</v>
       </c>
-      <c r="E8" s="46">
+      <c r="E8" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="F8" s="44"/>
+      <c r="G8" s="46">
         <v>610</v>
       </c>
-      <c r="F8" s="47"/>
-      <c r="G8" s="24" t="s">
+      <c r="H8" s="47"/>
+      <c r="I8" s="24" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="30" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>83</v>
@@ -4614,17 +5350,21 @@
       <c r="D9" s="44">
         <v>0.95</v>
       </c>
-      <c r="E9" s="46"/>
-      <c r="F9" s="47" t="s">
+      <c r="E9" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="F9" s="44"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="G9" s="24" t="s">
+      <c r="I9" s="24" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="30" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>85</v>
@@ -4635,32 +5375,36 @@
       <c r="D10" s="44">
         <v>1.75</v>
       </c>
-      <c r="E10" s="46">
+      <c r="E10" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="F10" s="44"/>
+      <c r="G10" s="46">
         <v>1370</v>
       </c>
-      <c r="F10" s="47"/>
-      <c r="G10" s="24" t="s">
+      <c r="H10" s="47"/>
+      <c r="I10" s="24" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <phoneticPr fontId="11" type="noConversion"/>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C2001" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>lstConsumables</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" showInputMessage="1" showErrorMessage="1" errorTitle="Consumable cost" error="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." promptTitle="Consumable cost" prompt="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." sqref="D7:D2001" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" showInputMessage="1" showErrorMessage="1" errorTitle="Consumable cost" error="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." promptTitle="Consumable cost" prompt="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." sqref="D7:D2001 E7:F10" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G7:G2001" xr:uid="{00000000-0002-0000-0200-000002000000}">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Max roll width mm" error="Enter 0 or more, in millimetres." promptTitle="Max roll width mm" prompt="The widest roll stock this printer can take, in millimetres. Leave blank if this printer cannot print on roll stock." sqref="E7:E10" xr:uid="{C0A2668E-6A17-4354-874C-F8907F30987B}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Max roll width mm" error="Enter 0 or more, in millimetres." promptTitle="Max roll width mm" prompt="The widest roll stock this printer can take, in millimetres. Leave blank if this printer cannot print on roll stock." sqref="G7:G10" xr:uid="{C0A2668E-6A17-4354-874C-F8907F30987B}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Max sheet size" error="Choose one of the standard sizes listed on Settings." promptTitle="Max sheet size" prompt="The largest standard sheet size this printer can take. Leave blank if this printer cannot print on sheet stock." sqref="F7:F10" xr:uid="{B526154C-BEC4-4000-8C38-838E3A63AF21}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Max sheet size" error="Choose one of the standard sizes listed on Settings." promptTitle="Max sheet size" prompt="The largest standard sheet size this printer can take. Leave blank if this printer cannot print on sheet stock." sqref="H7:H10" xr:uid="{B526154C-BEC4-4000-8C38-838E3A63AF21}">
       <formula1>RNG_STD_SIZES</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G11:G2001 I7:I10" xr:uid="{00000000-0002-0000-0200-000002000000}">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4746,7 +5490,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="30" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B7" s="24" t="s">
         <v>95</v>
@@ -4785,7 +5529,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="30" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>98</v>
@@ -4824,7 +5568,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="30" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>100</v>
@@ -4863,7 +5607,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="30" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>102</v>
@@ -4902,7 +5646,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="30" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B11" s="24" t="s">
         <v>104</v>
@@ -4937,7 +5681,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="30" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B12" s="24" t="s">
         <v>106</v>
@@ -4972,7 +5716,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="30" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B13" s="24" t="s">
         <v>108</v>
@@ -5007,7 +5751,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="30" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B14" s="24" t="s">
         <v>110</v>
@@ -5042,7 +5786,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="30" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B15" s="24" t="s">
         <v>112</v>
@@ -5078,7 +5822,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Supplied by student" error="Choose Yes or No." promptTitle="Supplied by student" prompt="Yes only for the two 'Supplied' catalogue rows - paper cost always computes to zero for these regardless of Cost." sqref="L7:L15" xr:uid="{2ED70CBA-D9C3-4CB5-A147-78652DAACDC7}">
       <formula1>"Yes,No"</formula1>
@@ -5118,7 +5862,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
@@ -5373,6 +6117,12 @@
       <c r="K13" s="8">
         <v>297</v>
       </c>
+      <c r="M13" s="24" t="s">
+        <v>289</v>
+      </c>
+      <c r="N13" s="24" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
@@ -5411,7 +6161,7 @@
         <v>29</v>
       </c>
       <c r="C15" s="40">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="D15" s="26" t="s">
         <v>30</v>
@@ -5507,7 +6257,7 @@
         <v>214</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>250</v>
+        <v>293</v>
       </c>
       <c r="D22" s="26" t="s">
         <v>249</v>
@@ -5515,16 +6265,16 @@
     </row>
     <row r="23" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="48" t="s">
+        <v>253</v>
+      </c>
+      <c r="D23" s="26" t="s">
         <v>252</v>
-      </c>
-      <c r="C23" s="48" t="s">
-        <v>254</v>
-      </c>
-      <c r="D23" s="26" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
@@ -5541,66 +6291,80 @@
         <v>217</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" ht="58" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
-        <v>236</v>
+        <v>290</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="C25" s="48">
-        <v>3</v>
+        <v>291</v>
+      </c>
+      <c r="C25" s="48" t="s">
+        <v>130</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>238</v>
+        <v>292</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C26" s="48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C27" s="48">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D27" s="26" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="C28" s="48">
+        <v>9</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="C29" s="48" t="s">
+        <v>257</v>
+      </c>
+      <c r="D29" s="26" t="s">
         <v>256</v>
       </c>
-      <c r="C28" s="48" t="s">
-        <v>258</v>
-      </c>
-      <c r="D28" s="26" t="s">
-        <v>257</v>
-      </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G9:G2003 N9:N2003" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G9:G2003 N9:N2004" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Dimension" error="Enter the size in millimetres." promptTitle="Dimension" prompt="Enter the size in millimetres." sqref="J9:K2003" xr:uid="{00000000-0002-0000-0000-000003000000}">
@@ -5700,7 +6464,7 @@
       <c r="K2" s="22"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -5714,7 +6478,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5725,7 +6489,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5754,7 +6518,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
0.11.0 (3-7/7): multi-pass costing - pass rows, colours, buttons, reports, import/export
Pass rows (modPasses), Consumables sheet (modConsumables, tblColours), Colour
mode / Template cost on printers, roll-up costing, Add/Remove pass and
collapse/expand, pass-column toggle layered under the view, notices level on
Status, Reports/Summary Passes and Set-up cost with a Pass type filter,
Export/Import/Restore of pass rows, Re-stamp, Backup guard. Schema 1.4.

Tests: test-multipass, -io and -views new; positional tests re-pointed.
Docs: ARCHITECTURE section 17 as built, CHANGELOG, SETUP.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A63511-F932-4C50-B688-8D925626494D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357BC0D6-54B8-4E86-A589-5EBD0AB74D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1433,37 +1433,6 @@
   </cellStyles>
   <dxfs count="90">
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1722,6 +1691,359 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF2E64A8"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF2E64A8"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF2E64A8"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1789,6 +2111,16 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
@@ -1817,338 +2149,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FF2E64A8"/>
-        </left>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FF2E64A8"/>
-        </left>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FF2E64A8"/>
-        </left>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -2612,11 +2612,11 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="74"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Student No" dataDxfId="73"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="Technician" dataDxfId="72"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="14"/>
-    <tableColumn id="25" xr3:uid="{09F3ECAE-609E-455B-9BA8-2E241E8FAF46}" name="Passes" dataDxfId="12">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="11"/>
+    <tableColumn id="25" xr3:uid="{09F3ECAE-609E-455B-9BA8-2E241E8FAF46}" name="Passes" dataDxfId="9">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="36" xr3:uid="{3444712F-EA34-42DA-B9B5-0EBBE8952B8B}" name="Colour" dataDxfId="13"/>
+    <tableColumn id="36" xr3:uid="{3444712F-EA34-42DA-B9B5-0EBBE8952B8B}" name="Colour" dataDxfId="10"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="71"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="70">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</calculatedColumnFormula>
@@ -2632,13 +2632,13 @@
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="63">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="8">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="5">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="37" xr3:uid="{9D5B92B2-8D8C-4AB8-B4C8-729D5FEC16B3}" name="Set-up Cost" dataDxfId="6">
+    <tableColumn id="37" xr3:uid="{9D5B92B2-8D8C-4AB8-B4C8-729D5FEC16B3}" name="Set-up Cost" dataDxfId="3">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="7">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="4">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Disregarded" dataDxfId="62">
@@ -2652,33 +2652,33 @@
       <calculatedColumnFormula>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Job ID" dataDxfId="58"/>
-    <tableColumn id="38" xr3:uid="{4D2F43D5-36A3-4912-BABA-E130C7C2146E}" name="Row Type" dataDxfId="18"/>
-    <tableColumn id="39" xr3:uid="{5A1BB7C9-ECFF-4CC8-8500-3A293A25528C}" name="Parent" dataDxfId="11"/>
-    <tableColumn id="40" xr3:uid="{3E507CE4-6A67-46A5-BB60-7B729C2D5A26}" name="Pass" dataDxfId="9"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="10"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="57">
+    <tableColumn id="38" xr3:uid="{4D2F43D5-36A3-4912-BABA-E130C7C2146E}" name="Row Type" dataDxfId="57"/>
+    <tableColumn id="39" xr3:uid="{5A1BB7C9-ECFF-4CC8-8500-3A293A25528C}" name="Parent" dataDxfId="8"/>
+    <tableColumn id="40" xr3:uid="{3E507CE4-6A67-46A5-BB60-7B729C2D5A26}" name="Pass" dataDxfId="6"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="7"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="56">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="41" xr3:uid="{82AE4E46-EF17-494F-A090-ADA99BEE4E30}" name="H_Ink" dataDxfId="17">
+    <tableColumn id="41" xr3:uid="{82AE4E46-EF17-494F-A090-ADA99BEE4E30}" name="H_Ink" dataDxfId="55">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{7A8AEB6A-0F1F-4F77-9521-2D3285156496}" name="H_Setup" dataDxfId="16">
+    <tableColumn id="42" xr3:uid="{7A8AEB6A-0F1F-4F77-9521-2D3285156496}" name="H_Setup" dataDxfId="54">
       <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="43" xr3:uid="{4F21AC66-121A-48B2-991A-1B25B7F679A0}" name="H_Notices" dataDxfId="15"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="56"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="55"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="54"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="53"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="52"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="51"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="50"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="5"/>
-    <tableColumn id="44" xr3:uid="{473158C1-5A71-4BCD-9231-D8A93A8E6E06}" name="S_SetupCost" dataDxfId="3"/>
-    <tableColumn id="45" xr3:uid="{AE04C717-F979-427D-9DE7-1B4ED6904D05}" name="S_ColourID" dataDxfId="4"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="49"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="48"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="47"/>
+    <tableColumn id="43" xr3:uid="{4F21AC66-121A-48B2-991A-1B25B7F679A0}" name="H_Notices" dataDxfId="53"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="52"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="51"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="50"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="49"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="48"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="47"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="46"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="2"/>
+    <tableColumn id="44" xr3:uid="{473158C1-5A71-4BCD-9231-D8A93A8E6E06}" name="S_SetupCost" dataDxfId="0"/>
+    <tableColumn id="45" xr3:uid="{AE04C717-F979-427D-9DE7-1B4ED6904D05}" name="S_ColourID" dataDxfId="1"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="45"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="44"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2699,54 +2699,54 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblTechnicians" displayName="tblTechnicians" ref="A6:D9" totalsRowShown="0" dataDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblTechnicians" displayName="tblTechnicians" ref="A6:D9" totalsRowShown="0" dataDxfId="42">
   <autoFilter ref="A6:D9" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Name" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Department" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Active" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Name" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Department" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Active" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblPrinters" displayName="tblPrinters" ref="A6:I10" totalsRowShown="0" dataDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblPrinters" displayName="tblPrinters" ref="A6:I10" totalsRowShown="0" dataDxfId="37">
   <autoFilter ref="A6:I10" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Model" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Consumable type" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{15CEC00B-A782-4C1F-9D8C-FC4996A5205D}" name="Colour mode" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{59F8E22B-28C7-46F1-991A-38D5C4091FF4}" name="Template cost" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{27EBC752-1CF1-48B9-B798-05BFAB38AF84}" name="Max roll width mm" dataDxfId="36"/>
-    <tableColumn id="8" xr3:uid="{78D66AB2-9A7B-410A-92C1-2CCFD2C22414}" name="Max sheet size" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Active" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Model" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Consumable type" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{15CEC00B-A782-4C1F-9D8C-FC4996A5205D}" name="Colour mode" dataDxfId="32"/>
+    <tableColumn id="9" xr3:uid="{59F8E22B-28C7-46F1-991A-38D5C4091FF4}" name="Template cost" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{27EBC752-1CF1-48B9-B798-05BFAB38AF84}" name="Max roll width mm" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{78D66AB2-9A7B-410A-92C1-2CCFD2C22414}" name="Max sheet size" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Active" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:L15" totalsRowShown="0" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:L15" totalsRowShown="0" dataDxfId="27">
   <autoFilter ref="A6:L15" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Description" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Paper type" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Measure" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Size mode" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Std. size" dataDxfId="27"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Width mm" dataDxfId="26"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Height mm" dataDxfId="25"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Cost" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Cost unit" dataDxfId="23">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Description" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Paper type" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Measure" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Size mode" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Std. size" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Width mm" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Height mm" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Cost" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Cost unit" dataDxfId="17">
       <calculatedColumnFormula>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Active" dataDxfId="22"/>
-    <tableColumn id="13" xr3:uid="{62AE4E30-01F2-4D26-B1F8-C8FD5BF6FCC9}" name="Supplied by student" dataDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Active" dataDxfId="16"/>
+    <tableColumn id="13" xr3:uid="{62AE4E30-01F2-4D26-B1F8-C8FD5BF6FCC9}" name="Supplied by student" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2808,8 +2808,8 @@
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Name"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Department"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="Rows"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="First date" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Last date" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="First date" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Last date" dataDxfId="13"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="State"/>
     <tableColumn id="9" xr3:uid="{F307D930-BB9C-468F-AC38-00DA61DF508D}" name="Last export"/>
     <tableColumn id="10" xr3:uid="{B7692E42-45DD-48C6-8B10-C3C464C1B69D}" name="Export sig"/>
@@ -3140,10 +3140,9 @@
     <col min="31" max="31" width="14.7265625" hidden="1" customWidth="1"/>
     <col min="32" max="32" width="11.7265625" hidden="1" customWidth="1"/>
     <col min="33" max="33" width="8.7265625" hidden="1" customWidth="1" collapsed="1"/>
-    <col min="34" max="34" width="8.7265625" hidden="1" customWidth="1"/>
-    <col min="35" max="35" width="0" hidden="1" customWidth="1"/>
+    <col min="34" max="35" width="8.7265625" hidden="1" customWidth="1"/>
     <col min="36" max="36" width="29.90625" hidden="1" customWidth="1"/>
-    <col min="37" max="44" width="0" hidden="1" customWidth="1"/>
+    <col min="37" max="44" width="8.7265625" hidden="1" customWidth="1"/>
     <col min="52" max="52" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4970,7 +4969,7 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <conditionalFormatting sqref="W18:W29">
-    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="1" stopIfTrue="1">
       <formula>AND(W18&lt;&gt;"",W18&lt;&gt;"OK")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5390,11 +5389,11 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <phoneticPr fontId="11" type="noConversion"/>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C2001" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>lstConsumables</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" showInputMessage="1" showErrorMessage="1" errorTitle="Consumable cost" error="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." promptTitle="Consumable cost" prompt="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." sqref="D7:D2001 E7:F10" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" showInputMessage="1" showErrorMessage="1" errorTitle="Consumable cost" error="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." promptTitle="Consumable cost" prompt="Estimated consumable cost to print one square metre, including typical coverage. Must be zero or more." sqref="D7:D2001" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Max roll width mm" error="Enter 0 or more, in millimetres." promptTitle="Max roll width mm" prompt="The widest roll stock this printer can take, in millimetres. Leave blank if this printer cannot print on roll stock." sqref="G7:G10" xr:uid="{C0A2668E-6A17-4354-874C-F8907F30987B}">
@@ -5405,6 +5404,12 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G11:G2001 I7:I10" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Colour mode" error="Choose single pass or multi-pass." promptTitle="Colour mode" prompt="single pass: one flat Cost per m2, as always. multi-pass (a RISO duplicator, say): each job is printed in several colour passes, costed from the Consumables sheet, and each pass costs the Template cost to set up." sqref="E7:E10" xr:uid="{7E0C9B4D-1CD0-4796-886B-114063CB99AA}">
+      <formula1>"single pass,multi-pass"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Template cost" error="Enter a number, zero or more." promptTitle="Template cost" prompt="Multi-pass printers only: what it costs to set up one colour pass (making a RISO master, for example). Charged once per pass, however many copies are run. Leave blank for none." sqref="F7:F10" xr:uid="{B07D5F39-D55C-4226-8ED1-070506AA0C67}">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
0.11.0: pass buttons clear of the job buttons; pass columns follow only their toggle
- Job row 24pt and pass row 26pt, pass buttons drawn 2pt into their row: the 22pt
  job buttons no longer run into them.
- ApplyMultiPassVisibility sets the pass columns both ways from the toggle alone,
  last in ApplyReducedView; Reduced/Minimal do not hide or show them, and a stale
  LOC_REDUCED_COLUMNS (e.g. restored from an older backup) can no longer leave the
  toggle hiding them with no way back.
- Template: Reduced list default back to its original value.
- Tests and docs updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357BC0D6-54B8-4E86-A589-5EBD0AB74D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{223B0383-FD45-44C1-95C8-7F969FEF17EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -965,7 +965,7 @@
     <t>Yes hides the multi-pass columns (Passes, Colour, Row Type, Parent, Pass) on every location sheet (toggled by the button on each one). No shows them. The Set-up Cost column belongs to the cost detail setting instead.</t>
   </si>
   <si>
-    <t>Status;Job ID;Area m2;S_SchemaVer;Passes;Colour;Row Type;Parent;Pass</t>
+    <t>Status;Job ID;Area m2;S_SchemaVer</t>
   </si>
 </sst>
 </file>
@@ -5405,10 +5405,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G11:G2001 I7:I10" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Colour mode" error="Choose single pass or multi-pass." promptTitle="Colour mode" prompt="single pass: one flat Cost per m2, as always. multi-pass (a RISO duplicator, say): each job is printed in several colour passes, costed from the Consumables sheet, and each pass costs the Template cost to set up." sqref="E7:E10" xr:uid="{7E0C9B4D-1CD0-4796-886B-114063CB99AA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Colour mode" error="Choose single pass or multi-pass." promptTitle="Colour mode" prompt="single pass: one flat Cost per m2, as always. multi-pass (a RISO duplicator, say): each job is printed in several colour passes, costed from the Consumables sheet, and each pass costs the Template cost to set up." sqref="E7:E10" xr:uid="{C7C9C186-E3F4-4132-81AC-1EF70CDD38BD}">
       <formula1>"single pass,multi-pass"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Template cost" error="Enter a number, zero or more." promptTitle="Template cost" prompt="Multi-pass printers only: what it costs to set up one colour pass (making a RISO master, for example). Charged once per pass, however many copies are run. Leave blank for none." sqref="F7:F10" xr:uid="{B07D5F39-D55C-4226-8ED1-070506AA0C67}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Template cost" error="Enter a number, zero or more." promptTitle="Template cost" prompt="Multi-pass printers only: what it costs to set up one colour pass (making a RISO master, for example). Charged once per pass, however many copies are run. Leave blank for none." sqref="F7:F10" xr:uid="{4A672B3A-63B2-4432-A54D-71083F4BA2FB}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Template: the sample room's code is EXAMPLE, not MAIN
MAIN is a natural code for a site's own first room. Re-runnable script
apply-example-code-template.ps1 rewrites LOC_Code, the table name and the twelve
sample Job IDs in src/PrintCosts.xlsx.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adash\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{223B0383-FD45-44C1-95C8-7F969FEF17EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0D7C1F7-FB22-4145-ABC6-E600B8368D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="-110" windowWidth="24420" windowHeight="14620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -473,9 +473,6 @@
     <t>Location code</t>
   </si>
   <si>
-    <t>MAIN</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -578,9 +575,6 @@
     <t>S_SchemaVer</t>
   </si>
   <si>
-    <t>UNI-MAIN-00001</t>
-  </si>
-  <si>
     <t>Jane Smith</t>
   </si>
   <si>
@@ -590,30 +584,18 @@
     <t>build</t>
   </si>
   <si>
-    <t>UNI-MAIN-00002</t>
-  </si>
-  <si>
     <t>Full-width canvas run</t>
   </si>
   <si>
-    <t>UNI-MAIN-00003</t>
-  </si>
-  <si>
     <t>Ravi Patel</t>
   </si>
   <si>
     <t>600mm print on the same roll</t>
   </si>
   <si>
-    <t>UNI-MAIN-00004</t>
-  </si>
-  <si>
     <t>Paper donated by the department</t>
   </si>
   <si>
-    <t>UNI-MAIN-00005</t>
-  </si>
-  <si>
     <t>Location settings</t>
   </si>
   <si>
@@ -632,42 +614,21 @@
     <t>Custom-size offcut stock, not a standard sheet size</t>
   </si>
   <si>
-    <t>UNI-MAIN-00006</t>
-  </si>
-  <si>
     <t>Outdoor banner vinyl, latex ink</t>
   </si>
   <si>
-    <t>UNI-MAIN-00007</t>
-  </si>
-  <si>
     <t>Student number only, given verbally at the counter</t>
   </si>
   <si>
-    <t>UNI-MAIN-00008</t>
-  </si>
-  <si>
     <t>Departmental job charged to School of Art, no student involved</t>
   </si>
   <si>
-    <t>UNI-MAIN-00009</t>
-  </si>
-  <si>
     <t>Large-format handout roll</t>
   </si>
   <si>
-    <t>UNI-MAIN-00010</t>
-  </si>
-  <si>
     <t>SAMPLE: invalid - missing student identification and print width exceeds the roll</t>
   </si>
   <si>
-    <t>UNI-MAIN-00011</t>
-  </si>
-  <si>
-    <t>UNI-MAIN-00012</t>
-  </si>
-  <si>
     <t>Open day posters</t>
   </si>
   <si>
@@ -966,6 +927,45 @@
   </si>
   <si>
     <t>Status;Job ID;Area m2;S_SchemaVer</t>
+  </si>
+  <si>
+    <t>EXAMPLE</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00001</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00002</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00003</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00004</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00005</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00006</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00007</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00008</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00009</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00010</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00011</t>
+  </si>
+  <si>
+    <t>UNI-EXAMPLE-00012</t>
   </si>
 </sst>
 </file>
@@ -1433,6 +1433,288 @@
   </cellStyles>
   <dxfs count="90">
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF2E64A8"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF2E64A8"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF2E64A8"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1495,8 +1777,79 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
-        <i/>
+        <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
@@ -1504,48 +1857,92 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF595959"/>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
-        <i/>
-        <color rgb="FF595959"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
-        <i/>
-        <color rgb="FF595959"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1589,22 +1986,6 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1633,497 +2014,6 @@
           <color rgb="FFBFBFBF"/>
         </right>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="#,##0.###"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FF2E64A8"/>
-        </left>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FF2E64A8"/>
-        </left>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FF2E64A8"/>
-        </left>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="\£#,##0.0000"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF808080"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9D9D9"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -2252,6 +2142,60 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <color rgb="FF595959"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <i/>
         <color rgb="FF595959"/>
       </font>
@@ -2400,6 +2344,62 @@
         </bottom>
         <vertical/>
         <horizontal/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="#,##0.###"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
       </border>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -2605,80 +2605,80 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_MAIN" displayName="tblJobs_MAIN" ref="A17:AS29" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="tblJobs_EXAMPLE" displayName="tblJobs_EXAMPLE" ref="A17:AS29" totalsRowShown="0">
   <autoFilter ref="A17:AS29" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="45">
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Date/Time" dataDxfId="75"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Student Name" dataDxfId="74"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Student No" dataDxfId="73"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="Technician" dataDxfId="72"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="11"/>
-    <tableColumn id="25" xr3:uid="{09F3ECAE-609E-455B-9BA8-2E241E8FAF46}" name="Passes" dataDxfId="9">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="Printer" dataDxfId="71"/>
+    <tableColumn id="25" xr3:uid="{09F3ECAE-609E-455B-9BA8-2E241E8FAF46}" name="Passes" dataDxfId="70">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="36" xr3:uid="{3444712F-EA34-42DA-B9B5-0EBBE8952B8B}" name="Colour" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="71"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="70">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</calculatedColumnFormula>
+    <tableColumn id="36" xr3:uid="{3444712F-EA34-42DA-B9B5-0EBBE8952B8B}" name="Colour" dataDxfId="69"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Paper Stock" dataDxfId="68"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="Unit" dataDxfId="67">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Qty" dataDxfId="69"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Print Width mm" dataDxfId="68"/>
-    <tableColumn id="35" xr3:uid="{E6BF4E83-281D-4CCB-8342-85AB57046527}" name="Sheet size" dataDxfId="67"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Disregard Paper" dataDxfId="66"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Disregard Consumable" dataDxfId="65"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Area m2" dataDxfId="64">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</calculatedColumnFormula>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Qty" dataDxfId="66"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Print Width mm" dataDxfId="65"/>
+    <tableColumn id="35" xr3:uid="{E6BF4E83-281D-4CCB-8342-85AB57046527}" name="Sheet size" dataDxfId="64"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Disregard Paper" dataDxfId="63"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Disregard Consumable" dataDxfId="62"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Area m2" dataDxfId="61">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="63">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Paper Cost" dataDxfId="60">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="5">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</calculatedColumnFormula>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Consumable Cost" dataDxfId="59">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="37" xr3:uid="{9D5B92B2-8D8C-4AB8-B4C8-729D5FEC16B3}" name="Set-up Cost" dataDxfId="3">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</calculatedColumnFormula>
+    <tableColumn id="37" xr3:uid="{9D5B92B2-8D8C-4AB8-B4C8-729D5FEC16B3}" name="Set-up Cost" dataDxfId="58">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="4">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</calculatedColumnFormula>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Gross Cost" dataDxfId="57">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Disregarded" dataDxfId="62">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</calculatedColumnFormula>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Disregarded" dataDxfId="56">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" name="Chargeable Cost" dataDxfId="61">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</calculatedColumnFormula>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0A00-000013000000}" name="Chargeable Cost" dataDxfId="55">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="34" xr3:uid="{9C12E379-305A-4AA1-8D70-0BFC2C6CF3C5}" name="Paid" dataDxfId="60"/>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Status" dataDxfId="59">
-      <calculatedColumnFormula>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</calculatedColumnFormula>
+    <tableColumn id="34" xr3:uid="{9C12E379-305A-4AA1-8D70-0BFC2C6CF3C5}" name="Paid" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Status" dataDxfId="53">
+      <calculatedColumnFormula>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Job ID" dataDxfId="58"/>
-    <tableColumn id="38" xr3:uid="{4D2F43D5-36A3-4912-BABA-E130C7C2146E}" name="Row Type" dataDxfId="57"/>
-    <tableColumn id="39" xr3:uid="{5A1BB7C9-ECFF-4CC8-8500-3A293A25528C}" name="Parent" dataDxfId="8"/>
-    <tableColumn id="40" xr3:uid="{3E507CE4-6A67-46A5-BB60-7B729C2D5A26}" name="Pass" dataDxfId="6"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="7"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="56">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Job ID" dataDxfId="52"/>
+    <tableColumn id="38" xr3:uid="{4D2F43D5-36A3-4912-BABA-E130C7C2146E}" name="Row Type" dataDxfId="51"/>
+    <tableColumn id="39" xr3:uid="{5A1BB7C9-ECFF-4CC8-8500-3A293A25528C}" name="Parent" dataDxfId="50"/>
+    <tableColumn id="40" xr3:uid="{3E507CE4-6A67-46A5-BB60-7B729C2D5A26}" name="Pass" dataDxfId="49"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0A00-000014000000}" name="Notes" dataDxfId="48"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0A00-000015000000}" name="H_Issues" dataDxfId="47">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="41" xr3:uid="{82AE4E46-EF17-494F-A090-ADA99BEE4E30}" name="H_Ink" dataDxfId="55">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</calculatedColumnFormula>
+    <tableColumn id="41" xr3:uid="{82AE4E46-EF17-494F-A090-ADA99BEE4E30}" name="H_Ink" dataDxfId="46">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{7A8AEB6A-0F1F-4F77-9521-2D3285156496}" name="H_Setup" dataDxfId="54">
-      <calculatedColumnFormula>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</calculatedColumnFormula>
+    <tableColumn id="42" xr3:uid="{7A8AEB6A-0F1F-4F77-9521-2D3285156496}" name="H_Setup" dataDxfId="45">
+      <calculatedColumnFormula>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="43" xr3:uid="{4F21AC66-121A-48B2-991A-1B25B7F679A0}" name="H_Notices" dataDxfId="53"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="52"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="51"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="50"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="49"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="48"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="47"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="46"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="2"/>
-    <tableColumn id="44" xr3:uid="{473158C1-5A71-4BCD-9231-D8A93A8E6E06}" name="S_SetupCost" dataDxfId="0"/>
-    <tableColumn id="45" xr3:uid="{AE04C717-F979-427D-9DE7-1B4ED6904D05}" name="S_ColourID" dataDxfId="1"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="45"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="44"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="43"/>
+    <tableColumn id="43" xr3:uid="{4F21AC66-121A-48B2-991A-1B25B7F679A0}" name="H_Notices" dataDxfId="44"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0A00-000016000000}" name="S_PrinterID" dataDxfId="43"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0A00-000017000000}" name="S_StockID" dataDxfId="42"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0A00-000018000000}" name="S_TechID" dataDxfId="41"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0A00-00001A000000}" name="S_Measure" dataDxfId="40"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0A00-00001B000000}" name="S_UnitCost" dataDxfId="39"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0A00-00001C000000}" name="S_StockWidth_mm" dataDxfId="38"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0A00-00001D000000}" name="S_SheetHeight_mm" dataDxfId="37"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0A00-00001E000000}" name="S_ConsRate" dataDxfId="36"/>
+    <tableColumn id="44" xr3:uid="{473158C1-5A71-4BCD-9231-D8A93A8E6E06}" name="S_SetupCost" dataDxfId="35"/>
+    <tableColumn id="45" xr3:uid="{AE04C717-F979-427D-9DE7-1B4ED6904D05}" name="S_ColourID" dataDxfId="34"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0A00-00001F000000}" name="S_StampedAt" dataDxfId="33"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0A00-000020000000}" name="S_StampedBy" dataDxfId="32"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0A00-000021000000}" name="S_SchemaVer" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2699,54 +2699,54 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblTechnicians" displayName="tblTechnicians" ref="A6:D9" totalsRowShown="0" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblTechnicians" displayName="tblTechnicians" ref="A6:D9" totalsRowShown="0" dataDxfId="30">
   <autoFilter ref="A6:D9" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Name" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Department" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Active" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="TechID" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Name" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Department" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Active" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblPrinters" displayName="tblPrinters" ref="A6:I10" totalsRowShown="0" dataDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblPrinters" displayName="tblPrinters" ref="A6:I10" totalsRowShown="0" dataDxfId="25">
   <autoFilter ref="A6:I10" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Model" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Consumable type" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="33"/>
-    <tableColumn id="5" xr3:uid="{15CEC00B-A782-4C1F-9D8C-FC4996A5205D}" name="Colour mode" dataDxfId="32"/>
-    <tableColumn id="9" xr3:uid="{59F8E22B-28C7-46F1-991A-38D5C4091FF4}" name="Template cost" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{27EBC752-1CF1-48B9-B798-05BFAB38AF84}" name="Max roll width mm" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{78D66AB2-9A7B-410A-92C1-2CCFD2C22414}" name="Max sheet size" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Active" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="PrinterID" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Model" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Consumable type" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Cost per m2" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{15CEC00B-A782-4C1F-9D8C-FC4996A5205D}" name="Colour mode" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{59F8E22B-28C7-46F1-991A-38D5C4091FF4}" name="Template cost" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{27EBC752-1CF1-48B9-B798-05BFAB38AF84}" name="Max roll width mm" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{78D66AB2-9A7B-410A-92C1-2CCFD2C22414}" name="Max sheet size" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Active" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:L15" totalsRowShown="0" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="tblPapers" displayName="tblPapers" ref="A6:L15" totalsRowShown="0" dataDxfId="15">
   <autoFilter ref="A6:L15" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Description" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Paper type" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Measure" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Size mode" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Std. size" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Width mm" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Height mm" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Cost" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Cost unit" dataDxfId="17">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="StockID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Description" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Paper type" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Measure" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Size mode" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Std. size" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Width mm" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Height mm" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Cost" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Cost unit" dataDxfId="5">
       <calculatedColumnFormula>IF(tblPapers[[#This Row],[Measure]]="","",IF(tblPapers[[#This Row],[Measure]]="Sheet","£ per sheet","£ per metre"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Active" dataDxfId="16"/>
-    <tableColumn id="13" xr3:uid="{62AE4E30-01F2-4D26-B1F8-C8FD5BF6FCC9}" name="Supplied by student" dataDxfId="15"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Active" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{62AE4E30-01F2-4D26-B1F8-C8FD5BF6FCC9}" name="Supplied by student" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2808,8 +2808,8 @@
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="Name"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Department"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="Rows"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="First date" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Last date" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="First date" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Last date" dataDxfId="1"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="State"/>
     <tableColumn id="9" xr3:uid="{F307D930-BB9C-468F-AC38-00DA61DF508D}" name="Last export"/>
     <tableColumn id="10" xr3:uid="{B7692E42-45DD-48C6-8B10-C3C464C1B69D}" name="Export sig"/>
@@ -3151,13 +3151,13 @@
         <v>127</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>196</v>
+        <v>183</v>
       </c>
       <c r="AW1" s="18" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="AZ1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:52" x14ac:dyDescent="0.35">
@@ -3171,74 +3171,74 @@
         <v>128</v>
       </c>
       <c r="AX2" t="s">
-        <v>129</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:52" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>225</v>
+        <v>212</v>
       </c>
       <c r="B4" s="32"/>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>226</v>
+        <v>213</v>
       </c>
       <c r="B5" s="33"/>
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>227</v>
+        <v>214</v>
       </c>
       <c r="B6" s="33"/>
       <c r="AW6" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="AX6" t="s">
         <v>131</v>
-      </c>
-      <c r="AX6" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:52" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:52" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AW8" s="42" t="s">
-        <v>233</v>
+        <v>220</v>
       </c>
       <c r="AX8" s="28" t="s">
-        <v>234</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AW9" s="18" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="AX9" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.35">
       <c r="AW10" s="19" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>228</v>
+        <v>215</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>229</v>
+        <v>216</v>
       </c>
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>230</v>
+        <v>217</v>
       </c>
       <c r="B12" s="5" t="str">
         <f>_xlfn.LET(_xlpm.list,LOC_Printers,_xlpm.n,IF(_xlpm.list="",0,LEN(_xlpm.list)-LEN(SUBSTITUTE(_xlpm.list,";",""))+1),IF(_xlpm.n=0,"0 printers ()",_xlpm.n&amp;" printer"&amp;IF(_xlpm.n=1,"","s")&amp;" ("&amp;SUBSTITUTE(_xlpm.list,";",", ")&amp;")"))</f>
@@ -3247,10 +3247,10 @@
     </row>
     <row r="13" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A13" s="27" t="s">
-        <v>231</v>
+        <v>218</v>
       </c>
       <c r="B13">
-        <f>ROWS(tblJobs_MAIN[])</f>
+        <f>ROWS(tblJobs_EXAMPLE[])</f>
         <v>12</v>
       </c>
     </row>
@@ -3265,139 +3265,139 @@
     </row>
     <row r="17" spans="1:45" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="F17" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="H17" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="H17" s="4" t="s">
+      <c r="I17" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="J17" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="K17" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="J17" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="K17" s="4" t="s">
+      <c r="L17" s="23" t="s">
+        <v>219</v>
+      </c>
+      <c r="M17" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="L17" s="23" t="s">
-        <v>232</v>
-      </c>
-      <c r="M17" s="4" t="s">
+      <c r="N17" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="N17" s="4" t="s">
+      <c r="O17" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="O17" s="4" t="s">
+      <c r="P17" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="P17" s="4" t="s">
+      <c r="Q17" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="Q17" s="4" t="s">
+      <c r="R17" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="S17" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="R17" s="4" t="s">
-        <v>276</v>
-      </c>
-      <c r="S17" s="4" t="s">
+      <c r="T17" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="T17" s="4" t="s">
+      <c r="U17" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="U17" s="4" t="s">
-        <v>151</v>
-      </c>
       <c r="V17" s="23" t="s">
-        <v>223</v>
+        <v>210</v>
       </c>
       <c r="W17" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="X17" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="X17" s="4" t="s">
-        <v>135</v>
-      </c>
       <c r="Y17" s="4" t="s">
-        <v>277</v>
+        <v>264</v>
       </c>
       <c r="Z17" s="4" t="s">
-        <v>278</v>
+        <v>265</v>
       </c>
       <c r="AA17" s="4" t="s">
-        <v>279</v>
+        <v>266</v>
       </c>
       <c r="AB17" s="4" t="s">
         <v>6</v>
       </c>
       <c r="AC17" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="AD17" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="AE17" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="AF17" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="AG17" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="AD17" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="AE17" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="AF17" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="AG17" s="4" t="s">
+      <c r="AH17" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="AH17" s="4" t="s">
+      <c r="AI17" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="AI17" s="4" t="s">
+      <c r="AJ17" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="AJ17" s="4" t="s">
+      <c r="AK17" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="AK17" s="4" t="s">
+      <c r="AL17" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="AL17" s="4" t="s">
+      <c r="AM17" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="AM17" s="4" t="s">
+      <c r="AN17" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="AN17" s="4" t="s">
+      <c r="AO17" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="AP17" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="AQ17" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="AO17" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="AP17" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="AQ17" s="4" t="s">
+      <c r="AR17" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="AR17" s="4" t="s">
+      <c r="AS17" s="4" t="s">
         <v>162</v>
-      </c>
-      <c r="AS17" s="4" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:45" x14ac:dyDescent="0.35">
@@ -3405,7 +3405,7 @@
         <v>46280.425000000003</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C18" s="12">
         <v>2201884</v>
@@ -3417,7 +3417,7 @@
         <v>83</v>
       </c>
       <c r="F18" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G18" s="12"/>
@@ -3425,7 +3425,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
       <c r="J18" s="13">
@@ -3434,65 +3434,65 @@
       <c r="K18" s="36"/>
       <c r="L18" s="39"/>
       <c r="M18" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N18" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O18" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>14.400000000000002</v>
       </c>
       <c r="P18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>31</v>
       </c>
       <c r="Q18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>13.68</v>
       </c>
       <c r="R18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>44.68</v>
       </c>
       <c r="T18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U18" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>44.68</v>
       </c>
       <c r="V18" s="34"/>
       <c r="W18" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X18" s="5" t="s">
-        <v>164</v>
+        <v>282</v>
       </c>
       <c r="Y18" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z18" s="5"/>
       <c r="AA18" s="49"/>
       <c r="AB18" s="12" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="AC18" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD18" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE18" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF18" s="16"/>
@@ -3526,7 +3526,7 @@
         <v>46280.425000000003</v>
       </c>
       <c r="AR18" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS18" s="16">
         <v>1</v>
@@ -3537,7 +3537,7 @@
         <v>46280.611111111109</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C19" s="12">
         <v>2201884</v>
@@ -3549,7 +3549,7 @@
         <v>79</v>
       </c>
       <c r="F19" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G19" s="12"/>
@@ -3557,7 +3557,7 @@
         <v>106</v>
       </c>
       <c r="I19" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="J19" s="13">
@@ -3566,65 +3566,65 @@
       <c r="K19" s="36"/>
       <c r="L19" s="39"/>
       <c r="M19" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N19" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O19" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>10.968</v>
       </c>
       <c r="P19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>105</v>
       </c>
       <c r="Q19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>31.26</v>
       </c>
       <c r="R19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>136.26</v>
       </c>
       <c r="T19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U19" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>136.26</v>
       </c>
       <c r="V19" s="35"/>
       <c r="W19" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X19" s="5" t="s">
-        <v>168</v>
+        <v>283</v>
       </c>
       <c r="Y19" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z19" s="5"/>
       <c r="AA19" s="49"/>
       <c r="AB19" s="12" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AC19" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD19" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE19" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF19" s="16"/>
@@ -3656,7 +3656,7 @@
         <v>46280.611111111109</v>
       </c>
       <c r="AR19" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS19" s="16">
         <v>1</v>
@@ -3667,7 +3667,7 @@
         <v>46281.461805555555</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C20" s="12">
         <v>2203110</v>
@@ -3679,7 +3679,7 @@
         <v>79</v>
       </c>
       <c r="F20" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G20" s="12"/>
@@ -3687,7 +3687,7 @@
         <v>106</v>
       </c>
       <c r="I20" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="J20" s="13">
@@ -3698,65 +3698,65 @@
       </c>
       <c r="L20" s="39"/>
       <c r="M20" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N20" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O20" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>7.1999999999999993</v>
       </c>
       <c r="P20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>105</v>
       </c>
       <c r="Q20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>20.52</v>
       </c>
       <c r="R20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>125.52</v>
       </c>
       <c r="T20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U20" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>125.52</v>
       </c>
       <c r="V20" s="35"/>
       <c r="W20" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X20" s="5" t="s">
-        <v>170</v>
+        <v>284</v>
       </c>
       <c r="Y20" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z20" s="5"/>
       <c r="AA20" s="49"/>
       <c r="AB20" s="12" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="AC20" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD20" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE20" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF20" s="16"/>
@@ -3788,7 +3788,7 @@
         <v>46281.461805555555</v>
       </c>
       <c r="AR20" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS20" s="16">
         <v>1</v>
@@ -3799,7 +3799,7 @@
         <v>46281.638888888891</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C21" s="12">
         <v>2203110</v>
@@ -3811,7 +3811,7 @@
         <v>79</v>
       </c>
       <c r="F21" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G21" s="12"/>
@@ -3819,7 +3819,7 @@
         <v>104</v>
       </c>
       <c r="I21" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="J21" s="13">
@@ -3831,62 +3831,62 @@
         <v>38</v>
       </c>
       <c r="N21" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O21" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>3.05</v>
       </c>
       <c r="P21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>15.5</v>
       </c>
       <c r="Q21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>8.69</v>
       </c>
       <c r="R21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>24.189999999999998</v>
       </c>
       <c r="T21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>15.499999999999998</v>
       </c>
       <c r="U21" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>8.69</v>
       </c>
       <c r="V21" s="35"/>
       <c r="W21" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X21" s="5" t="s">
-        <v>173</v>
+        <v>285</v>
       </c>
       <c r="Y21" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z21" s="5"/>
       <c r="AA21" s="49"/>
       <c r="AB21" s="12" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="AC21" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD21" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE21" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF21" s="16"/>
@@ -3918,7 +3918,7 @@
         <v>46281.638888888891</v>
       </c>
       <c r="AR21" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS21" s="16">
         <v>1</v>
@@ -3929,7 +3929,7 @@
         <v>46282.381944444445</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C22" s="12">
         <v>2204521</v>
@@ -3941,7 +3941,7 @@
         <v>83</v>
       </c>
       <c r="F22" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G22" s="12"/>
@@ -3949,7 +3949,7 @@
         <v>102</v>
       </c>
       <c r="I22" s="9" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
       <c r="J22" s="13">
@@ -3958,65 +3958,65 @@
       <c r="K22" s="36"/>
       <c r="L22" s="39"/>
       <c r="M22" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N22" s="12" t="s">
         <v>38</v>
       </c>
       <c r="O22" s="14">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>3.1184999999999996</v>
       </c>
       <c r="P22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>2.25</v>
       </c>
       <c r="Q22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>2.96</v>
       </c>
       <c r="R22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>5.21</v>
       </c>
       <c r="T22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>2.96</v>
       </c>
       <c r="U22" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>2.25</v>
       </c>
       <c r="V22" s="35"/>
       <c r="W22" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X22" s="5" t="s">
-        <v>175</v>
+        <v>286</v>
       </c>
       <c r="Y22" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z22" s="5"/>
       <c r="AA22" s="49"/>
       <c r="AB22" s="12" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="AC22" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD22" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE22" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF22" s="16"/>
@@ -4050,7 +4050,7 @@
         <v>46282.381944444445</v>
       </c>
       <c r="AR22" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS22" s="16">
         <v>1</v>
@@ -4061,7 +4061,7 @@
         <v>46282.559027777781</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C23" s="12">
         <v>2204521</v>
@@ -4073,7 +4073,7 @@
         <v>83</v>
       </c>
       <c r="F23" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G23" s="12"/>
@@ -4081,7 +4081,7 @@
         <v>112</v>
       </c>
       <c r="I23" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
       <c r="J23" s="13">
@@ -4090,65 +4090,65 @@
       <c r="K23" s="36"/>
       <c r="L23" s="39"/>
       <c r="M23" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N23" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O23" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>2.16</v>
       </c>
       <c r="P23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>2.7</v>
       </c>
       <c r="Q23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>2.0499999999999998</v>
       </c>
       <c r="R23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>4.75</v>
       </c>
       <c r="T23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U23" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>4.75</v>
       </c>
       <c r="V23" s="35"/>
       <c r="W23" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X23" s="5" t="s">
-        <v>182</v>
+        <v>287</v>
       </c>
       <c r="Y23" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z23" s="5"/>
       <c r="AA23" s="49"/>
       <c r="AB23" s="12" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="AC23" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD23" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE23" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF23" s="16"/>
@@ -4182,7 +4182,7 @@
         <v>46282.559027777781</v>
       </c>
       <c r="AR23" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS23" s="16">
         <v>1</v>
@@ -4193,7 +4193,7 @@
         <v>46282.666666666664</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C24" s="12">
         <v>2204521</v>
@@ -4205,7 +4205,7 @@
         <v>85</v>
       </c>
       <c r="F24" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G24" s="12"/>
@@ -4213,7 +4213,7 @@
         <v>108</v>
       </c>
       <c r="I24" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="J24" s="13">
@@ -4222,65 +4222,65 @@
       <c r="K24" s="36"/>
       <c r="L24" s="39"/>
       <c r="M24" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N24" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O24" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>10.96</v>
       </c>
       <c r="P24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>91.2</v>
       </c>
       <c r="Q24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>19.18</v>
       </c>
       <c r="R24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>110.38</v>
       </c>
       <c r="T24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U24" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>110.38</v>
       </c>
       <c r="V24" s="35"/>
       <c r="W24" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X24" s="5" t="s">
-        <v>184</v>
+        <v>288</v>
       </c>
       <c r="Y24" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z24" s="5"/>
       <c r="AA24" s="49"/>
       <c r="AB24" s="12" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="AC24" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD24" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE24" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF24" s="16"/>
@@ -4312,7 +4312,7 @@
         <v>46282.666666666664</v>
       </c>
       <c r="AR24" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS24" s="16">
         <v>1</v>
@@ -4333,7 +4333,7 @@
         <v>81</v>
       </c>
       <c r="F25" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G25" s="12"/>
@@ -4341,7 +4341,7 @@
         <v>104</v>
       </c>
       <c r="I25" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="J25" s="13">
@@ -4350,65 +4350,65 @@
       <c r="K25" s="36"/>
       <c r="L25" s="39"/>
       <c r="M25" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N25" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O25" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>1.83</v>
       </c>
       <c r="P25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>9.3000000000000007</v>
       </c>
       <c r="Q25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>4.3899999999999997</v>
       </c>
       <c r="R25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>13.690000000000001</v>
       </c>
       <c r="T25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U25" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>13.690000000000001</v>
       </c>
       <c r="V25" s="35"/>
       <c r="W25" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X25" s="5" t="s">
-        <v>186</v>
+        <v>289</v>
       </c>
       <c r="Y25" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z25" s="5"/>
       <c r="AA25" s="49"/>
       <c r="AB25" s="12" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="AC25" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD25" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE25" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF25" s="16"/>
@@ -4440,7 +4440,7 @@
         <v>46283.427083333336</v>
       </c>
       <c r="AR25" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS25" s="16">
         <v>1</v>
@@ -4461,7 +4461,7 @@
         <v>83</v>
       </c>
       <c r="F26" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G26" s="12"/>
@@ -4469,7 +4469,7 @@
         <v>98</v>
       </c>
       <c r="I26" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
       <c r="J26" s="13">
@@ -4478,65 +4478,65 @@
       <c r="K26" s="36"/>
       <c r="L26" s="39"/>
       <c r="M26" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N26" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O26" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>7.4843999999999991</v>
       </c>
       <c r="P26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>7.2</v>
       </c>
       <c r="Q26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>7.11</v>
       </c>
       <c r="R26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>14.31</v>
       </c>
       <c r="T26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U26" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>14.31</v>
       </c>
       <c r="V26" s="35"/>
       <c r="W26" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X26" s="5" t="s">
-        <v>188</v>
+        <v>290</v>
       </c>
       <c r="Y26" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z26" s="5"/>
       <c r="AA26" s="49"/>
       <c r="AB26" s="12" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="AC26" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD26" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE26" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF26" s="16"/>
@@ -4570,7 +4570,7 @@
         <v>46283.486111111109</v>
       </c>
       <c r="AR26" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS26" s="16">
         <v>1</v>
@@ -4581,7 +4581,7 @@
         <v>46283.638888888891</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C27" s="12">
         <v>2204521</v>
@@ -4593,7 +4593,7 @@
         <v>79</v>
       </c>
       <c r="F27" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G27" s="12"/>
@@ -4601,7 +4601,7 @@
         <v>110</v>
       </c>
       <c r="I27" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="J27" s="13">
@@ -4610,65 +4610,65 @@
       <c r="K27" s="36"/>
       <c r="L27" s="39"/>
       <c r="M27" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N27" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O27" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>21.34</v>
       </c>
       <c r="P27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>112</v>
       </c>
       <c r="Q27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>60.82</v>
       </c>
       <c r="R27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>172.82</v>
       </c>
       <c r="T27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U27" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>172.82</v>
       </c>
       <c r="V27" s="35"/>
       <c r="W27" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X27" s="5" t="s">
-        <v>190</v>
+        <v>291</v>
       </c>
       <c r="Y27" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z27" s="5"/>
       <c r="AA27" s="49"/>
       <c r="AB27" s="12" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="AC27" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD27" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE27" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF27" s="16"/>
@@ -4700,7 +4700,7 @@
         <v>46283.638888888891</v>
       </c>
       <c r="AR27" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS27" s="16">
         <v>1</v>
@@ -4711,7 +4711,7 @@
         <v>46284.34375</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C28" s="12">
         <v>2203110</v>
@@ -4723,7 +4723,7 @@
         <v>83</v>
       </c>
       <c r="F28" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G28" s="12"/>
@@ -4731,7 +4731,7 @@
         <v>95</v>
       </c>
       <c r="I28" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>sheets</v>
       </c>
       <c r="J28" s="13">
@@ -4740,65 +4740,65 @@
       <c r="K28" s="36"/>
       <c r="L28" s="39"/>
       <c r="M28" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N28" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O28" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>19.982159999999997</v>
       </c>
       <c r="P28" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>16.8</v>
       </c>
       <c r="Q28" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>18.98</v>
       </c>
       <c r="R28" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S28" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>35.78</v>
       </c>
       <c r="T28" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U28" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>35.78</v>
       </c>
       <c r="V28" s="35"/>
       <c r="W28" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>OK</v>
       </c>
       <c r="X28" s="5" t="s">
-        <v>192</v>
+        <v>292</v>
       </c>
       <c r="Y28" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z28" s="5"/>
       <c r="AA28" s="49"/>
       <c r="AB28" s="12" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="AC28" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v/>
       </c>
       <c r="AD28" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE28" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF28" s="16"/>
@@ -4832,7 +4832,7 @@
         <v>46284.34375</v>
       </c>
       <c r="AR28" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS28" s="16">
         <v>1</v>
@@ -4851,7 +4851,7 @@
         <v>79</v>
       </c>
       <c r="F29" s="49" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]])=0,"",COUNTIFS(tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v/>
       </c>
       <c r="G29" s="12"/>
@@ -4859,7 +4859,7 @@
         <v>106</v>
       </c>
       <c r="I29" s="20" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[S_Measure]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet","sheets",IF(LOC_RollUnit="Centimetres","cm","metres")))</f>
         <v>metres</v>
       </c>
       <c r="J29" s="13">
@@ -4870,65 +4870,65 @@
       </c>
       <c r="L29" s="39"/>
       <c r="M29" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N29" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O29" s="21">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",IF(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",(tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_MAIN[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_MAIN[[#This Row],[Qty]],(IF(tblJobs_MAIN[[#This Row],[Print Width mm]]="",tblJobs_MAIN[[#This Row],[S_StockWidth_mm]],tblJobs_MAIN[[#This Row],[Print Width mm]])/1000)*tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",IF(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",(tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]/1000)*(tblJobs_EXAMPLE[[#This Row],[S_SheetHeight_mm]]/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]],(IF(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]="",tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]],tblJobs_EXAMPLE[[#This Row],[Print Width mm]])/1000)*tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)))</f>
         <v>14.399999999999999</v>
       </c>
       <c r="P29" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Qty]]="","",ROUND(tblJobs_MAIN[[#This Row],[Qty]]/IF(tblJobs_MAIN[[#This Row],[Unit]]="cm",100,1)*tblJobs_MAIN[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Qty]]/IF(tblJobs_EXAMPLE[[#This Row],[Unit]]="cm",100,1)*tblJobs_EXAMPLE[[#This Row],[S_UnitCost]],SET_ROUND_DP))</f>
         <v>105</v>
       </c>
       <c r="Q29" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Ink]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",ROUND(tblJobs_MAIN[[#This Row],[Area m2]]*tblJobs_MAIN[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Ink],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Ink]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",ROUND(tblJobs_EXAMPLE[[#This Row],[Area m2]]*tblJobs_EXAMPLE[[#This Row],[S_ConsRate]],SET_ROUND_DP)+IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Ink],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>41.04</v>
       </c>
       <c r="R29" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]="Pass",tblJobs_MAIN[[#This Row],[H_Setup]],IF(tblJobs_MAIN[[#This Row],[Area m2]]="","",IF(tblJobs_MAIN[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_MAIN[H_Setup],tblJobs_MAIN[Parent],tblJobs_MAIN[[#This Row],[Job ID]]))))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]="Pass",tblJobs_EXAMPLE[[#This Row],[H_Setup]],IF(tblJobs_EXAMPLE[[#This Row],[Area m2]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",0,SUMIFS(tblJobs_EXAMPLE[H_Setup],tblJobs_EXAMPLE[Parent],tblJobs_EXAMPLE[[#This Row],[Job ID]]))))</f>
         <v>0</v>
       </c>
       <c r="S29" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",tblJobs_MAIN[[#This Row],[Paper Cost]]+tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Paper Cost]]+tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]]))</f>
         <v>146.04</v>
       </c>
       <c r="T29" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Gross Cost]]="","",tblJobs_MAIN[[#This Row],[Gross Cost]]-tblJobs_MAIN[[#This Row],[Chargeable Cost]])</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Gross Cost]]="","",tblJobs_EXAMPLE[[#This Row],[Gross Cost]]-tblJobs_EXAMPLE[[#This Row],[Chargeable Cost]])</f>
         <v>0</v>
       </c>
       <c r="U29" s="15">
-        <f>IF(tblJobs_MAIN[[#This Row],[Paper Cost]]="","",IF(tblJobs_MAIN[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_MAIN[[#This Row],[Paper Cost]])+IF(tblJobs_MAIN[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_MAIN[[#This Row],[Consumable Cost]]+N(tblJobs_MAIN[[#This Row],[Set-up Cost]])))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Paper Cost]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Disregard Paper]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Paper Cost]])+IF(tblJobs_EXAMPLE[[#This Row],[Disregard Consumable]]="Yes",0,tblJobs_EXAMPLE[[#This Row],[Consumable Cost]]+N(tblJobs_EXAMPLE[[#This Row],[Set-up Cost]])))</f>
         <v>146.04</v>
       </c>
       <c r="V29" s="35"/>
       <c r="W29" s="9" t="str">
-        <f>IF(AND(tblJobs_MAIN[[#This Row],[Job ID]]="",tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_MAIN[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Issues]],3,255),IF(tblJobs_MAIN[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_MAIN[[#This Row],[H_Notices]],3,255),"OK")))</f>
+        <f>IF(AND(tblJobs_EXAMPLE[[#This Row],[Job ID]]="",tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass"),"",IF(tblJobs_EXAMPLE[[#This Row],[H_Issues]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Issues]],3,255),IF(tblJobs_EXAMPLE[[#This Row],[H_Notices]]&lt;&gt;"",MID(tblJobs_EXAMPLE[[#This Row],[H_Notices]],3,255),"OK")))</f>
         <v>Student name or number required; Print width exceeds stock width</v>
       </c>
       <c r="X29" s="5" t="s">
-        <v>193</v>
+        <v>293</v>
       </c>
       <c r="Y29" s="5" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="Z29" s="5"/>
       <c r="AA29" s="49"/>
       <c r="AB29" s="12" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="AC29" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Job ID]]="","",IF(tblJobs_MAIN[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Student Name]]="",tblJobs_MAIN[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_MAIN[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_MAIN[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_MAIN[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_MAIN[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_MAIN[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_MAIN[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[S_Measure]]="Sheet",tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_MAIN[[#This Row],[Print Width mm]]&gt;tblJobs_MAIN[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_MAIN[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_MAIN[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_MAIN[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Job ID]]="","",IF(tblJobs_EXAMPLE[[#This Row],[Date/Time]]="","; Date and time required","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Student Name]]="",tblJobs_EXAMPLE[[#This Row],[Student No]]=""),"; Student name or number required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Technician]]="","; Technician required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Printer]]="","; Printer required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="","; Paper stock required","")&amp;IF(tblJobs_EXAMPLE[[#This Row],[Qty]]="","; Quantity required",IF(tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;=0,"; Quantity must be greater than zero",""))&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Qty]]&lt;&gt;INT(tblJobs_EXAMPLE[[#This Row],[Qty]])),"; Sheet quantity must be a whole number","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[S_Measure]]="Sheet",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;""),"; Print width does not apply to sheet stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&lt;&gt;"",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]&gt;tblJobs_EXAMPLE[[#This Row],[S_StockWidth_mm]]),"; Print width exceeds stock width","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Roll)",tblJobs_EXAMPLE[[#This Row],[Print Width mm]]=""),"; Print width required for student-supplied roll stock","")&amp;IF(AND(tblJobs_EXAMPLE[[#This Row],[Paper Stock]]="Supplied (Sheet)",tblJobs_EXAMPLE[[#This Row],[Sheet size]]=""),"; Sheet size required for student-supplied sheet stock",""))</f>
         <v>; Student name or number required; Print width exceeds stock width</v>
       </c>
       <c r="AD29" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_MAIN[[#This Row],[Parent]],tblJobs_MAIN[Job ID],tblJobs_MAIN[Area m2])*N(tblJobs_MAIN[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",IFERROR(ROUND(_xlfn.XLOOKUP(tblJobs_EXAMPLE[[#This Row],[Parent]],tblJobs_EXAMPLE[Job ID],tblJobs_EXAMPLE[Area m2])*N(tblJobs_EXAMPLE[[#This Row],[S_ConsRate]]),SET_ROUND_DP),0))</f>
         <v/>
       </c>
       <c r="AE29" s="16" t="str">
-        <f>IF(tblJobs_MAIN[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_MAIN[[#This Row],[S_SetupCost]]))</f>
+        <f>IF(tblJobs_EXAMPLE[[#This Row],[Row Type]]&lt;&gt;"Pass","",N(tblJobs_EXAMPLE[[#This Row],[S_SetupCost]]))</f>
         <v/>
       </c>
       <c r="AF29" s="16"/>
@@ -4960,7 +4960,7 @@
         <v>46284.395833333336</v>
       </c>
       <c r="AR29" s="16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="AS29" s="16">
         <v>1</v>
@@ -4969,7 +4969,7 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <conditionalFormatting sqref="W18:W29">
-    <cfRule type="expression" dxfId="12" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
       <formula>AND(W18&lt;&gt;"",W18&lt;&gt;"OK")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5170,7 +5170,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="30" t="s">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="B7" s="24" t="s">
         <v>67</v>
@@ -5184,7 +5184,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="30" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>69</v>
@@ -5198,7 +5198,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="30" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>71</v>
@@ -5251,7 +5251,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="H4" s="2" t="s">
-        <v>221</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -5271,16 +5271,16 @@
         <v>77</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>36</v>
@@ -5288,7 +5288,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="30" t="s">
-        <v>261</v>
+        <v>248</v>
       </c>
       <c r="B7" s="24" t="s">
         <v>79</v>
@@ -5300,7 +5300,7 @@
         <v>2.85</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="F7" s="44"/>
       <c r="G7" s="45">
@@ -5313,7 +5313,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="30" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>81</v>
@@ -5325,7 +5325,7 @@
         <v>2.4</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="F8" s="44"/>
       <c r="G8" s="46">
@@ -5338,7 +5338,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="30" t="s">
-        <v>263</v>
+        <v>250</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>83</v>
@@ -5350,7 +5350,7 @@
         <v>0.95</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="F9" s="44"/>
       <c r="G9" s="46"/>
@@ -5363,7 +5363,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="30" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>85</v>
@@ -5375,7 +5375,7 @@
         <v>1.75</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="F10" s="44"/>
       <c r="G10" s="46">
@@ -5472,7 +5472,7 @@
         <v>91</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>48</v>
@@ -5490,12 +5490,12 @@
         <v>36</v>
       </c>
       <c r="L6" s="22" t="s">
-        <v>222</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="30" t="s">
-        <v>265</v>
+        <v>252</v>
       </c>
       <c r="B7" s="24" t="s">
         <v>95</v>
@@ -5529,12 +5529,12 @@
         <v>38</v>
       </c>
       <c r="L7" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="30" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>98</v>
@@ -5568,12 +5568,12 @@
         <v>38</v>
       </c>
       <c r="L8" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="30" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>100</v>
@@ -5607,12 +5607,12 @@
         <v>38</v>
       </c>
       <c r="L9" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="30" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>102</v>
@@ -5646,12 +5646,12 @@
         <v>38</v>
       </c>
       <c r="L10" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="30" t="s">
-        <v>269</v>
+        <v>256</v>
       </c>
       <c r="B11" s="24" t="s">
         <v>104</v>
@@ -5681,12 +5681,12 @@
         <v>38</v>
       </c>
       <c r="L11" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="30" t="s">
-        <v>270</v>
+        <v>257</v>
       </c>
       <c r="B12" s="24" t="s">
         <v>106</v>
@@ -5716,12 +5716,12 @@
         <v>38</v>
       </c>
       <c r="L12" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="30" t="s">
-        <v>271</v>
+        <v>258</v>
       </c>
       <c r="B13" s="24" t="s">
         <v>108</v>
@@ -5751,12 +5751,12 @@
         <v>38</v>
       </c>
       <c r="L13" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="30" t="s">
-        <v>272</v>
+        <v>259</v>
       </c>
       <c r="B14" s="24" t="s">
         <v>110</v>
@@ -5786,12 +5786,12 @@
         <v>38</v>
       </c>
       <c r="L14" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="30" t="s">
-        <v>273</v>
+        <v>260</v>
       </c>
       <c r="B15" s="24" t="s">
         <v>112</v>
@@ -5823,7 +5823,7 @@
         <v>38</v>
       </c>
       <c r="L15" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -6123,7 +6123,7 @@
         <v>297</v>
       </c>
       <c r="M13" s="24" t="s">
-        <v>289</v>
+        <v>276</v>
       </c>
       <c r="N13" s="24" t="s">
         <v>38</v>
@@ -6188,182 +6188,182 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="C17" s="40" t="s">
-        <v>245</v>
+        <v>232</v>
       </c>
       <c r="D17" s="26" t="s">
-        <v>202</v>
+        <v>189</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>203</v>
+        <v>190</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="C18" s="43">
         <v>46294.403460648151</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>205</v>
+        <v>192</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="C19" s="40" t="s">
-        <v>235</v>
+        <v>222</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>208</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>210</v>
+        <v>197</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="26" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>246</v>
+        <v>233</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>248</v>
+        <v>235</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>213</v>
+        <v>200</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>293</v>
+        <v>280</v>
       </c>
       <c r="D22" s="26" t="s">
-        <v>249</v>
+        <v>236</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
-        <v>250</v>
+        <v>237</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>251</v>
+        <v>238</v>
       </c>
       <c r="C23" s="48" t="s">
-        <v>253</v>
+        <v>240</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>216</v>
+        <v>203</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>217</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="58" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
-        <v>290</v>
+        <v>277</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="C25" s="48" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>292</v>
+        <v>279</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="C26" s="48">
         <v>3</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>238</v>
+        <v>225</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
-        <v>239</v>
+        <v>226</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>240</v>
+        <v>227</v>
       </c>
       <c r="C27" s="48">
         <v>4</v>
       </c>
       <c r="D27" s="26" t="s">
-        <v>241</v>
+        <v>228</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>242</v>
+        <v>229</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>243</v>
+        <v>230</v>
       </c>
       <c r="C28" s="48">
         <v>9</v>
       </c>
       <c r="D28" s="26" t="s">
-        <v>244</v>
+        <v>231</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>255</v>
+        <v>242</v>
       </c>
       <c r="C29" s="48" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="D29" s="26" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -6430,24 +6430,24 @@
         <v>120</v>
       </c>
       <c r="I1" s="22" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="J1" s="22" t="s">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="K1" s="22" t="s">
-        <v>199</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="22" t="s">
-        <v>196</v>
+        <v>183</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>129</v>
+        <v>281</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>196</v>
+        <v>183</v>
       </c>
       <c r="D2" s="22" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Stop a new print room taking another room's code (0.11.4)
Add print room's code prompt refuses a code another room has and
re-asks with a free suggestion (RoomUsingCode, FreeCode). Refresh
Locations now lets registered rooms claim their codes before newcomers:
in plain sheet order a new room, inserted right after the first room,
took a later room's code, that room was renumbered while its jobs kept
the old IDs, and the new room issued the same job IDs again.

Template: the sample jobs' snapshot IDs now follow the catalogue model
(UNI-PRN-0003 etc.), via mac/apply-sample-ids-template.py. New
test-roomcode (.ps1 and mac/.py). SETUP.md also corrected on the
Settings lookup tables' + and - buttons.

Not yet run in Excel; Windows untested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -284,19 +284,19 @@
     <t>Name</t>
   </si>
   <si>
-    <t>TEC-001</t>
+    <t>UNI-TCH-0001</t>
   </si>
   <si>
     <t>A. Shailer</t>
   </si>
   <si>
-    <t>TEC-002</t>
+    <t>UNI-TCH-0002</t>
   </si>
   <si>
     <t>J. Okonkwo</t>
   </si>
   <si>
-    <t>TEC-003</t>
+    <t>UNI-TCH-0003</t>
   </si>
   <si>
     <t>M. Da Silva</t>
@@ -320,25 +320,25 @@
     <t>Cost per m2</t>
   </si>
   <si>
-    <t>PRN-001</t>
+    <t>UNI-PRN-0001</t>
   </si>
   <si>
     <t>Epson SureColor P9500</t>
   </si>
   <si>
-    <t>PRN-002</t>
+    <t>UNI-PRN-0002</t>
   </si>
   <si>
     <t>HP DesignJet Z9+</t>
   </si>
   <si>
-    <t>PRN-003</t>
+    <t>UNI-PRN-0003</t>
   </si>
   <si>
     <t>Xerox Versant 180</t>
   </si>
   <si>
-    <t>PRN-004</t>
+    <t>UNI-PRN-0004</t>
   </si>
   <si>
     <t>HP Latex 335</t>
@@ -368,7 +368,7 @@
     <t>Cost unit</t>
   </si>
   <si>
-    <t>STK-001</t>
+    <t>UNI-STK-0001</t>
   </si>
   <si>
     <t>Matte 180gsm A1 sheet</t>
@@ -377,49 +377,49 @@
     <t>Standard</t>
   </si>
   <si>
-    <t>STK-002</t>
+    <t>UNI-STK-0002</t>
   </si>
   <si>
     <t>Matte 180gsm A2 sheet</t>
   </si>
   <si>
-    <t>STK-003</t>
+    <t>UNI-STK-0003</t>
   </si>
   <si>
     <t>Gloss 200gsm SRA3 sheet</t>
   </si>
   <si>
-    <t>STK-004</t>
+    <t>UNI-STK-0004</t>
   </si>
   <si>
     <t>Uncoated 120gsm A3 sheet</t>
   </si>
   <si>
-    <t>STK-005</t>
+    <t>UNI-STK-0005</t>
   </si>
   <si>
     <t>Satin photo 610mm roll</t>
   </si>
   <si>
-    <t>STK-006</t>
+    <t>UNI-STK-0006</t>
   </si>
   <si>
     <t>Canvas 914mm roll</t>
   </si>
   <si>
-    <t>STK-007</t>
+    <t>UNI-STK-0007</t>
   </si>
   <si>
     <t>Vinyl self-adhesive 1370mm roll</t>
   </si>
   <si>
-    <t>STK-008</t>
+    <t>UNI-STK-0008</t>
   </si>
   <si>
     <t>Matte 180gsm 1067mm roll</t>
   </si>
   <si>
-    <t>STK-009</t>
+    <t>UNI-STK-0009</t>
   </si>
   <si>
     <t>Gloss offcut 320x450 sheet</t>

</xml_diff>

<commit_message>
0.11.5: Summary Chargeable ####, unlocked Unit/Area m2, Qty display
- Summary legend and side buttons move from O:P to Q:R (SUM_SIDE_COL):
  the table reaches O since 0.11.0 and the legend had narrowed it to 4,
  so Chargeable showed ####.
- Unit and Area m2 locked on added rows: the template's table-column
  formats said unlocked (mac/apply-calc-lock-template.py, applied), and
  PreparePassSheet locks both on every Refresh Locations.
- Qty: whole numbers show #,##0 through a conditional format, not "100.";
  validation allows a blank, so pass rows' Qty is not flagged.
- Tests: test-summaryformat and test-multipass (.ps1 and mac/.py).
- CHANGELOG, Release-Notes, ARCHITECTURE (legend position).

Found from the 2026-10-28 Mac screenshots. Mac only so far; not run yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/PrintCosts.xlsx
+++ b/src/PrintCosts.xlsx
@@ -2207,7 +2207,7 @@
         </patternFill>
       </fill>
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="0" hidden="0"/>
+      <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2325,7 +2325,7 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="0" hidden="0"/>
+      <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>

</xml_diff>